<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-17 04:41 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -4829,7 +4829,7 @@
         <v>46134.79240423611</v>
       </c>
       <c r="D53" s="8">
-        <v>46134.792419756945</v>
+        <v>46190.18859494213</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>193</v>
@@ -4873,8 +4873,8 @@
       <c r="R53" s="8">
         <v>46197</v>
       </c>
-      <c r="S53" s="11" t="s">
-        <v>90</v>
+      <c r="S53" s="12" t="s">
+        <v>79</v>
       </c>
       <c r="T53" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-18 17:40 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -9059,7 +9059,7 @@
       </c>
       <c r="C129" s="9"/>
       <c r="D129" s="8">
-        <v>46125.58906165509</v>
+        <v>46191.706051354166</v>
       </c>
       <c r="E129" s="9" t="s">
         <v>340</v>
@@ -9738,9 +9738,11 @@
       <c r="B142" s="5">
         <v>46122.55174869213</v>
       </c>
-      <c r="C142" s="6"/>
+      <c r="C142" s="5">
+        <v>46191.70598530093</v>
+      </c>
       <c r="D142" s="5">
-        <v>46185.6436540162</v>
+        <v>46191.706001886574</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>362</v>
@@ -9786,10 +9788,10 @@
         <v>90</v>
       </c>
       <c r="T142" s="6">
-        <v>0</v>
-      </c>
-      <c r="U142" s="10" t="s">
-        <v>114</v>
+        <v>1</v>
+      </c>
+      <c r="U142" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -10054,9 +10056,11 @@
       <c r="B148" s="5">
         <v>46122.551753472224</v>
       </c>
-      <c r="C148" s="6"/>
+      <c r="C148" s="5">
+        <v>46191.70604009259</v>
+      </c>
       <c r="D148" s="5">
-        <v>46125.764779895835</v>
+        <v>46191.706057812495</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>371</v>
@@ -10102,10 +10106,10 @@
         <v>90</v>
       </c>
       <c r="T148" s="6">
-        <v>0</v>
-      </c>
-      <c r="U148" s="10" t="s">
-        <v>114</v>
+        <v>1</v>
+      </c>
+      <c r="U148" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.25">
@@ -10419,7 +10423,7 @@
       </c>
       <c r="C155" s="9"/>
       <c r="D155" s="8">
-        <v>46125.594011458335</v>
+        <v>46191.70605767361</v>
       </c>
       <c r="E155" s="9" t="s">
         <v>382</v>
@@ -10469,8 +10473,8 @@
       <c r="T155" s="9">
         <v>0</v>
       </c>
-      <c r="U155" s="10" t="s">
-        <v>114</v>
+      <c r="U155" s="12" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.25">
@@ -10482,7 +10486,7 @@
       </c>
       <c r="C156" s="6"/>
       <c r="D156" s="5">
-        <v>46125.59400841435</v>
+        <v>46191.70605090278</v>
       </c>
       <c r="E156" s="6" t="s">
         <v>386</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-20 22:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -217,9 +217,6 @@
     <t>Ingenieria Basica Motor,Ingenieria basica Rodete,Ingenieria Detalle</t>
   </si>
   <si>
-    <t>Tarea en curso</t>
-  </si>
-  <si>
     <t>1214004989966429</t>
   </si>
   <si>
@@ -312,6 +309,9 @@
   </si>
   <si>
     <t>Propuesta compras:,Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1214005097392408</t>
@@ -2213,9 +2213,11 @@
       <c r="B10" s="5">
         <v>46122.55119412037</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="5">
+        <v>46193.93280347223</v>
+      </c>
       <c r="D10" s="5">
-        <v>46192.97384186342</v>
+        <v>46193.9328209838</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>48</v>
@@ -2250,14 +2252,16 @@
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
       <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="12" t="s">
-        <v>50</v>
+      <c r="T10" s="6">
+        <v>1</v>
+      </c>
+      <c r="U10" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="8">
         <v>46122.5513631713</v>
@@ -2269,7 +2273,7 @@
         <v>46192.97382803241</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>26</v>
@@ -2290,7 +2294,7 @@
         <v>26</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="M11" s="9" t="s">
         <v>26</v>
@@ -2302,7 +2306,7 @@
         <v>41</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="Q11" s="8">
         <v>46127</v>
@@ -2322,7 +2326,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B12" s="5">
         <v>46122.551369050925</v>
@@ -2334,7 +2338,7 @@
         <v>46192.97382813657</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
@@ -2355,7 +2359,7 @@
         <v>26</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M12" s="6" t="s">
         <v>26</v>
@@ -2367,7 +2371,7 @@
         <v>41</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Q12" s="5">
         <v>46127</v>
@@ -2387,7 +2391,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B13" s="8">
         <v>46122.5513746875</v>
@@ -2399,7 +2403,7 @@
         <v>46192.97382800926</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>26</v>
@@ -2432,7 +2436,7 @@
         <v>41</v>
       </c>
       <c r="P13" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q13" s="8">
         <v>46127</v>
@@ -2452,7 +2456,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B14" s="5">
         <v>46122.553594178244</v>
@@ -2464,7 +2468,7 @@
         <v>46136.20601917824</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
@@ -2485,7 +2489,7 @@
         <v>26</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>26</v>
@@ -2497,7 +2501,7 @@
         <v>41</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="Q14" s="5">
         <v>46127</v>
@@ -2517,7 +2521,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B15" s="8">
         <v>46122.55119946759</v>
@@ -2527,7 +2531,7 @@
         <v>46181.66640564815</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>25</v>
@@ -2551,7 +2555,7 @@
         <v>26</v>
       </c>
       <c r="O15" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P15" s="9" t="s">
         <v>26</v>
@@ -2564,7 +2568,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B16" s="5">
         <v>46122.55138855324</v>
@@ -2576,7 +2580,7 @@
         <v>46133.17999505787</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2603,13 +2607,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Q16" s="5">
         <v>46129</v>
@@ -2629,7 +2633,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B17" s="8">
         <v>46122.55139482639</v>
@@ -2641,7 +2645,7 @@
         <v>46132.182206921294</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
@@ -2668,13 +2672,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Q17" s="8">
         <v>46136</v>
@@ -2683,7 +2687,7 @@
         <v>46139</v>
       </c>
       <c r="S17" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
@@ -2694,7 +2698,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18" s="5">
         <v>46122.55140040509</v>
@@ -2704,16 +2708,16 @@
         <v>46139.170930567125</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>78</v>
-      </c>
       <c r="H18" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I18" s="5">
         <v>46136</v>
@@ -2731,13 +2735,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q18" s="5">
         <v>46136</v>
@@ -2746,13 +2750,13 @@
         <v>46139</v>
       </c>
       <c r="S18" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="T18" s="6">
         <v>0</v>
       </c>
       <c r="U18" s="12" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -2796,7 +2800,7 @@
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O19" s="9" t="s">
         <v>84</v>
@@ -2834,7 +2838,7 @@
         <v>46132.1822065625</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2861,10 +2865,10 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>89</v>
@@ -2876,7 +2880,7 @@
         <v>46139</v>
       </c>
       <c r="S20" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="T20" s="6">
         <v>1</v>
@@ -2926,7 +2930,7 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O21" s="9" t="s">
         <v>84</v>
@@ -2991,7 +2995,7 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O22" s="6" t="s">
         <v>84</v>
@@ -3056,7 +3060,7 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O23" s="9" t="s">
         <v>84</v>
@@ -3236,7 +3240,7 @@
         <v>103</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>109</v>
@@ -3419,7 +3423,7 @@
         <v>115</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="P29" s="9" t="s">
         <v>119</v>
@@ -3604,7 +3608,7 @@
         <v>124</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="P32" s="6" t="s">
         <v>128</v>
@@ -4039,7 +4043,7 @@
         <v>147</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P39" s="9" t="s">
         <v>150</v>
@@ -4721,7 +4725,7 @@
         <v>181</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="P51" s="9" t="s">
         <v>187</v>
@@ -4798,7 +4802,7 @@
         <v>46197</v>
       </c>
       <c r="S52" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="T52" s="6">
         <v>1</v>
@@ -4861,7 +4865,7 @@
         <v>46198</v>
       </c>
       <c r="S53" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="T53" s="9">
         <v>1</v>
@@ -6459,7 +6463,7 @@
         <v>0</v>
       </c>
       <c r="U81" s="12" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6522,7 +6526,7 @@
         <v>0</v>
       </c>
       <c r="U82" s="12" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -6585,7 +6589,7 @@
         <v>0</v>
       </c>
       <c r="U83" s="12" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
@@ -6595,9 +6599,11 @@
       <c r="B84" s="5">
         <v>46122.59399163195</v>
       </c>
-      <c r="C84" s="6"/>
+      <c r="C84" s="5">
+        <v>46193.93315311342</v>
+      </c>
       <c r="D84" s="5">
-        <v>46181.66696350694</v>
+        <v>46193.9332800463</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>267</v>
@@ -6645,10 +6651,10 @@
         <v>86</v>
       </c>
       <c r="T84" s="6">
-        <v>0</v>
-      </c>
-      <c r="U84" s="12" t="s">
-        <v>50</v>
+        <v>1</v>
+      </c>
+      <c r="U84" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -6707,7 +6713,7 @@
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46181.668712280094</v>
+        <v>46193.93317614583</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>273</v>
@@ -6716,10 +6722,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I86" s="5">
         <v>46260</v>
@@ -6757,8 +6763,8 @@
       <c r="T86" s="6">
         <v>0</v>
       </c>
-      <c r="U86" s="10" t="s">
-        <v>110</v>
+      <c r="U86" s="12" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -6770,7 +6776,7 @@
       </c>
       <c r="C87" s="9"/>
       <c r="D87" s="8">
-        <v>46181.66865702547</v>
+        <v>46193.933163194444</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>200</v>
@@ -6779,10 +6785,10 @@
         <v>26</v>
       </c>
       <c r="G87" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H87" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I87" s="8">
         <v>46260</v>
@@ -6823,7 +6829,7 @@
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46181.668672858796</v>
+        <v>46193.93316084491</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>200</v>
@@ -6832,10 +6838,10 @@
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I88" s="5">
         <v>46260</v>
@@ -6876,7 +6882,7 @@
       </c>
       <c r="C89" s="9"/>
       <c r="D89" s="8">
-        <v>46181.668682986114</v>
+        <v>46193.93316216435</v>
       </c>
       <c r="E89" s="9" t="s">
         <v>200</v>
@@ -6885,10 +6891,10 @@
         <v>26</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H89" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I89" s="8">
         <v>46260</v>
@@ -6929,7 +6935,7 @@
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46181.66869396991</v>
+        <v>46193.933167083334</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>200</v>
@@ -6938,10 +6944,10 @@
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I90" s="5">
         <v>46260</v>
@@ -6982,7 +6988,7 @@
       </c>
       <c r="C91" s="9"/>
       <c r="D91" s="8">
-        <v>46181.66871287037</v>
+        <v>46193.93316814815</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>200</v>
@@ -6991,10 +6997,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H91" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I91" s="8">
         <v>46260</v>
@@ -7044,10 +7050,10 @@
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I92" s="5">
         <v>46280</v>
@@ -7107,10 +7113,10 @@
         <v>26</v>
       </c>
       <c r="G93" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H93" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I93" s="8">
         <v>46280</v>
@@ -7160,10 +7166,10 @@
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I94" s="5">
         <v>46280</v>
@@ -7213,10 +7219,10 @@
         <v>26</v>
       </c>
       <c r="G95" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H95" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I95" s="8">
         <v>46280</v>
@@ -7266,10 +7272,10 @@
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I96" s="5">
         <v>46280</v>
@@ -7319,10 +7325,10 @@
         <v>26</v>
       </c>
       <c r="G97" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H97" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I97" s="8">
         <v>46280</v>
@@ -7372,10 +7378,10 @@
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I98" s="5">
         <v>46286</v>
@@ -7435,10 +7441,10 @@
         <v>26</v>
       </c>
       <c r="G99" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H99" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I99" s="8">
         <v>46286</v>
@@ -7488,10 +7494,10 @@
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I100" s="5">
         <v>46286</v>
@@ -7541,10 +7547,10 @@
         <v>26</v>
       </c>
       <c r="G101" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H101" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I101" s="8">
         <v>46286</v>
@@ -7594,10 +7600,10 @@
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I102" s="5">
         <v>46286</v>
@@ -7647,10 +7653,10 @@
         <v>26</v>
       </c>
       <c r="G103" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H103" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I103" s="8">
         <v>46286</v>
@@ -7700,10 +7706,10 @@
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I104" s="5">
         <v>46289</v>
@@ -7763,10 +7769,10 @@
         <v>26</v>
       </c>
       <c r="G105" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H105" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I105" s="8">
         <v>46289</v>
@@ -7816,10 +7822,10 @@
         <v>26</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I106" s="5">
         <v>46289</v>
@@ -7869,10 +7875,10 @@
         <v>26</v>
       </c>
       <c r="G107" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H107" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I107" s="8">
         <v>46289</v>
@@ -7922,10 +7928,10 @@
         <v>26</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I108" s="5">
         <v>46289</v>
@@ -7975,10 +7981,10 @@
         <v>26</v>
       </c>
       <c r="G109" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H109" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I109" s="8">
         <v>46289</v>
@@ -8028,10 +8034,10 @@
         <v>26</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H110" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I110" s="5">
         <v>46311</v>
@@ -8091,10 +8097,10 @@
         <v>26</v>
       </c>
       <c r="G111" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H111" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I111" s="8">
         <v>46311</v>
@@ -8144,10 +8150,10 @@
         <v>26</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H112" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I112" s="5">
         <v>46311</v>
@@ -8197,10 +8203,10 @@
         <v>26</v>
       </c>
       <c r="G113" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H113" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I113" s="8">
         <v>46311</v>
@@ -8250,10 +8256,10 @@
         <v>26</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H114" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I114" s="5">
         <v>46311</v>
@@ -8303,10 +8309,10 @@
         <v>26</v>
       </c>
       <c r="G115" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H115" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I115" s="8">
         <v>46311</v>
@@ -8356,10 +8362,10 @@
         <v>26</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I116" s="5">
         <v>46315</v>
@@ -8419,10 +8425,10 @@
         <v>26</v>
       </c>
       <c r="G117" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H117" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I117" s="9"/>
       <c r="J117" s="8">
@@ -8470,10 +8476,10 @@
         <v>26</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H118" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I118" s="6"/>
       <c r="J118" s="5">
@@ -8521,10 +8527,10 @@
         <v>26</v>
       </c>
       <c r="G119" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H119" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I119" s="9"/>
       <c r="J119" s="8">
@@ -8572,10 +8578,10 @@
         <v>26</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H120" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I120" s="6"/>
       <c r="J120" s="5">
@@ -8623,10 +8629,10 @@
         <v>26</v>
       </c>
       <c r="G121" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H121" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I121" s="9"/>
       <c r="J121" s="8">
@@ -8674,10 +8680,10 @@
         <v>26</v>
       </c>
       <c r="G122" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H122" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I122" s="5">
         <v>46317</v>
@@ -8737,10 +8743,10 @@
         <v>26</v>
       </c>
       <c r="G123" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H123" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I123" s="9"/>
       <c r="J123" s="8">
@@ -8788,10 +8794,10 @@
         <v>26</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H124" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I124" s="6"/>
       <c r="J124" s="5">
@@ -8839,10 +8845,10 @@
         <v>26</v>
       </c>
       <c r="G125" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H125" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I125" s="9"/>
       <c r="J125" s="8">
@@ -8890,10 +8896,10 @@
         <v>26</v>
       </c>
       <c r="G126" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H126" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I126" s="6"/>
       <c r="J126" s="5">
@@ -8941,10 +8947,10 @@
         <v>26</v>
       </c>
       <c r="G127" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H127" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I127" s="9"/>
       <c r="J127" s="8">
@@ -9357,10 +9363,10 @@
         <v>26</v>
       </c>
       <c r="G135" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H135" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I135" s="9"/>
       <c r="J135" s="8">
@@ -9418,10 +9424,10 @@
         <v>26</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H136" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I136" s="6"/>
       <c r="J136" s="5">
@@ -9469,10 +9475,10 @@
         <v>26</v>
       </c>
       <c r="G137" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H137" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I137" s="9"/>
       <c r="J137" s="8">
@@ -9520,10 +9526,10 @@
         <v>26</v>
       </c>
       <c r="G138" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H138" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I138" s="6"/>
       <c r="J138" s="5">
@@ -9571,10 +9577,10 @@
         <v>26</v>
       </c>
       <c r="G139" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H139" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I139" s="9"/>
       <c r="J139" s="8">
@@ -9622,10 +9628,10 @@
         <v>26</v>
       </c>
       <c r="G140" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H140" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I140" s="6"/>
       <c r="J140" s="5">
@@ -10398,7 +10404,7 @@
         <v>0</v>
       </c>
       <c r="U154" s="12" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
     </row>
     <row r="155" spans="1:21" x14ac:dyDescent="0.25">
@@ -10461,7 +10467,7 @@
         <v>0</v>
       </c>
       <c r="U155" s="12" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 14:25 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1814" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1817" uniqueCount="383">
   <si>
     <t xml:space="preserve"> 50001466 - ZITRON PERU (PODEROSA) </t>
   </si>
@@ -842,6 +842,9 @@
     <t>Recepcion Rodete,Recepcion Alabe,Recepcion motor,Recepcion Sensor</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
     <t>1214005013744127</t>
   </si>
   <si>
@@ -1212,9 +1215,6 @@
   </si>
   <si>
     <t>nicolas.tello@zitron.com</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1214005018360998</t>
@@ -6324,9 +6324,11 @@
       <c r="B79" s="8">
         <v>46122.55160357639</v>
       </c>
-      <c r="C79" s="9"/>
+      <c r="C79" s="8">
+        <v>46195.563125636574</v>
+      </c>
       <c r="D79" s="8">
-        <v>46195.50752947917</v>
+        <v>46195.563290335645</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>206</v>
@@ -6361,22 +6363,28 @@
       <c r="Q79" s="9"/>
       <c r="R79" s="9"/>
       <c r="S79" s="9"/>
-      <c r="T79" s="9"/>
-      <c r="U79" s="9"/>
+      <c r="T79" s="9">
+        <v>1</v>
+      </c>
+      <c r="U79" s="12" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B80" s="5">
         <v>46122.55160679398</v>
       </c>
-      <c r="C80" s="6"/>
+      <c r="C80" s="5">
+        <v>46195.563269363425</v>
+      </c>
       <c r="D80" s="5">
-        <v>46193.175859236115</v>
+        <v>46195.563288715275</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
@@ -6409,7 +6417,7 @@
         <v>120</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q80" s="5">
         <v>46191</v>
@@ -6421,15 +6429,15 @@
         <v>32</v>
       </c>
       <c r="T80" s="6">
-        <v>0</v>
-      </c>
-      <c r="U80" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U80" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B81" s="8">
         <v>46122.551612256946</v>
@@ -6441,7 +6449,7 @@
         <v>46195.50753130787</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6474,7 +6482,7 @@
         <v>111</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q81" s="8">
         <v>46266</v>
@@ -6494,7 +6502,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B82" s="5">
         <v>46122.55161756944</v>
@@ -6506,7 +6514,7 @@
         <v>46195.50753259259</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6539,7 +6547,7 @@
         <v>129</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q82" s="5">
         <v>46309</v>
@@ -6559,7 +6567,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B83" s="8">
         <v>46122.55162288195</v>
@@ -6571,7 +6579,7 @@
         <v>46195.507539479164</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>26</v>
@@ -6604,7 +6612,7 @@
         <v>151</v>
       </c>
       <c r="P83" s="9" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q83" s="8">
         <v>46189</v>
@@ -6624,7 +6632,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B84" s="5">
         <v>46122.59399163195</v>
@@ -6636,7 +6644,7 @@
         <v>46193.9332800463</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
@@ -6669,7 +6677,7 @@
         <v>169</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q84" s="5">
         <v>46239</v>
@@ -6689,17 +6697,19 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B85" s="8">
         <v>46122.551628182875</v>
       </c>
-      <c r="C85" s="9"/>
+      <c r="C85" s="8">
+        <v>46195.5630599537</v>
+      </c>
       <c r="D85" s="8">
-        <v>46195.507700347225</v>
+        <v>46195.56307581019</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>25</v>
@@ -6723,7 +6733,7 @@
         <v>26</v>
       </c>
       <c r="O85" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="P85" s="9" t="s">
         <v>26</v>
@@ -6731,12 +6741,16 @@
       <c r="Q85" s="9"/>
       <c r="R85" s="9"/>
       <c r="S85" s="9"/>
-      <c r="T85" s="9"/>
-      <c r="U85" s="9"/>
+      <c r="T85" s="9">
+        <v>1</v>
+      </c>
+      <c r="U85" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B86" s="5">
         <v>46122.55163158565</v>
@@ -6748,7 +6762,7 @@
         <v>46195.507707129625</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
@@ -6775,13 +6789,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q86" s="5">
         <v>46260</v>
@@ -6801,7 +6815,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B87" s="8">
         <v>46125.5974969213</v>
@@ -6838,10 +6852,10 @@
         <v>26</v>
       </c>
       <c r="N87" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="O87" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P87" s="9" t="s">
         <v>199</v>
@@ -6854,7 +6868,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B88" s="5">
         <v>46125.59754570602</v>
@@ -6891,10 +6905,10 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P88" s="6" t="s">
         <v>199</v>
@@ -6907,7 +6921,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B89" s="8">
         <v>46125.59760710648</v>
@@ -6944,10 +6958,10 @@
         <v>26</v>
       </c>
       <c r="N89" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="O89" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P89" s="9" t="s">
         <v>199</v>
@@ -6960,7 +6974,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B90" s="5">
         <v>46125.59765891204</v>
@@ -6997,10 +7011,10 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P90" s="6" t="s">
         <v>199</v>
@@ -7013,7 +7027,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B91" s="8">
         <v>46125.597703391206</v>
@@ -7050,10 +7064,10 @@
         <v>26</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="O91" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P91" s="9" t="s">
         <v>199</v>
@@ -7066,7 +7080,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B92" s="5">
         <v>46122.55170659722</v>
@@ -7076,7 +7090,7 @@
         <v>46125.65705061343</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
@@ -7103,13 +7117,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O92" s="6" t="s">
         <v>197</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q92" s="5">
         <v>46280</v>
@@ -7129,7 +7143,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B93" s="8">
         <v>46125.59982741898</v>
@@ -7166,13 +7180,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O93" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P93" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q93" s="9"/>
       <c r="R93" s="9"/>
@@ -7182,7 +7196,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B94" s="5">
         <v>46125.599890833335</v>
@@ -7219,13 +7233,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="Q94" s="6"/>
       <c r="R94" s="6"/>
@@ -7235,7 +7249,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B95" s="8">
         <v>46125.59993134259</v>
@@ -7272,13 +7286,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O95" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P95" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q95" s="9"/>
       <c r="R95" s="9"/>
@@ -7288,7 +7302,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B96" s="5">
         <v>46125.59996929398</v>
@@ -7325,13 +7339,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q96" s="6"/>
       <c r="R96" s="6"/>
@@ -7341,7 +7355,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B97" s="8">
         <v>46125.6000115162</v>
@@ -7378,13 +7392,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O97" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P97" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q97" s="9"/>
       <c r="R97" s="9"/>
@@ -7394,7 +7408,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B98" s="5">
         <v>46122.55164413195</v>
@@ -7404,7 +7418,7 @@
         <v>46125.65705466435</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7431,13 +7445,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q98" s="5">
         <v>46286</v>
@@ -7457,7 +7471,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B99" s="8">
         <v>46125.599162743056</v>
@@ -7494,13 +7508,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O99" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="P99" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Q99" s="9"/>
       <c r="R99" s="9"/>
@@ -7510,7 +7524,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B100" s="5">
         <v>46125.599302511575</v>
@@ -7547,13 +7561,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O100" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="P100" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Q100" s="6"/>
       <c r="R100" s="6"/>
@@ -7563,7 +7577,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B101" s="8">
         <v>46125.59934644676</v>
@@ -7600,13 +7614,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O101" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="P101" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Q101" s="9"/>
       <c r="R101" s="9"/>
@@ -7616,7 +7630,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B102" s="5">
         <v>46125.59938857639</v>
@@ -7653,13 +7667,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Q102" s="6"/>
       <c r="R102" s="6"/>
@@ -7669,7 +7683,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B103" s="8">
         <v>46125.59943094908</v>
@@ -7706,13 +7720,13 @@
         <v>26</v>
       </c>
       <c r="N103" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O103" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="P103" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Q103" s="9"/>
       <c r="R103" s="9"/>
@@ -7722,7 +7736,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B104" s="5">
         <v>46122.551650995374</v>
@@ -7732,7 +7746,7 @@
         <v>46125.65705875</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
@@ -7759,13 +7773,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O104" s="6" t="s">
         <v>197</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q104" s="5">
         <v>46289</v>
@@ -7785,14 +7799,14 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B105" s="8">
         <v>46125.59953013889</v>
       </c>
       <c r="C105" s="9"/>
       <c r="D105" s="8">
-        <v>46134.79248056713</v>
+        <v>46195.56328270833</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>199</v>
@@ -7822,13 +7836,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O105" s="9" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P105" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q105" s="9"/>
       <c r="R105" s="9"/>
@@ -7838,14 +7852,14 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B106" s="5">
         <v>46125.59961423611</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46134.792473194444</v>
+        <v>46195.56328116899</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>199</v>
@@ -7875,13 +7889,13 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -7891,14 +7905,14 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B107" s="8">
         <v>46125.599654317135</v>
       </c>
       <c r="C107" s="9"/>
       <c r="D107" s="8">
-        <v>46134.792470844906</v>
+        <v>46195.56328055555</v>
       </c>
       <c r="E107" s="9" t="s">
         <v>199</v>
@@ -7928,13 +7942,13 @@
         <v>26</v>
       </c>
       <c r="N107" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O107" s="9" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P107" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q107" s="9"/>
       <c r="R107" s="9"/>
@@ -7944,14 +7958,14 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B108" s="5">
         <v>46125.59957065972</v>
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46134.79247670139</v>
+        <v>46195.56328217592</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>199</v>
@@ -7981,13 +7995,13 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P108" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q108" s="6"/>
       <c r="R108" s="6"/>
@@ -7997,14 +8011,14 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B109" s="8">
         <v>46125.59969711806</v>
       </c>
       <c r="C109" s="9"/>
       <c r="D109" s="8">
-        <v>46134.792476076385</v>
+        <v>46195.563281724535</v>
       </c>
       <c r="E109" s="9" t="s">
         <v>199</v>
@@ -8034,13 +8048,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O109" s="9" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P109" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q109" s="9"/>
       <c r="R109" s="9"/>
@@ -8050,7 +8064,7 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B110" s="5">
         <v>46122.55163725694</v>
@@ -8060,7 +8074,7 @@
         <v>46125.65706174768</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>26</v>
@@ -8087,13 +8101,13 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O110" s="6" t="s">
         <v>197</v>
       </c>
       <c r="P110" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q110" s="5">
         <v>46311</v>
@@ -8113,7 +8127,7 @@
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B111" s="8">
         <v>46125.59780210648</v>
@@ -8150,13 +8164,13 @@
         <v>26</v>
       </c>
       <c r="N111" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O111" s="9" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P111" s="9" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q111" s="9"/>
       <c r="R111" s="9"/>
@@ -8166,7 +8180,7 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B112" s="5">
         <v>46125.597836932866</v>
@@ -8203,13 +8217,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q112" s="6"/>
       <c r="R112" s="6"/>
@@ -8219,7 +8233,7 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B113" s="8">
         <v>46125.5979208912</v>
@@ -8256,13 +8270,13 @@
         <v>26</v>
       </c>
       <c r="N113" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O113" s="9" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P113" s="9" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q113" s="9"/>
       <c r="R113" s="9"/>
@@ -8272,7 +8286,7 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B114" s="5">
         <v>46125.59788087963</v>
@@ -8309,13 +8323,13 @@
         <v>26</v>
       </c>
       <c r="N114" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P114" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q114" s="6"/>
       <c r="R114" s="6"/>
@@ -8325,7 +8339,7 @@
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B115" s="8">
         <v>46125.597965023146</v>
@@ -8362,13 +8376,13 @@
         <v>26</v>
       </c>
       <c r="N115" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O115" s="9" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P115" s="9" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q115" s="9"/>
       <c r="R115" s="9"/>
@@ -8378,7 +8392,7 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B116" s="5">
         <v>46122.55172043982</v>
@@ -8388,7 +8402,7 @@
         <v>46125.658894120366</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
@@ -8415,13 +8429,13 @@
         <v>26</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O116" s="6" t="s">
         <v>197</v>
       </c>
       <c r="P116" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q116" s="5">
         <v>46315</v>
@@ -8441,7 +8455,7 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B117" s="8">
         <v>46125.60038253472</v>
@@ -8476,13 +8490,13 @@
         <v>26</v>
       </c>
       <c r="N117" s="9" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O117" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P117" s="9" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Q117" s="9"/>
       <c r="R117" s="9"/>
@@ -8492,7 +8506,7 @@
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B118" s="5">
         <v>46125.60043012731</v>
@@ -8527,13 +8541,13 @@
         <v>26</v>
       </c>
       <c r="N118" s="6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O118" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P118" s="6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Q118" s="6"/>
       <c r="R118" s="6"/>
@@ -8543,7 +8557,7 @@
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B119" s="8">
         <v>46125.60047290509</v>
@@ -8578,13 +8592,13 @@
         <v>26</v>
       </c>
       <c r="N119" s="9" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O119" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P119" s="9" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Q119" s="9"/>
       <c r="R119" s="9"/>
@@ -8594,7 +8608,7 @@
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B120" s="5">
         <v>46125.600514074074</v>
@@ -8629,13 +8643,13 @@
         <v>26</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O120" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Q120" s="6"/>
       <c r="R120" s="6"/>
@@ -8645,7 +8659,7 @@
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B121" s="8">
         <v>46125.60055859954</v>
@@ -8680,13 +8694,13 @@
         <v>26</v>
       </c>
       <c r="N121" s="9" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O121" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P121" s="9" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Q121" s="9"/>
       <c r="R121" s="9"/>
@@ -8696,7 +8710,7 @@
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B122" s="5">
         <v>46122.55172986111</v>
@@ -8706,7 +8720,7 @@
         <v>46125.66066717592</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>26</v>
@@ -8733,13 +8747,13 @@
         <v>26</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O122" s="6" t="s">
         <v>197</v>
       </c>
       <c r="P122" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="Q122" s="5">
         <v>46317</v>
@@ -8759,7 +8773,7 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B123" s="8">
         <v>46125.60064416667</v>
@@ -8794,13 +8808,13 @@
         <v>26</v>
       </c>
       <c r="N123" s="9" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O123" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P123" s="9" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Q123" s="9"/>
       <c r="R123" s="9"/>
@@ -8810,7 +8824,7 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B124" s="5">
         <v>46125.60068740741</v>
@@ -8845,13 +8859,13 @@
         <v>26</v>
       </c>
       <c r="N124" s="6" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O124" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P124" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Q124" s="6"/>
       <c r="R124" s="6"/>
@@ -8861,7 +8875,7 @@
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B125" s="8">
         <v>46125.60073844907</v>
@@ -8896,13 +8910,13 @@
         <v>26</v>
       </c>
       <c r="N125" s="9" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O125" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P125" s="9" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Q125" s="9"/>
       <c r="R125" s="9"/>
@@ -8912,7 +8926,7 @@
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B126" s="5">
         <v>46125.60077622686</v>
@@ -8947,13 +8961,13 @@
         <v>26</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O126" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P126" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Q126" s="6"/>
       <c r="R126" s="6"/>
@@ -8963,7 +8977,7 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B127" s="8">
         <v>46125.600829143514</v>
@@ -8998,13 +9012,13 @@
         <v>26</v>
       </c>
       <c r="N127" s="9" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O127" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P127" s="9" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Q127" s="9"/>
       <c r="R127" s="9"/>
@@ -9014,17 +9028,19 @@
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B128" s="5">
         <v>46122.5517350463</v>
       </c>
-      <c r="C128" s="6"/>
+      <c r="C128" s="5">
+        <v>46195.56317517361</v>
+      </c>
       <c r="D128" s="5">
-        <v>46191.706051354166</v>
+        <v>46195.56318964121</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>25</v>
@@ -9048,7 +9064,7 @@
         <v>26</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="P128" s="6" t="s">
         <v>26</v>
@@ -9056,12 +9072,16 @@
       <c r="Q128" s="6"/>
       <c r="R128" s="6"/>
       <c r="S128" s="6"/>
-      <c r="T128" s="6"/>
-      <c r="U128" s="6"/>
+      <c r="T128" s="6">
+        <v>1</v>
+      </c>
+      <c r="U128" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B129" s="8">
         <v>46122.5517390625</v>
@@ -9071,16 +9091,16 @@
         <v>46189.53573824074</v>
       </c>
       <c r="E129" s="9" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G129" s="9" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H129" s="9" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I129" s="8">
         <v>46318</v>
@@ -9098,13 +9118,13 @@
         <v>26</v>
       </c>
       <c r="N129" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="O129" s="9" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="P129" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="Q129" s="8">
         <v>46318</v>
@@ -9124,7 +9144,7 @@
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B130" s="5">
         <v>46125.60093731481</v>
@@ -9140,10 +9160,10 @@
         <v>26</v>
       </c>
       <c r="G130" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H130" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I130" s="6"/>
       <c r="J130" s="5">
@@ -9159,13 +9179,13 @@
         <v>26</v>
       </c>
       <c r="N130" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O130" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P130" s="6" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q130" s="6"/>
       <c r="R130" s="6"/>
@@ -9175,7 +9195,7 @@
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B131" s="8">
         <v>46125.601380821754</v>
@@ -9191,10 +9211,10 @@
         <v>26</v>
       </c>
       <c r="G131" s="9" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H131" s="9" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I131" s="9"/>
       <c r="J131" s="8">
@@ -9210,13 +9230,13 @@
         <v>26</v>
       </c>
       <c r="N131" s="9" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O131" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P131" s="9" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q131" s="9"/>
       <c r="R131" s="9"/>
@@ -9226,7 +9246,7 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B132" s="5">
         <v>46125.60142481481</v>
@@ -9242,10 +9262,10 @@
         <v>26</v>
       </c>
       <c r="G132" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H132" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I132" s="6"/>
       <c r="J132" s="5">
@@ -9261,13 +9281,13 @@
         <v>26</v>
       </c>
       <c r="N132" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O132" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P132" s="6" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q132" s="6"/>
       <c r="R132" s="6"/>
@@ -9277,7 +9297,7 @@
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B133" s="8">
         <v>46125.60146085648</v>
@@ -9293,10 +9313,10 @@
         <v>26</v>
       </c>
       <c r="G133" s="9" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H133" s="9" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I133" s="9"/>
       <c r="J133" s="8">
@@ -9312,13 +9332,13 @@
         <v>26</v>
       </c>
       <c r="N133" s="9" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O133" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P133" s="9" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q133" s="9"/>
       <c r="R133" s="9"/>
@@ -9328,7 +9348,7 @@
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B134" s="5">
         <v>46125.60150208333</v>
@@ -9344,10 +9364,10 @@
         <v>26</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I134" s="6"/>
       <c r="J134" s="5">
@@ -9363,13 +9383,13 @@
         <v>26</v>
       </c>
       <c r="N134" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O134" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P134" s="6" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q134" s="6"/>
       <c r="R134" s="6"/>
@@ -9379,7 +9399,7 @@
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B135" s="8">
         <v>46122.55174383102</v>
@@ -9389,7 +9409,7 @@
         <v>46185.646541435184</v>
       </c>
       <c r="E135" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>26</v>
@@ -9414,13 +9434,13 @@
         <v>26</v>
       </c>
       <c r="N135" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="O135" s="9" t="s">
         <v>197</v>
       </c>
       <c r="P135" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="Q135" s="8">
         <v>46321</v>
@@ -9440,7 +9460,7 @@
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B136" s="5">
         <v>46125.601086979164</v>
@@ -9475,13 +9495,13 @@
         <v>26</v>
       </c>
       <c r="N136" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O136" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P136" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Q136" s="6"/>
       <c r="R136" s="6"/>
@@ -9491,7 +9511,7 @@
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B137" s="8">
         <v>46125.60115318287</v>
@@ -9526,13 +9546,13 @@
         <v>26</v>
       </c>
       <c r="N137" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O137" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P137" s="9" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Q137" s="9"/>
       <c r="R137" s="9"/>
@@ -9542,7 +9562,7 @@
     </row>
     <row r="138" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B138" s="5">
         <v>46125.60120391204</v>
@@ -9577,13 +9597,13 @@
         <v>26</v>
       </c>
       <c r="N138" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O138" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P138" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Q138" s="6"/>
       <c r="R138" s="6"/>
@@ -9593,7 +9613,7 @@
     </row>
     <row r="139" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B139" s="8">
         <v>46125.60125796296</v>
@@ -9628,13 +9648,13 @@
         <v>26</v>
       </c>
       <c r="N139" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O139" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P139" s="9" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Q139" s="9"/>
       <c r="R139" s="9"/>
@@ -9644,7 +9664,7 @@
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B140" s="5">
         <v>46125.601304282405</v>
@@ -9679,13 +9699,13 @@
         <v>26</v>
       </c>
       <c r="N140" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O140" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P140" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Q140" s="6"/>
       <c r="R140" s="6"/>
@@ -9695,7 +9715,7 @@
     </row>
     <row r="141" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A141" s="7" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B141" s="8">
         <v>46122.55174869213</v>
@@ -9707,7 +9727,7 @@
         <v>46191.706001886574</v>
       </c>
       <c r="E141" s="9" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>26</v>
@@ -9732,13 +9752,13 @@
         <v>26</v>
       </c>
       <c r="N141" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="O141" s="9" t="s">
         <v>197</v>
       </c>
       <c r="P141" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="Q141" s="8">
         <v>46322</v>
@@ -9758,7 +9778,7 @@
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B142" s="5">
         <v>46125.60158650463</v>
@@ -9793,13 +9813,13 @@
         <v>26</v>
       </c>
       <c r="N142" s="6" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="O142" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P142" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q142" s="6"/>
       <c r="R142" s="6"/>
@@ -9809,7 +9829,7 @@
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B143" s="8">
         <v>46125.60163133102</v>
@@ -9844,13 +9864,13 @@
         <v>26</v>
       </c>
       <c r="N143" s="9" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="O143" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P143" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q143" s="9"/>
       <c r="R143" s="9"/>
@@ -9860,7 +9880,7 @@
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B144" s="5">
         <v>46125.60167016204</v>
@@ -9895,13 +9915,13 @@
         <v>26</v>
       </c>
       <c r="N144" s="6" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="O144" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P144" s="6" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="Q144" s="6"/>
       <c r="R144" s="6"/>
@@ -9911,7 +9931,7 @@
     </row>
     <row r="145" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A145" s="7" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B145" s="8">
         <v>46125.60170435185</v>
@@ -9946,13 +9966,13 @@
         <v>26</v>
       </c>
       <c r="N145" s="9" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="O145" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P145" s="9" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="Q145" s="9"/>
       <c r="R145" s="9"/>
@@ -9962,7 +9982,7 @@
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B146" s="5">
         <v>46125.60173947917</v>
@@ -9997,13 +10017,13 @@
         <v>26</v>
       </c>
       <c r="N146" s="6" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="O146" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P146" s="6" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="Q146" s="6"/>
       <c r="R146" s="6"/>
@@ -10013,7 +10033,7 @@
     </row>
     <row r="147" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B147" s="8">
         <v>46122.551753472224</v>
@@ -10025,7 +10045,7 @@
         <v>46191.706057812495</v>
       </c>
       <c r="E147" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>26</v>
@@ -10050,13 +10070,13 @@
         <v>26</v>
       </c>
       <c r="N147" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="O147" s="9" t="s">
         <v>197</v>
       </c>
       <c r="P147" s="9" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="Q147" s="8">
         <v>46323</v>
@@ -10076,7 +10096,7 @@
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B148" s="5">
         <v>46125.60181555555</v>
@@ -10111,13 +10131,13 @@
         <v>26</v>
       </c>
       <c r="N148" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O148" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P148" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q148" s="6"/>
       <c r="R148" s="6"/>
@@ -10127,7 +10147,7 @@
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B149" s="8">
         <v>46125.60185690972</v>
@@ -10162,13 +10182,13 @@
         <v>26</v>
       </c>
       <c r="N149" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O149" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P149" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q149" s="9"/>
       <c r="R149" s="9"/>
@@ -10178,7 +10198,7 @@
     </row>
     <row r="150" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B150" s="5">
         <v>46125.601899490735</v>
@@ -10213,13 +10233,13 @@
         <v>26</v>
       </c>
       <c r="N150" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O150" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P150" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q150" s="6"/>
       <c r="R150" s="6"/>
@@ -10229,7 +10249,7 @@
     </row>
     <row r="151" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B151" s="8">
         <v>46125.60193935185</v>
@@ -10264,13 +10284,13 @@
         <v>26</v>
       </c>
       <c r="N151" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O151" s="9" t="s">
         <v>199</v>
       </c>
       <c r="P151" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q151" s="9"/>
       <c r="R151" s="9"/>
@@ -10280,7 +10300,7 @@
     </row>
     <row r="152" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A152" s="4" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B152" s="5">
         <v>46125.60197710648</v>
@@ -10315,13 +10335,13 @@
         <v>26</v>
       </c>
       <c r="N152" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O152" s="6" t="s">
         <v>199</v>
       </c>
       <c r="P152" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q152" s="6"/>
       <c r="R152" s="6"/>
@@ -10331,7 +10351,7 @@
     </row>
     <row r="153" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A153" s="7" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B153" s="8">
         <v>46122.551758622685</v>
@@ -10341,7 +10361,7 @@
         <v>46125.58936878473</v>
       </c>
       <c r="E153" s="9" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>25</v>
@@ -10365,7 +10385,7 @@
         <v>26</v>
       </c>
       <c r="O153" s="9" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="P153" s="9" t="s">
         <v>26</v>
@@ -10378,7 +10398,7 @@
     </row>
     <row r="154" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B154" s="5">
         <v>46122.55176134259</v>
@@ -10388,16 +10408,16 @@
         <v>46191.70605767361</v>
       </c>
       <c r="E154" s="6" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F154" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G154" s="6" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H154" s="6" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="I154" s="5">
         <v>46324</v>
@@ -10415,13 +10435,13 @@
         <v>26</v>
       </c>
       <c r="N154" s="6" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="O154" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P154" s="6" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="Q154" s="5">
         <v>46324</v>
@@ -10436,7 +10456,7 @@
         <v>0</v>
       </c>
       <c r="U154" s="12" t="s">
-        <v>380</v>
+        <v>256</v>
       </c>
     </row>
     <row r="155" spans="1:21" x14ac:dyDescent="0.25">
@@ -10457,10 +10477,10 @@
         <v>26</v>
       </c>
       <c r="G155" s="9" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H155" s="9" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="I155" s="8">
         <v>46324</v>
@@ -10478,13 +10498,13 @@
         <v>26</v>
       </c>
       <c r="N155" s="9" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="O155" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P155" s="9" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="Q155" s="8">
         <v>46324</v>
@@ -10499,7 +10519,7 @@
         <v>0</v>
       </c>
       <c r="U155" s="12" t="s">
-        <v>380</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-23 18:51 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -4911,7 +4911,7 @@
         <v>46195.50761325231</v>
       </c>
       <c r="D54" s="5">
-        <v>46195.50762895834</v>
+        <v>46196.76907818287</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>195</v>
@@ -4959,8 +4959,8 @@
       <c r="T54" s="6">
         <v>1</v>
       </c>
-      <c r="U54" s="11" t="s">
-        <v>33</v>
+      <c r="U54" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
@@ -4970,9 +4970,11 @@
       <c r="B55" s="8">
         <v>46125.603622118055</v>
       </c>
-      <c r="C55" s="9"/>
+      <c r="C55" s="8">
+        <v>46196.76904752315</v>
+      </c>
       <c r="D55" s="8">
-        <v>46125.65979525463</v>
+        <v>46196.7690521412</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>200</v>
@@ -5021,9 +5023,11 @@
       <c r="B56" s="5">
         <v>46125.60367094907</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46196.769048449074</v>
+      </c>
       <c r="D56" s="5">
-        <v>46125.65985976852</v>
+        <v>46196.769052523145</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>200</v>
@@ -5072,9 +5076,11 @@
       <c r="B57" s="8">
         <v>46125.60371951389</v>
       </c>
-      <c r="C57" s="9"/>
+      <c r="C57" s="8">
+        <v>46196.76904929398</v>
+      </c>
       <c r="D57" s="8">
-        <v>46125.65983615741</v>
+        <v>46196.76905283565</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>200</v>
@@ -5123,9 +5129,11 @@
       <c r="B58" s="5">
         <v>46125.60376462963</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46196.769050069444</v>
+      </c>
       <c r="D58" s="5">
-        <v>46125.659875694444</v>
+        <v>46196.76905314815</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>200</v>
@@ -5174,9 +5182,11 @@
       <c r="B59" s="8">
         <v>46125.60381739584</v>
       </c>
-      <c r="C59" s="9"/>
+      <c r="C59" s="8">
+        <v>46196.76905077546</v>
+      </c>
       <c r="D59" s="8">
-        <v>46125.659896990735</v>
+        <v>46196.76905349537</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>200</v>
@@ -6710,7 +6720,7 @@
         <v>46195.5630599537</v>
       </c>
       <c r="D85" s="8">
-        <v>46195.56307581019</v>
+        <v>46196.769192685184</v>
       </c>
       <c r="E85" s="9" t="s">
         <v>270</v>
@@ -6748,8 +6758,8 @@
       <c r="T85" s="9">
         <v>1</v>
       </c>
-      <c r="U85" s="11" t="s">
-        <v>33</v>
+      <c r="U85" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
@@ -6824,9 +6834,11 @@
       <c r="B87" s="8">
         <v>46125.5974969213</v>
       </c>
-      <c r="C87" s="9"/>
+      <c r="C87" s="8">
+        <v>46196.76791707176</v>
+      </c>
       <c r="D87" s="8">
-        <v>46193.933163194444</v>
+        <v>46196.767918831014</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>200</v>
@@ -6877,9 +6889,11 @@
       <c r="B88" s="5">
         <v>46125.59754570602</v>
       </c>
-      <c r="C88" s="6"/>
+      <c r="C88" s="5">
+        <v>46196.76795405093</v>
+      </c>
       <c r="D88" s="5">
-        <v>46193.93316084491</v>
+        <v>46196.76795645834</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>200</v>
@@ -6930,9 +6944,11 @@
       <c r="B89" s="8">
         <v>46125.59760710648</v>
       </c>
-      <c r="C89" s="9"/>
+      <c r="C89" s="8">
+        <v>46196.767928217596</v>
+      </c>
       <c r="D89" s="8">
-        <v>46193.93316216435</v>
+        <v>46196.76793001157</v>
       </c>
       <c r="E89" s="9" t="s">
         <v>200</v>
@@ -6983,9 +6999,11 @@
       <c r="B90" s="5">
         <v>46125.59765891204</v>
       </c>
-      <c r="C90" s="6"/>
+      <c r="C90" s="5">
+        <v>46196.76794651621</v>
+      </c>
       <c r="D90" s="5">
-        <v>46193.933167083334</v>
+        <v>46196.76794809027</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>200</v>
@@ -7036,9 +7054,11 @@
       <c r="B91" s="8">
         <v>46125.597703391206</v>
       </c>
-      <c r="C91" s="9"/>
+      <c r="C91" s="8">
+        <v>46196.76794100694</v>
+      </c>
       <c r="D91" s="8">
-        <v>46193.93316814815</v>
+        <v>46196.76794287037</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>200</v>
@@ -7089,9 +7109,11 @@
       <c r="B92" s="5">
         <v>46122.55170659722</v>
       </c>
-      <c r="C92" s="6"/>
+      <c r="C92" s="5">
+        <v>46196.76755512731</v>
+      </c>
       <c r="D92" s="5">
-        <v>46125.65705061343</v>
+        <v>46196.76807780092</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>282</v>
@@ -7139,10 +7161,10 @@
         <v>105</v>
       </c>
       <c r="T92" s="6">
-        <v>0</v>
-      </c>
-      <c r="U92" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U92" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -7152,9 +7174,11 @@
       <c r="B93" s="8">
         <v>46125.59982741898</v>
       </c>
-      <c r="C93" s="9"/>
+      <c r="C93" s="8">
+        <v>46196.76800195602</v>
+      </c>
       <c r="D93" s="8">
-        <v>46195.50753101852</v>
+        <v>46196.76800386574</v>
       </c>
       <c r="E93" s="9" t="s">
         <v>200</v>
@@ -7205,9 +7229,11 @@
       <c r="B94" s="5">
         <v>46125.599890833335</v>
       </c>
-      <c r="C94" s="6"/>
+      <c r="C94" s="5">
+        <v>46196.768023020835</v>
+      </c>
       <c r="D94" s="5">
-        <v>46195.50752997685</v>
+        <v>46196.768024687495</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>200</v>
@@ -7258,9 +7284,11 @@
       <c r="B95" s="8">
         <v>46125.59993134259</v>
       </c>
-      <c r="C95" s="9"/>
+      <c r="C95" s="8">
+        <v>46196.76801494213</v>
+      </c>
       <c r="D95" s="8">
-        <v>46195.50753152778</v>
+        <v>46196.76801675926</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>200</v>
@@ -7311,9 +7339,11 @@
       <c r="B96" s="5">
         <v>46125.59996929398</v>
       </c>
-      <c r="C96" s="6"/>
+      <c r="C96" s="5">
+        <v>46196.76805109954</v>
+      </c>
       <c r="D96" s="5">
-        <v>46195.507530532406</v>
+        <v>46196.76805278935</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>200</v>
@@ -7364,9 +7394,11 @@
       <c r="B97" s="8">
         <v>46125.6000115162</v>
       </c>
-      <c r="C97" s="9"/>
+      <c r="C97" s="8">
+        <v>46196.76805706018</v>
+      </c>
       <c r="D97" s="8">
-        <v>46195.50753190972</v>
+        <v>46196.76805907408</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>200</v>
@@ -7417,9 +7449,11 @@
       <c r="B98" s="5">
         <v>46122.55164413195</v>
       </c>
-      <c r="C98" s="6"/>
+      <c r="C98" s="5">
+        <v>46196.76839824074</v>
+      </c>
       <c r="D98" s="5">
-        <v>46125.65705466435</v>
+        <v>46196.76840872686</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>292</v>
@@ -7467,10 +7501,10 @@
         <v>105</v>
       </c>
       <c r="T98" s="6">
-        <v>0</v>
-      </c>
-      <c r="U98" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U98" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -7480,9 +7514,11 @@
       <c r="B99" s="8">
         <v>46125.599162743056</v>
       </c>
-      <c r="C99" s="9"/>
+      <c r="C99" s="8">
+        <v>46196.76818966435</v>
+      </c>
       <c r="D99" s="8">
-        <v>46195.50752082176</v>
+        <v>46196.7681912963</v>
       </c>
       <c r="E99" s="9" t="s">
         <v>200</v>
@@ -7533,9 +7569,11 @@
       <c r="B100" s="5">
         <v>46125.599302511575</v>
       </c>
-      <c r="C100" s="6"/>
+      <c r="C100" s="5">
+        <v>46196.76820421296</v>
+      </c>
       <c r="D100" s="5">
-        <v>46195.507520127314</v>
+        <v>46196.76820597222</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>200</v>
@@ -7586,9 +7624,11 @@
       <c r="B101" s="8">
         <v>46125.59934644676</v>
       </c>
-      <c r="C101" s="9"/>
+      <c r="C101" s="8">
+        <v>46196.768375949076</v>
+      </c>
       <c r="D101" s="8">
-        <v>46195.507522314816</v>
+        <v>46196.76837958333</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>200</v>
@@ -7639,9 +7679,11 @@
       <c r="B102" s="5">
         <v>46125.59938857639</v>
       </c>
-      <c r="C102" s="6"/>
+      <c r="C102" s="5">
+        <v>46196.76837696759</v>
+      </c>
       <c r="D102" s="5">
-        <v>46195.50752153935</v>
+        <v>46196.76838008102</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>200</v>
@@ -7692,9 +7734,11 @@
       <c r="B103" s="8">
         <v>46125.59943094908</v>
       </c>
-      <c r="C103" s="9"/>
+      <c r="C103" s="8">
+        <v>46196.76837790509</v>
+      </c>
       <c r="D103" s="8">
-        <v>46195.50752328704</v>
+        <v>46196.768380520836</v>
       </c>
       <c r="E103" s="9" t="s">
         <v>200</v>
@@ -7745,9 +7789,11 @@
       <c r="B104" s="5">
         <v>46122.551650995374</v>
       </c>
-      <c r="C104" s="6"/>
+      <c r="C104" s="5">
+        <v>46196.76854788195</v>
+      </c>
       <c r="D104" s="5">
-        <v>46125.65705875</v>
+        <v>46196.76856074074</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>302</v>
@@ -7795,10 +7841,10 @@
         <v>105</v>
       </c>
       <c r="T104" s="6">
-        <v>0</v>
-      </c>
-      <c r="U104" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U104" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7808,9 +7854,11 @@
       <c r="B105" s="8">
         <v>46125.59953013889</v>
       </c>
-      <c r="C105" s="9"/>
+      <c r="C105" s="8">
+        <v>46196.76852783565</v>
+      </c>
       <c r="D105" s="8">
-        <v>46195.56328270833</v>
+        <v>46196.768531724534</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>200</v>
@@ -7861,9 +7909,11 @@
       <c r="B106" s="5">
         <v>46125.59961423611</v>
       </c>
-      <c r="C106" s="6"/>
+      <c r="C106" s="5">
+        <v>46196.76846329861</v>
+      </c>
       <c r="D106" s="5">
-        <v>46195.56328116899</v>
+        <v>46196.76846496528</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>200</v>
@@ -7914,9 +7964,11 @@
       <c r="B107" s="8">
         <v>46125.599654317135</v>
       </c>
-      <c r="C107" s="9"/>
+      <c r="C107" s="8">
+        <v>46196.768528796296</v>
+      </c>
       <c r="D107" s="8">
-        <v>46195.56328055555</v>
+        <v>46196.76853203704</v>
       </c>
       <c r="E107" s="9" t="s">
         <v>200</v>
@@ -7967,9 +8019,11 @@
       <c r="B108" s="5">
         <v>46125.59957065972</v>
       </c>
-      <c r="C108" s="6"/>
+      <c r="C108" s="5">
+        <v>46196.768529548615</v>
+      </c>
       <c r="D108" s="5">
-        <v>46195.56328217592</v>
+        <v>46196.76853233796</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>200</v>
@@ -8020,9 +8074,11 @@
       <c r="B109" s="8">
         <v>46125.59969711806</v>
       </c>
-      <c r="C109" s="9"/>
+      <c r="C109" s="8">
+        <v>46196.7685304051</v>
+      </c>
       <c r="D109" s="8">
-        <v>46195.563281724535</v>
+        <v>46196.76853265046</v>
       </c>
       <c r="E109" s="9" t="s">
         <v>200</v>
@@ -8073,9 +8129,11 @@
       <c r="B110" s="5">
         <v>46122.55163725694</v>
       </c>
-      <c r="C110" s="6"/>
+      <c r="C110" s="5">
+        <v>46196.76866755787</v>
+      </c>
       <c r="D110" s="5">
-        <v>46125.65706174768</v>
+        <v>46196.76867908565</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>310</v>
@@ -8123,10 +8181,10 @@
         <v>105</v>
       </c>
       <c r="T110" s="6">
-        <v>0</v>
-      </c>
-      <c r="U110" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U110" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
@@ -8136,9 +8194,11 @@
       <c r="B111" s="8">
         <v>46125.59780210648</v>
       </c>
-      <c r="C111" s="9"/>
+      <c r="C111" s="8">
+        <v>46196.76864902778</v>
+      </c>
       <c r="D111" s="8">
-        <v>46195.50753145834</v>
+        <v>46196.76865387731</v>
       </c>
       <c r="E111" s="9" t="s">
         <v>200</v>
@@ -8189,9 +8249,11 @@
       <c r="B112" s="5">
         <v>46125.597836932866</v>
       </c>
-      <c r="C112" s="6"/>
+      <c r="C112" s="5">
+        <v>46196.76865</v>
+      </c>
       <c r="D112" s="5">
-        <v>46195.50752924768</v>
+        <v>46196.76865427083</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>200</v>
@@ -8242,9 +8304,11 @@
       <c r="B113" s="8">
         <v>46125.5979208912</v>
       </c>
-      <c r="C113" s="9"/>
+      <c r="C113" s="8">
+        <v>46196.76865077546</v>
+      </c>
       <c r="D113" s="8">
-        <v>46195.507530347226</v>
+        <v>46196.76865460648</v>
       </c>
       <c r="E113" s="9" t="s">
         <v>200</v>
@@ -8295,9 +8359,11 @@
       <c r="B114" s="5">
         <v>46125.59788087963</v>
       </c>
-      <c r="C114" s="6"/>
+      <c r="C114" s="5">
+        <v>46196.768651527775</v>
+      </c>
       <c r="D114" s="5">
-        <v>46195.507528125</v>
+        <v>46196.768654942134</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>200</v>
@@ -8348,9 +8414,11 @@
       <c r="B115" s="8">
         <v>46125.597965023146</v>
       </c>
-      <c r="C115" s="9"/>
+      <c r="C115" s="8">
+        <v>46196.768652314815</v>
+      </c>
       <c r="D115" s="8">
-        <v>46195.507526608795</v>
+        <v>46196.768655312495</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>200</v>
@@ -8401,9 +8469,11 @@
       <c r="B116" s="5">
         <v>46122.55172043982</v>
       </c>
-      <c r="C116" s="6"/>
+      <c r="C116" s="5">
+        <v>46196.76877224537</v>
+      </c>
       <c r="D116" s="5">
-        <v>46125.658894120366</v>
+        <v>46196.768798784724</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>319</v>
@@ -8451,10 +8521,10 @@
         <v>105</v>
       </c>
       <c r="T116" s="6">
-        <v>0</v>
-      </c>
-      <c r="U116" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U116" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
@@ -8464,9 +8534,11 @@
       <c r="B117" s="8">
         <v>46125.60038253472</v>
       </c>
-      <c r="C117" s="9"/>
+      <c r="C117" s="8">
+        <v>46196.76875258102</v>
+      </c>
       <c r="D117" s="8">
-        <v>46125.658321932875</v>
+        <v>46196.768757337966</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>200</v>
@@ -8515,9 +8587,11 @@
       <c r="B118" s="5">
         <v>46125.60043012731</v>
       </c>
-      <c r="C118" s="6"/>
+      <c r="C118" s="5">
+        <v>46196.7687534838</v>
+      </c>
       <c r="D118" s="5">
-        <v>46125.658344236115</v>
+        <v>46196.76875768519</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>200</v>
@@ -8566,9 +8640,11 @@
       <c r="B119" s="8">
         <v>46125.60047290509</v>
       </c>
-      <c r="C119" s="9"/>
+      <c r="C119" s="8">
+        <v>46196.768754178236</v>
+      </c>
       <c r="D119" s="8">
-        <v>46125.65837160879</v>
+        <v>46196.76875800926</v>
       </c>
       <c r="E119" s="9" t="s">
         <v>200</v>
@@ -8617,9 +8693,11 @@
       <c r="B120" s="5">
         <v>46125.600514074074</v>
       </c>
-      <c r="C120" s="6"/>
+      <c r="C120" s="5">
+        <v>46196.768754930556</v>
+      </c>
       <c r="D120" s="5">
-        <v>46125.6583996875</v>
+        <v>46196.76875832176</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>200</v>
@@ -8668,9 +8746,11 @@
       <c r="B121" s="8">
         <v>46125.60055859954</v>
       </c>
-      <c r="C121" s="9"/>
+      <c r="C121" s="8">
+        <v>46196.7687558912</v>
+      </c>
       <c r="D121" s="8">
-        <v>46125.65844143518</v>
+        <v>46196.76875862268</v>
       </c>
       <c r="E121" s="9" t="s">
         <v>200</v>
@@ -8719,9 +8799,11 @@
       <c r="B122" s="5">
         <v>46122.55172986111</v>
       </c>
-      <c r="C122" s="6"/>
+      <c r="C122" s="5">
+        <v>46196.76917457176</v>
+      </c>
       <c r="D122" s="5">
-        <v>46125.66066717592</v>
+        <v>46196.76918584491</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>327</v>
@@ -8769,10 +8851,10 @@
         <v>105</v>
       </c>
       <c r="T122" s="6">
-        <v>0</v>
-      </c>
-      <c r="U122" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U122" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
@@ -8782,9 +8864,11 @@
       <c r="B123" s="8">
         <v>46125.60064416667</v>
       </c>
-      <c r="C123" s="9"/>
+      <c r="C123" s="8">
+        <v>46196.76915099537</v>
+      </c>
       <c r="D123" s="8">
-        <v>46125.66201921296</v>
+        <v>46196.76915743056</v>
       </c>
       <c r="E123" s="9" t="s">
         <v>200</v>
@@ -8833,9 +8917,11 @@
       <c r="B124" s="5">
         <v>46125.60068740741</v>
       </c>
-      <c r="C124" s="6"/>
+      <c r="C124" s="5">
+        <v>46196.76915237268</v>
+      </c>
       <c r="D124" s="5">
-        <v>46125.66205158565</v>
+        <v>46196.76915791667</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>200</v>
@@ -8884,9 +8970,11 @@
       <c r="B125" s="8">
         <v>46125.60073844907</v>
       </c>
-      <c r="C125" s="9"/>
+      <c r="C125" s="8">
+        <v>46196.76915341435</v>
+      </c>
       <c r="D125" s="8">
-        <v>46125.66207341435</v>
+        <v>46196.76915841435</v>
       </c>
       <c r="E125" s="9" t="s">
         <v>200</v>
@@ -8935,9 +9023,11 @@
       <c r="B126" s="5">
         <v>46125.60077622686</v>
       </c>
-      <c r="C126" s="6"/>
+      <c r="C126" s="5">
+        <v>46196.76915438657</v>
+      </c>
       <c r="D126" s="5">
-        <v>46125.66209603009</v>
+        <v>46196.769158842595</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>200</v>
@@ -8986,9 +9076,11 @@
       <c r="B127" s="8">
         <v>46125.600829143514</v>
       </c>
-      <c r="C127" s="9"/>
+      <c r="C127" s="8">
+        <v>46196.769155358794</v>
+      </c>
       <c r="D127" s="8">
-        <v>46125.66214039351</v>
+        <v>46196.76915931713</v>
       </c>
       <c r="E127" s="9" t="s">
         <v>200</v>
@@ -9041,7 +9133,7 @@
         <v>46195.56317517361</v>
       </c>
       <c r="D128" s="5">
-        <v>46195.56318964121</v>
+        <v>46196.76960409722</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>336</v>
@@ -9079,8 +9171,8 @@
       <c r="T128" s="6">
         <v>1</v>
       </c>
-      <c r="U128" s="11" t="s">
-        <v>33</v>
+      <c r="U128" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.25">
@@ -9090,9 +9182,11 @@
       <c r="B129" s="8">
         <v>46122.5517390625</v>
       </c>
-      <c r="C129" s="9"/>
+      <c r="C129" s="8">
+        <v>46196.76936652778</v>
+      </c>
       <c r="D129" s="8">
-        <v>46189.53573824074</v>
+        <v>46196.76939736111</v>
       </c>
       <c r="E129" s="9" t="s">
         <v>339</v>
@@ -9140,10 +9234,10 @@
         <v>105</v>
       </c>
       <c r="T129" s="9">
-        <v>0</v>
-      </c>
-      <c r="U129" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U129" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
@@ -9153,9 +9247,11 @@
       <c r="B130" s="5">
         <v>46125.60093731481</v>
       </c>
-      <c r="C130" s="6"/>
+      <c r="C130" s="5">
+        <v>46196.76934515046</v>
+      </c>
       <c r="D130" s="5">
-        <v>46125.664177071754</v>
+        <v>46196.769350682865</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>200</v>
@@ -9204,9 +9300,11 @@
       <c r="B131" s="8">
         <v>46125.601380821754</v>
       </c>
-      <c r="C131" s="9"/>
+      <c r="C131" s="8">
+        <v>46196.769346307876</v>
+      </c>
       <c r="D131" s="8">
-        <v>46125.66419668982</v>
+        <v>46196.769351145835</v>
       </c>
       <c r="E131" s="9" t="s">
         <v>200</v>
@@ -9255,9 +9353,11 @@
       <c r="B132" s="5">
         <v>46125.60142481481</v>
       </c>
-      <c r="C132" s="6"/>
+      <c r="C132" s="5">
+        <v>46196.7693472338</v>
+      </c>
       <c r="D132" s="5">
-        <v>46125.66421920139</v>
+        <v>46196.76935155093</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>200</v>
@@ -9306,9 +9406,11 @@
       <c r="B133" s="8">
         <v>46125.60146085648</v>
       </c>
-      <c r="C133" s="9"/>
+      <c r="C133" s="8">
+        <v>46196.769348125</v>
+      </c>
       <c r="D133" s="8">
-        <v>46125.66424142361</v>
+        <v>46196.76935192129</v>
       </c>
       <c r="E133" s="9" t="s">
         <v>200</v>
@@ -9357,9 +9459,11 @@
       <c r="B134" s="5">
         <v>46125.60150208333</v>
       </c>
-      <c r="C134" s="6"/>
+      <c r="C134" s="5">
+        <v>46196.769348981485</v>
+      </c>
       <c r="D134" s="5">
-        <v>46125.664280972225</v>
+        <v>46196.76935229167</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>200</v>
@@ -9408,9 +9512,11 @@
       <c r="B135" s="8">
         <v>46122.55174383102</v>
       </c>
-      <c r="C135" s="9"/>
+      <c r="C135" s="8">
+        <v>46196.769596921295</v>
+      </c>
       <c r="D135" s="8">
-        <v>46185.646541435184</v>
+        <v>46196.76961396991</v>
       </c>
       <c r="E135" s="9" t="s">
         <v>350</v>
@@ -9456,10 +9562,10 @@
         <v>105</v>
       </c>
       <c r="T135" s="9">
-        <v>0</v>
-      </c>
-      <c r="U135" s="10" t="s">
-        <v>109</v>
+        <v>1</v>
+      </c>
+      <c r="U135" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
@@ -9469,9 +9575,11 @@
       <c r="B136" s="5">
         <v>46125.601086979164</v>
       </c>
-      <c r="C136" s="6"/>
+      <c r="C136" s="5">
+        <v>46196.76947155093</v>
+      </c>
       <c r="D136" s="5">
-        <v>46125.66761228009</v>
+        <v>46196.76947347222</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>200</v>
@@ -9520,9 +9628,11 @@
       <c r="B137" s="8">
         <v>46125.60115318287</v>
       </c>
-      <c r="C137" s="9"/>
+      <c r="C137" s="8">
+        <v>46196.7695043287</v>
+      </c>
       <c r="D137" s="8">
-        <v>46125.66765621528</v>
+        <v>46196.76950902778</v>
       </c>
       <c r="E137" s="9" t="s">
         <v>200</v>
@@ -9571,9 +9681,11 @@
       <c r="B138" s="5">
         <v>46125.60120391204</v>
       </c>
-      <c r="C138" s="6"/>
+      <c r="C138" s="5">
+        <v>46196.76950549769</v>
+      </c>
       <c r="D138" s="5">
-        <v>46125.66769103009</v>
+        <v>46196.76950944445</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>200</v>
@@ -9622,9 +9734,11 @@
       <c r="B139" s="8">
         <v>46125.60125796296</v>
       </c>
-      <c r="C139" s="9"/>
+      <c r="C139" s="8">
+        <v>46196.76950637731</v>
+      </c>
       <c r="D139" s="8">
-        <v>46125.667712152775</v>
+        <v>46196.76950987268</v>
       </c>
       <c r="E139" s="9" t="s">
         <v>200</v>
@@ -9673,9 +9787,11 @@
       <c r="B140" s="5">
         <v>46125.601304282405</v>
       </c>
-      <c r="C140" s="6"/>
+      <c r="C140" s="5">
+        <v>46196.76950730324</v>
+      </c>
       <c r="D140" s="5">
-        <v>46125.6677272338</v>
+        <v>46196.769510266204</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>200</v>
@@ -9728,7 +9844,7 @@
         <v>46191.70598530093</v>
       </c>
       <c r="D141" s="8">
-        <v>46191.706001886574</v>
+        <v>46196.769715787035</v>
       </c>
       <c r="E141" s="9" t="s">
         <v>358</v>
@@ -9776,8 +9892,8 @@
       <c r="T141" s="9">
         <v>1</v>
       </c>
-      <c r="U141" s="11" t="s">
-        <v>33</v>
+      <c r="U141" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
@@ -9787,9 +9903,11 @@
       <c r="B142" s="5">
         <v>46125.60158650463</v>
       </c>
-      <c r="C142" s="6"/>
+      <c r="C142" s="5">
+        <v>46196.76968462963</v>
+      </c>
       <c r="D142" s="5">
-        <v>46125.76574587963</v>
+        <v>46196.76968989584</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>200</v>
@@ -9838,9 +9956,11 @@
       <c r="B143" s="8">
         <v>46125.60163133102</v>
       </c>
-      <c r="C143" s="9"/>
+      <c r="C143" s="8">
+        <v>46196.76968585648</v>
+      </c>
       <c r="D143" s="8">
-        <v>46125.7630881713</v>
+        <v>46196.7696903125</v>
       </c>
       <c r="E143" s="9" t="s">
         <v>200</v>
@@ -9889,9 +10009,11 @@
       <c r="B144" s="5">
         <v>46125.60167016204</v>
       </c>
-      <c r="C144" s="6"/>
+      <c r="C144" s="5">
+        <v>46196.7696866551</v>
+      </c>
       <c r="D144" s="5">
-        <v>46125.76385471065</v>
+        <v>46196.769690706016</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>200</v>
@@ -9940,9 +10062,11 @@
       <c r="B145" s="8">
         <v>46125.60170435185</v>
       </c>
-      <c r="C145" s="9"/>
+      <c r="C145" s="8">
+        <v>46196.769687395834</v>
+      </c>
       <c r="D145" s="8">
-        <v>46125.76313709491</v>
+        <v>46196.76969114583</v>
       </c>
       <c r="E145" s="9" t="s">
         <v>200</v>
@@ -9991,9 +10115,11 @@
       <c r="B146" s="5">
         <v>46125.60173947917</v>
       </c>
-      <c r="C146" s="6"/>
+      <c r="C146" s="5">
+        <v>46196.769688113425</v>
+      </c>
       <c r="D146" s="5">
-        <v>46125.763172210645</v>
+        <v>46196.76969164352</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>200</v>
@@ -10046,7 +10172,7 @@
         <v>46191.70604009259</v>
       </c>
       <c r="D147" s="8">
-        <v>46191.706057812495</v>
+        <v>46196.76981105324</v>
       </c>
       <c r="E147" s="9" t="s">
         <v>367</v>
@@ -10094,8 +10220,8 @@
       <c r="T147" s="9">
         <v>1</v>
       </c>
-      <c r="U147" s="11" t="s">
-        <v>33</v>
+      <c r="U147" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
@@ -10105,9 +10231,11 @@
       <c r="B148" s="5">
         <v>46125.60181555555</v>
       </c>
-      <c r="C148" s="6"/>
+      <c r="C148" s="5">
+        <v>46196.76979265046</v>
+      </c>
       <c r="D148" s="5">
-        <v>46125.76413488426</v>
+        <v>46196.76979569445</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>200</v>
@@ -10156,9 +10284,11 @@
       <c r="B149" s="8">
         <v>46125.60185690972</v>
       </c>
-      <c r="C149" s="9"/>
+      <c r="C149" s="8">
+        <v>46196.76979356482</v>
+      </c>
       <c r="D149" s="8">
-        <v>46125.764156805555</v>
+        <v>46196.76979614583</v>
       </c>
       <c r="E149" s="9" t="s">
         <v>200</v>
@@ -10207,9 +10337,11 @@
       <c r="B150" s="5">
         <v>46125.601899490735</v>
       </c>
-      <c r="C150" s="6"/>
+      <c r="C150" s="5">
+        <v>46196.769794224536</v>
+      </c>
       <c r="D150" s="5">
-        <v>46125.76418171296</v>
+        <v>46196.76979648148</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>200</v>
@@ -10258,9 +10390,11 @@
       <c r="B151" s="8">
         <v>46125.60193935185</v>
       </c>
-      <c r="C151" s="9"/>
+      <c r="C151" s="8">
+        <v>46196.76976476852</v>
+      </c>
       <c r="D151" s="8">
-        <v>46125.764207615735</v>
+        <v>46196.769766875004</v>
       </c>
       <c r="E151" s="9" t="s">
         <v>200</v>
@@ -10309,9 +10443,11 @@
       <c r="B152" s="5">
         <v>46125.60197710648</v>
       </c>
-      <c r="C152" s="6"/>
+      <c r="C152" s="5">
+        <v>46196.76977206019</v>
+      </c>
       <c r="D152" s="5">
-        <v>46125.764245451384</v>
+        <v>46196.76977370371</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>200</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-26 12:53 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -4848,7 +4848,7 @@
         <v>46134.79245146991</v>
       </c>
       <c r="D53" s="8">
-        <v>46191.18981792824</v>
+        <v>46199.18371805556</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>83</v>
@@ -4890,8 +4890,8 @@
       <c r="R53" s="8">
         <v>46198</v>
       </c>
-      <c r="S53" s="12" t="s">
-        <v>74</v>
+      <c r="S53" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T53" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-30 12:52 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -2778,7 +2778,7 @@
         <v>46181.666399050926</v>
       </c>
       <c r="D19" s="8">
-        <v>46195.20558476852</v>
+        <v>46203.203668229165</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>80</v>
@@ -2822,8 +2822,8 @@
       <c r="R19" s="8">
         <v>46202</v>
       </c>
-      <c r="S19" s="12" t="s">
-        <v>74</v>
+      <c r="S19" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T19" s="9">
         <v>1</v>
@@ -2908,7 +2908,7 @@
         <v>46181.66636053241</v>
       </c>
       <c r="D21" s="8">
-        <v>46195.20558446759</v>
+        <v>46203.20366833333</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>89</v>
@@ -2952,8 +2952,8 @@
       <c r="R21" s="8">
         <v>46202</v>
       </c>
-      <c r="S21" s="12" t="s">
-        <v>74</v>
+      <c r="S21" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T21" s="9">
         <v>1</v>
@@ -2973,7 +2973,7 @@
         <v>46181.66637630787</v>
       </c>
       <c r="D22" s="5">
-        <v>46195.20558434028</v>
+        <v>46203.20366849537</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -3017,8 +3017,8 @@
       <c r="R22" s="5">
         <v>46202</v>
       </c>
-      <c r="S22" s="12" t="s">
-        <v>74</v>
+      <c r="S22" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T22" s="6">
         <v>1</v>
@@ -3038,7 +3038,7 @@
         <v>46181.66643224537</v>
       </c>
       <c r="D23" s="8">
-        <v>46195.205584386575</v>
+        <v>46203.2036682176</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>95</v>
@@ -3082,8 +3082,8 @@
       <c r="R23" s="8">
         <v>46202</v>
       </c>
-      <c r="S23" s="12" t="s">
-        <v>74</v>
+      <c r="S23" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T23" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-03 12:59 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -3778,7 +3778,7 @@
         <v>46181.66687207176</v>
       </c>
       <c r="D35" s="8">
-        <v>46181.66688577546</v>
+        <v>46206.19763560186</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>136</v>
@@ -3822,8 +3822,8 @@
       <c r="R35" s="8">
         <v>46213</v>
       </c>
-      <c r="S35" s="11" t="s">
-        <v>105</v>
+      <c r="S35" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T35" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-08 13:56 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -4490,7 +4490,7 @@
         <v>46181.66722120371</v>
       </c>
       <c r="D47" s="8">
-        <v>46181.66723511574</v>
+        <v>46211.17825179399</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>173</v>
@@ -4534,8 +4534,8 @@
       <c r="R47" s="8">
         <v>46218</v>
       </c>
-      <c r="S47" s="11" t="s">
-        <v>105</v>
+      <c r="S47" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T47" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-10 13:27 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -4140,7 +4140,7 @@
         <v>46181.666767002316</v>
       </c>
       <c r="D41" s="8">
-        <v>46181.666783252316</v>
+        <v>46213.20535120371</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>155</v>
@@ -4184,8 +4184,8 @@
       <c r="R41" s="8">
         <v>46220</v>
       </c>
-      <c r="S41" s="11" t="s">
-        <v>105</v>
+      <c r="S41" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T41" s="9">
         <v>1</v>
@@ -5418,7 +5418,7 @@
         <v>46181.667430127316</v>
       </c>
       <c r="D63" s="8">
-        <v>46181.66744925926</v>
+        <v>46213.20535071759</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>218</v>
@@ -5462,8 +5462,8 @@
       <c r="R63" s="8">
         <v>46220</v>
       </c>
-      <c r="S63" s="11" t="s">
-        <v>105</v>
+      <c r="S63" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T63" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-11 10:33 Chile
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -3778,7 +3778,7 @@
         <v>46181.66687207176</v>
       </c>
       <c r="D35" s="8">
-        <v>46206.19763560186</v>
+        <v>46214.17760775463</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>136</v>
@@ -3822,8 +3822,8 @@
       <c r="R35" s="8">
         <v>46213</v>
       </c>
-      <c r="S35" s="12" t="s">
-        <v>74</v>
+      <c r="S35" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T35" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-16 15:04 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -4471,7 +4471,7 @@
         <v>46181.66722120371</v>
       </c>
       <c r="D47" s="8">
-        <v>46211.17825179399</v>
+        <v>46219.16816725694</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>170</v>
@@ -4515,8 +4515,8 @@
       <c r="R47" s="8">
         <v>46218</v>
       </c>
-      <c r="S47" s="12" t="s">
-        <v>74</v>
+      <c r="S47" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T47" s="9">
         <v>1</v>
@@ -5464,7 +5464,7 @@
         <v>46181.66775587963</v>
       </c>
       <c r="D64" s="5">
-        <v>46181.66777241898</v>
+        <v>46219.19909722223</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>213</v>
@@ -5508,8 +5508,8 @@
       <c r="R64" s="5">
         <v>46226</v>
       </c>
-      <c r="S64" s="11" t="s">
-        <v>102</v>
+      <c r="S64" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T64" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-28 15:24 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -4312,7 +4312,7 @@
         <v>46181.666958472226</v>
       </c>
       <c r="D44" s="5">
-        <v>46223.42579010417</v>
+        <v>46231.18084584491</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4356,8 +4356,8 @@
       <c r="R44" s="5">
         <v>46238</v>
       </c>
-      <c r="S44" s="11" t="s">
-        <v>104</v>
+      <c r="S44" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T44" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-30 15:16 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -6652,7 +6652,7 @@
         <v>46193.93315311342</v>
       </c>
       <c r="D84" s="5">
-        <v>46193.9332800463</v>
+        <v>46233.180653414354</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>266</v>
@@ -6696,8 +6696,8 @@
       <c r="R84" s="5">
         <v>46240</v>
       </c>
-      <c r="S84" s="11" t="s">
-        <v>104</v>
+      <c r="S84" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T84" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-04 14:23 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -5594,7 +5594,7 @@
         <v>46181.666093576394</v>
       </c>
       <c r="D66" s="5">
-        <v>46230.185321261575</v>
+        <v>46238.1884728125</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>228</v>
@@ -5638,8 +5638,8 @@
       <c r="R66" s="5">
         <v>46237</v>
       </c>
-      <c r="S66" s="12" t="s">
-        <v>74</v>
+      <c r="S66" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T66" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-05 15:23 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -4312,7 +4312,7 @@
         <v>46181.666958472226</v>
       </c>
       <c r="D44" s="5">
-        <v>46231.18084584491</v>
+        <v>46239.17159243056</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4356,8 +4356,8 @@
       <c r="R44" s="5">
         <v>46238</v>
       </c>
-      <c r="S44" s="12" t="s">
-        <v>74</v>
+      <c r="S44" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T44" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-06 11:27 Chile
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -6392,7 +6392,7 @@
         <v>46195.563269363425</v>
       </c>
       <c r="D80" s="5">
-        <v>46195.711846817125</v>
+        <v>46240.605594189816</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>257</v>
@@ -6442,8 +6442,8 @@
       <c r="T80" s="6">
         <v>1</v>
       </c>
-      <c r="U80" s="12" t="s">
-        <v>115</v>
+      <c r="U80" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -9183,7 +9183,7 @@
         <v>46196.76936652778</v>
       </c>
       <c r="D129" s="8">
-        <v>46196.76939736111</v>
+        <v>46240.60562268519</v>
       </c>
       <c r="E129" s="9" t="s">
         <v>338</v>
@@ -9233,8 +9233,8 @@
       <c r="T129" s="9">
         <v>1</v>
       </c>
-      <c r="U129" s="12" t="s">
-        <v>115</v>
+      <c r="U129" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
@@ -9841,7 +9841,7 @@
         <v>46191.70598530093</v>
       </c>
       <c r="D141" s="8">
-        <v>46228.14621358796</v>
+        <v>46240.605638368055</v>
       </c>
       <c r="E141" s="9" t="s">
         <v>357</v>
@@ -9889,8 +9889,8 @@
       <c r="T141" s="9">
         <v>1</v>
       </c>
-      <c r="U141" s="12" t="s">
-        <v>115</v>
+      <c r="U141" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
@@ -10169,7 +10169,7 @@
         <v>46191.70604009259</v>
       </c>
       <c r="D147" s="8">
-        <v>46196.76981105324</v>
+        <v>46240.60565322917</v>
       </c>
       <c r="E147" s="9" t="s">
         <v>366</v>
@@ -10217,8 +10217,8 @@
       <c r="T147" s="9">
         <v>1</v>
       </c>
-      <c r="U147" s="12" t="s">
-        <v>115</v>
+      <c r="U147" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-07 14:23 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -6652,7 +6652,7 @@
         <v>46193.93315311342</v>
       </c>
       <c r="D84" s="5">
-        <v>46233.180653414354</v>
+        <v>46241.18852804398</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>266</v>
@@ -6696,8 +6696,8 @@
       <c r="R84" s="5">
         <v>46240</v>
       </c>
-      <c r="S84" s="12" t="s">
-        <v>74</v>
+      <c r="S84" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T84" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-14 14:26 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -5659,7 +5659,7 @@
         <v>46181.6661986574</v>
       </c>
       <c r="D67" s="8">
-        <v>46228.10617515046</v>
+        <v>46248.187867650464</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>233</v>
@@ -5703,8 +5703,8 @@
       <c r="R67" s="8">
         <v>46255</v>
       </c>
-      <c r="S67" s="11" t="s">
-        <v>104</v>
+      <c r="S67" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T67" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-18 13:49 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -5999,7 +5999,7 @@
         <v>46181.66878061343</v>
       </c>
       <c r="D73" s="8">
-        <v>46228.106273067126</v>
+        <v>46252.20192400463</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>244</v>
@@ -6043,8 +6043,8 @@
       <c r="R73" s="8">
         <v>46259</v>
       </c>
-      <c r="S73" s="11" t="s">
-        <v>104</v>
+      <c r="S73" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T73" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-22 09:44 Chile
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -5659,7 +5659,7 @@
         <v>46181.6661986574</v>
       </c>
       <c r="D67" s="8">
-        <v>46248.187867650464</v>
+        <v>46256.20327105324</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>233</v>
@@ -5703,8 +5703,8 @@
       <c r="R67" s="8">
         <v>46255</v>
       </c>
-      <c r="S67" s="12" t="s">
-        <v>74</v>
+      <c r="S67" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T67" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-24 13:55 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -386,16 +386,16 @@
     <t>Generación OC Alabe - OT 4302,Fabricación Alabe - OT 4302</t>
   </si>
   <si>
+    <t>1214005097392571</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe - OT 4302</t>
+  </si>
+  <si>
+    <t>Alabe- OT 4302,Fabricación Alabe - OT 4302</t>
+  </si>
+  <si>
     <t>Baja</t>
-  </si>
-  <si>
-    <t>1214005097392571</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe - OT 4302</t>
-  </si>
-  <si>
-    <t>Alabe- OT 4302,Fabricación Alabe - OT 4302</t>
   </si>
   <si>
     <t>Tarea sin iniciar</t>
@@ -1844,13 +1844,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46122.55118912037</v>
+        <v>46122.38452245371</v>
       </c>
       <c r="C4" s="5">
-        <v>46128.59300771991</v>
+        <v>46128.426341053244</v>
       </c>
       <c r="D4" s="5">
-        <v>46158.10300121528</v>
+        <v>46157.93633454861</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1893,13 +1893,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46122.55134571759</v>
+        <v>46122.38467905093</v>
       </c>
       <c r="C5" s="8">
-        <v>46128.59299462963</v>
+        <v>46128.42632796297</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.876021724536</v>
+        <v>46133.70935505787</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1956,13 +1956,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46122.55134947917</v>
+        <v>46122.384682812495</v>
       </c>
       <c r="C6" s="5">
-        <v>46128.59267868055</v>
+        <v>46128.42601201389</v>
       </c>
       <c r="D6" s="5">
-        <v>46128.60382631945</v>
+        <v>46128.43715965278</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -2019,13 +2019,13 @@
         <v>37</v>
       </c>
       <c r="B7" s="8">
-        <v>46122.551352546296</v>
+        <v>46122.38468587963</v>
       </c>
       <c r="C7" s="8">
-        <v>46128.59269866898</v>
+        <v>46128.42603200232</v>
       </c>
       <c r="D7" s="8">
-        <v>46161.62726047453</v>
+        <v>46161.460593807875</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>38</v>
@@ -2082,13 +2082,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46122.551355567135</v>
+        <v>46122.38468890046</v>
       </c>
       <c r="C8" s="5">
-        <v>46128.59271722222</v>
+        <v>46128.42605055556</v>
       </c>
       <c r="D8" s="5">
-        <v>46128.60400607639</v>
+        <v>46128.43733940972</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -2145,13 +2145,13 @@
         <v>44</v>
       </c>
       <c r="B9" s="8">
-        <v>46122.551359386576</v>
+        <v>46122.384692719905</v>
       </c>
       <c r="C9" s="8">
-        <v>46128.592850057874</v>
+        <v>46128.4261833912</v>
       </c>
       <c r="D9" s="8">
-        <v>46156.83577310185</v>
+        <v>46156.66910643518</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>45</v>
@@ -2208,13 +2208,13 @@
         <v>47</v>
       </c>
       <c r="B10" s="5">
-        <v>46122.55119412037</v>
+        <v>46122.3845274537</v>
       </c>
       <c r="C10" s="5">
-        <v>46193.93280347223</v>
+        <v>46193.766136805556</v>
       </c>
       <c r="D10" s="5">
-        <v>46223.423621180555</v>
+        <v>46223.25695451389</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>48</v>
@@ -2261,13 +2261,13 @@
         <v>50</v>
       </c>
       <c r="B11" s="8">
-        <v>46122.5513631713</v>
+        <v>46122.384696504625</v>
       </c>
       <c r="C11" s="8">
-        <v>46128.60435520833</v>
+        <v>46128.43768854167</v>
       </c>
       <c r="D11" s="8">
-        <v>46192.97382803241</v>
+        <v>46192.80716136574</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>51</v>
@@ -2326,13 +2326,13 @@
         <v>54</v>
       </c>
       <c r="B12" s="5">
-        <v>46122.551369050925</v>
+        <v>46122.38470238426</v>
       </c>
       <c r="C12" s="5">
-        <v>46128.60643114583</v>
+        <v>46128.43976447917</v>
       </c>
       <c r="D12" s="5">
-        <v>46192.97382813657</v>
+        <v>46192.80716146991</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>55</v>
@@ -2391,13 +2391,13 @@
         <v>58</v>
       </c>
       <c r="B13" s="8">
-        <v>46122.5513746875</v>
+        <v>46122.384708020836</v>
       </c>
       <c r="C13" s="8">
-        <v>46132.57072561343</v>
+        <v>46132.40405894676</v>
       </c>
       <c r="D13" s="8">
-        <v>46192.97382800926</v>
+        <v>46192.80716134259</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>59</v>
@@ -2456,13 +2456,13 @@
         <v>61</v>
       </c>
       <c r="B14" s="5">
-        <v>46122.553594178244</v>
+        <v>46122.38692751157</v>
       </c>
       <c r="C14" s="5">
-        <v>46128.60941575232</v>
+        <v>46128.44274908565</v>
       </c>
       <c r="D14" s="5">
-        <v>46136.20601917824</v>
+        <v>46136.03935251157</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>62</v>
@@ -2521,13 +2521,13 @@
         <v>65</v>
       </c>
       <c r="B15" s="8">
-        <v>46122.55119946759</v>
+        <v>46122.38453280093</v>
       </c>
       <c r="C15" s="8">
-        <v>46195.50723163194</v>
+        <v>46195.34056496528</v>
       </c>
       <c r="D15" s="8">
-        <v>46228.10468802083</v>
+        <v>46227.938021354166</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>66</v>
@@ -2574,13 +2574,13 @@
         <v>68</v>
       </c>
       <c r="B16" s="5">
-        <v>46122.55138855324</v>
+        <v>46122.38472188657</v>
       </c>
       <c r="C16" s="5">
-        <v>46128.60700391204</v>
+        <v>46128.44033724537</v>
       </c>
       <c r="D16" s="5">
-        <v>46133.17999505787</v>
+        <v>46133.0133283912</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>69</v>
@@ -2639,13 +2639,13 @@
         <v>71</v>
       </c>
       <c r="B17" s="8">
-        <v>46122.55139482639</v>
+        <v>46122.38472815973</v>
       </c>
       <c r="C17" s="8">
-        <v>46128.60701157407</v>
+        <v>46128.44034490741</v>
       </c>
       <c r="D17" s="8">
-        <v>46132.182206921294</v>
+        <v>46132.01554025463</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>72</v>
@@ -2704,13 +2704,13 @@
         <v>75</v>
       </c>
       <c r="B18" s="5">
-        <v>46122.55140040509</v>
+        <v>46122.38473373842</v>
       </c>
       <c r="C18" s="5">
-        <v>46195.50721171296</v>
+        <v>46195.340545046296</v>
       </c>
       <c r="D18" s="5">
-        <v>46223.606554259255</v>
+        <v>46223.43988759259</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>76</v>
@@ -2769,13 +2769,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46122.55140604167</v>
+        <v>46122.384739375004</v>
       </c>
       <c r="C19" s="8">
-        <v>46181.666399050926</v>
+        <v>46181.499732384254</v>
       </c>
       <c r="D19" s="8">
-        <v>46223.606550833334</v>
+        <v>46223.43988416667</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2834,13 +2834,13 @@
         <v>84</v>
       </c>
       <c r="B20" s="5">
-        <v>46122.55141162037</v>
+        <v>46122.3847449537</v>
       </c>
       <c r="C20" s="5">
-        <v>46128.609497881946</v>
+        <v>46128.442831215274</v>
       </c>
       <c r="D20" s="5">
-        <v>46132.1822065625</v>
+        <v>46132.01553989583</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>64</v>
@@ -2899,13 +2899,13 @@
         <v>87</v>
       </c>
       <c r="B21" s="8">
-        <v>46122.566545787035</v>
+        <v>46122.39987912037</v>
       </c>
       <c r="C21" s="8">
-        <v>46181.66636053241</v>
+        <v>46181.49969386574</v>
       </c>
       <c r="D21" s="8">
-        <v>46223.60654709491</v>
+        <v>46223.43988042824</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>88</v>
@@ -2964,13 +2964,13 @@
         <v>90</v>
       </c>
       <c r="B22" s="5">
-        <v>46122.56661521991</v>
+        <v>46122.39994855324</v>
       </c>
       <c r="C22" s="5">
-        <v>46181.66637630787</v>
+        <v>46181.499709641204</v>
       </c>
       <c r="D22" s="5">
-        <v>46223.60654385417</v>
+        <v>46223.4398771875</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>91</v>
@@ -3029,13 +3029,13 @@
         <v>93</v>
       </c>
       <c r="B23" s="8">
-        <v>46122.57286273148</v>
+        <v>46122.40619606481</v>
       </c>
       <c r="C23" s="8">
-        <v>46181.66643224537</v>
+        <v>46181.4997655787</v>
       </c>
       <c r="D23" s="8">
-        <v>46223.60653833333</v>
+        <v>46223.43987166666</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>94</v>
@@ -3094,13 +3094,13 @@
         <v>96</v>
       </c>
       <c r="B24" s="5">
-        <v>46122.55120394676</v>
+        <v>46122.38453728009</v>
       </c>
       <c r="C24" s="5">
-        <v>46195.50733982639</v>
+        <v>46195.34067315972</v>
       </c>
       <c r="D24" s="5">
-        <v>46223.425103263886</v>
+        <v>46223.25843659722</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>97</v>
@@ -3147,13 +3147,13 @@
         <v>99</v>
       </c>
       <c r="B25" s="8">
-        <v>46122.55141694444</v>
+        <v>46122.38475027778</v>
       </c>
       <c r="C25" s="8">
-        <v>46174.626168703704</v>
+        <v>46174.45950203703</v>
       </c>
       <c r="D25" s="8">
-        <v>46250.21356391204</v>
+        <v>46258.02963747685</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>100</v>
@@ -3197,8 +3197,8 @@
       <c r="R25" s="8">
         <v>46265</v>
       </c>
-      <c r="S25" s="11" t="s">
-        <v>104</v>
+      <c r="S25" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T25" s="9">
         <v>1</v>
@@ -3209,19 +3209,19 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B26" s="5">
+        <v>46122.38475541667</v>
+      </c>
+      <c r="C26" s="5">
+        <v>46174.45658625</v>
+      </c>
+      <c r="D26" s="5">
+        <v>46174.456587824076</v>
+      </c>
+      <c r="E26" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="B26" s="5">
-        <v>46122.55142208333</v>
-      </c>
-      <c r="C26" s="5">
-        <v>46174.62325291667</v>
-      </c>
-      <c r="D26" s="5">
-        <v>46174.62325449074</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>106</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
@@ -3254,12 +3254,12 @@
         <v>72</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q26" s="6"/>
       <c r="R26" s="6"/>
       <c r="S26" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T26" s="6">
         <v>0</v>
@@ -3273,13 +3273,13 @@
         <v>109</v>
       </c>
       <c r="B27" s="8">
-        <v>46122.55142699074</v>
+        <v>46122.38476032407</v>
       </c>
       <c r="C27" s="8">
-        <v>46174.626152893514</v>
+        <v>46174.45948622686</v>
       </c>
       <c r="D27" s="8">
-        <v>46174.62615429398</v>
+        <v>46174.45948762732</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>110</v>
@@ -3312,7 +3312,7 @@
         <v>100</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P27" s="9" t="s">
         <v>111</v>
@@ -3320,7 +3320,7 @@
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
       <c r="S27" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T27" s="9">
         <v>0</v>
@@ -3334,13 +3334,13 @@
         <v>112</v>
       </c>
       <c r="B28" s="5">
-        <v>46122.5514322338</v>
+        <v>46122.38476556713</v>
       </c>
       <c r="C28" s="5">
-        <v>46195.50732521991</v>
+        <v>46195.340658553236</v>
       </c>
       <c r="D28" s="5">
-        <v>46195.71184679398</v>
+        <v>46195.545180127316</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>113</v>
@@ -3399,13 +3399,13 @@
         <v>116</v>
       </c>
       <c r="B29" s="8">
-        <v>46122.551437546295</v>
+        <v>46122.38477087963</v>
       </c>
       <c r="C29" s="8">
-        <v>46195.71138274306</v>
+        <v>46195.54471607639</v>
       </c>
       <c r="D29" s="8">
-        <v>46195.71138517361</v>
+        <v>46195.54471850695</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>117</v>
@@ -3446,7 +3446,7 @@
       <c r="Q29" s="9"/>
       <c r="R29" s="9"/>
       <c r="S29" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T29" s="9">
         <v>0</v>
@@ -3460,13 +3460,13 @@
         <v>119</v>
       </c>
       <c r="B30" s="5">
-        <v>46122.55144255787</v>
+        <v>46122.3847758912</v>
       </c>
       <c r="C30" s="5">
-        <v>46195.711830960645</v>
+        <v>46195.54516429398</v>
       </c>
       <c r="D30" s="5">
-        <v>46195.711832500005</v>
+        <v>46195.54516583333</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>120</v>
@@ -3507,7 +3507,7 @@
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T30" s="6">
         <v>0</v>
@@ -3521,13 +3521,13 @@
         <v>122</v>
       </c>
       <c r="B31" s="8">
-        <v>46122.551447708334</v>
+        <v>46122.38478104166</v>
       </c>
       <c r="C31" s="8">
-        <v>46133.82779993056</v>
+        <v>46133.661133263886</v>
       </c>
       <c r="D31" s="8">
-        <v>46133.82781321759</v>
+        <v>46133.66114655093</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>123</v>
@@ -3572,7 +3572,7 @@
         <v>46308</v>
       </c>
       <c r="S31" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T31" s="9">
         <v>1</v>
@@ -3586,13 +3586,13 @@
         <v>125</v>
       </c>
       <c r="B32" s="5">
-        <v>46122.5514527662</v>
+        <v>46122.38478609954</v>
       </c>
       <c r="C32" s="5">
-        <v>46133.827731122685</v>
+        <v>46133.66106445601</v>
       </c>
       <c r="D32" s="5">
-        <v>46133.82773260417</v>
+        <v>46133.6610659375</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>126</v>
@@ -3633,7 +3633,7 @@
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T32" s="6">
         <v>0</v>
@@ -3647,13 +3647,13 @@
         <v>128</v>
       </c>
       <c r="B33" s="8">
-        <v>46122.55145796297</v>
+        <v>46122.384791296296</v>
       </c>
       <c r="C33" s="8">
-        <v>46133.827786875</v>
+        <v>46133.66112020833</v>
       </c>
       <c r="D33" s="8">
-        <v>46133.82778807871</v>
+        <v>46133.661121412035</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>129</v>
@@ -3694,7 +3694,7 @@
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
       <c r="S33" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T33" s="9">
         <v>0</v>
@@ -3708,13 +3708,13 @@
         <v>131</v>
       </c>
       <c r="B34" s="5">
-        <v>46122.55146299768</v>
+        <v>46122.38479633102</v>
       </c>
       <c r="C34" s="5">
-        <v>46133.82776796297</v>
+        <v>46133.6611012963</v>
       </c>
       <c r="D34" s="5">
-        <v>46133.827769131945</v>
+        <v>46133.66110246528</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>132</v>
@@ -3755,7 +3755,7 @@
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
@@ -3769,13 +3769,13 @@
         <v>134</v>
       </c>
       <c r="B35" s="8">
-        <v>46122.55146795139</v>
+        <v>46122.38480128472</v>
       </c>
       <c r="C35" s="8">
-        <v>46181.66687207176</v>
+        <v>46181.50020540509</v>
       </c>
       <c r="D35" s="8">
-        <v>46214.17760775463</v>
+        <v>46214.01094108797</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>135</v>
@@ -3834,13 +3834,13 @@
         <v>139</v>
       </c>
       <c r="B36" s="5">
-        <v>46122.551472974534</v>
+        <v>46122.38480630787</v>
       </c>
       <c r="C36" s="5">
-        <v>46181.66681767361</v>
+        <v>46181.50015100694</v>
       </c>
       <c r="D36" s="5">
-        <v>46181.66681946759</v>
+        <v>46181.50015280093</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>140</v>
@@ -3881,7 +3881,7 @@
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
       <c r="S36" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T36" s="6">
         <v>0</v>
@@ -3895,13 +3895,13 @@
         <v>142</v>
       </c>
       <c r="B37" s="8">
-        <v>46122.55152253472</v>
+        <v>46122.384855868055</v>
       </c>
       <c r="C37" s="8">
-        <v>46181.66685679398</v>
+        <v>46181.50019012731</v>
       </c>
       <c r="D37" s="8">
-        <v>46181.66685818287</v>
+        <v>46181.5001915162</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>143</v>
@@ -3942,7 +3942,7 @@
       <c r="Q37" s="9"/>
       <c r="R37" s="9"/>
       <c r="S37" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T37" s="9">
         <v>0</v>
@@ -3956,13 +3956,13 @@
         <v>145</v>
       </c>
       <c r="B38" s="5">
-        <v>46122.55152891204</v>
+        <v>46122.384862245366</v>
       </c>
       <c r="C38" s="5">
-        <v>46154.867667812505</v>
+        <v>46154.70100114583</v>
       </c>
       <c r="D38" s="5">
-        <v>46189.172213136575</v>
+        <v>46189.00554646991</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>146</v>
@@ -4021,13 +4021,13 @@
         <v>148</v>
       </c>
       <c r="B39" s="8">
-        <v>46122.5515340625</v>
+        <v>46122.384867395835</v>
       </c>
       <c r="C39" s="8">
-        <v>46154.86751693287</v>
+        <v>46154.70085026621</v>
       </c>
       <c r="D39" s="8">
-        <v>46154.86751927083</v>
+        <v>46154.70085260417</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>86</v>
@@ -4076,13 +4076,13 @@
         <v>150</v>
       </c>
       <c r="B40" s="5">
-        <v>46122.55153844907</v>
+        <v>46122.38487178241</v>
       </c>
       <c r="C40" s="5">
-        <v>46154.867576273144</v>
+        <v>46154.70090960649</v>
       </c>
       <c r="D40" s="5">
-        <v>46154.867577453704</v>
+        <v>46154.70091078704</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>151</v>
@@ -4131,13 +4131,13 @@
         <v>153</v>
       </c>
       <c r="B41" s="8">
-        <v>46122.574933449076</v>
+        <v>46122.40826678241</v>
       </c>
       <c r="C41" s="8">
-        <v>46181.666767002316</v>
+        <v>46181.500100335645</v>
       </c>
       <c r="D41" s="8">
-        <v>46221.20228239583</v>
+        <v>46221.03561572917</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>154</v>
@@ -4196,13 +4196,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46122.575920972224</v>
+        <v>46122.40925430556</v>
       </c>
       <c r="C42" s="5">
-        <v>46181.66670739584</v>
+        <v>46181.500040729166</v>
       </c>
       <c r="D42" s="5">
-        <v>46181.66670855324</v>
+        <v>46181.500041886575</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>89</v>
@@ -4251,13 +4251,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46122.57608475695</v>
+        <v>46122.409418090276</v>
       </c>
       <c r="C43" s="8">
-        <v>46181.666752812496</v>
+        <v>46181.50008614583</v>
       </c>
       <c r="D43" s="8">
-        <v>46181.666754351856</v>
+        <v>46181.500087685185</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4306,13 +4306,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46122.57501438657</v>
+        <v>46122.40834771991</v>
       </c>
       <c r="C44" s="5">
-        <v>46181.666958472226</v>
+        <v>46181.500291805554</v>
       </c>
       <c r="D44" s="5">
-        <v>46239.17159243056</v>
+        <v>46239.00492576389</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4371,13 +4371,13 @@
         <v>166</v>
       </c>
       <c r="B45" s="8">
-        <v>46122.57922111111</v>
+        <v>46122.41255444444</v>
       </c>
       <c r="C45" s="8">
-        <v>46181.666901516204</v>
+        <v>46181.50023484953</v>
       </c>
       <c r="D45" s="8">
-        <v>46181.66690306713</v>
+        <v>46181.50023640046</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>95</v>
@@ -4426,13 +4426,13 @@
         <v>168</v>
       </c>
       <c r="B46" s="5">
-        <v>46122.57949202546</v>
+        <v>46122.4128253588</v>
       </c>
       <c r="C46" s="5">
-        <v>46181.66694322917</v>
+        <v>46181.500276562496</v>
       </c>
       <c r="D46" s="5">
-        <v>46181.66694460648</v>
+        <v>46181.50027793982</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>169</v>
@@ -4481,13 +4481,13 @@
         <v>171</v>
       </c>
       <c r="B47" s="8">
-        <v>46125.529618217595</v>
+        <v>46125.362951550924</v>
       </c>
       <c r="C47" s="8">
-        <v>46181.66722120371</v>
+        <v>46181.50055453704</v>
       </c>
       <c r="D47" s="8">
-        <v>46228.07776863426</v>
+        <v>46227.91110196759</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>172</v>
@@ -4546,13 +4546,13 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46125.52977997685</v>
+        <v>46125.36311331019</v>
       </c>
       <c r="C48" s="5">
-        <v>46181.66715732639</v>
+        <v>46181.50049065972</v>
       </c>
       <c r="D48" s="5">
-        <v>46181.66715912037</v>
+        <v>46181.500492453706</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>92</v>
@@ -4601,13 +4601,13 @@
         <v>176</v>
       </c>
       <c r="B49" s="8">
-        <v>46125.52991815972</v>
+        <v>46125.36325149305</v>
       </c>
       <c r="C49" s="8">
-        <v>46181.66720412037</v>
+        <v>46181.5005374537</v>
       </c>
       <c r="D49" s="8">
-        <v>46181.66720563658</v>
+        <v>46181.50053896991</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>177</v>
@@ -4656,13 +4656,13 @@
         <v>179</v>
       </c>
       <c r="B50" s="5">
-        <v>46122.55120855324</v>
+        <v>46122.384541886575</v>
       </c>
       <c r="C50" s="5">
-        <v>46195.5074512963</v>
+        <v>46195.34078462963</v>
       </c>
       <c r="D50" s="5">
-        <v>46195.50756488426</v>
+        <v>46195.34089821759</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>180</v>
@@ -4709,13 +4709,13 @@
         <v>182</v>
       </c>
       <c r="B51" s="8">
-        <v>46122.55154344907</v>
+        <v>46122.38487678241</v>
       </c>
       <c r="C51" s="8">
-        <v>46133.79584481481</v>
+        <v>46133.62917814815</v>
       </c>
       <c r="D51" s="8">
-        <v>46143.171145879634</v>
+        <v>46143.00447921296</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>183</v>
@@ -4774,13 +4774,13 @@
         <v>187</v>
       </c>
       <c r="B52" s="5">
-        <v>46122.551548993055</v>
+        <v>46122.38488232639</v>
       </c>
       <c r="C52" s="5">
-        <v>46134.79240423611</v>
+        <v>46134.62573756944</v>
       </c>
       <c r="D52" s="5">
-        <v>46198.18781711806</v>
+        <v>46198.021150451386</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>188</v>
@@ -4839,13 +4839,13 @@
         <v>191</v>
       </c>
       <c r="B53" s="8">
-        <v>46122.55155721065</v>
+        <v>46122.38489054398</v>
       </c>
       <c r="C53" s="8">
-        <v>46134.79245146991</v>
+        <v>46134.62578480324</v>
       </c>
       <c r="D53" s="8">
-        <v>46199.18371805556</v>
+        <v>46199.01705138889</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>82</v>
@@ -4902,13 +4902,13 @@
         <v>193</v>
       </c>
       <c r="B54" s="5">
-        <v>46122.55156568287</v>
+        <v>46122.38489901621</v>
       </c>
       <c r="C54" s="5">
-        <v>46195.50761325231</v>
+        <v>46195.34094658565</v>
       </c>
       <c r="D54" s="5">
-        <v>46196.76907818287</v>
+        <v>46196.6024115162</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>194</v>
@@ -4951,7 +4951,7 @@
         <v>46316</v>
       </c>
       <c r="S54" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T54" s="6">
         <v>1</v>
@@ -4965,13 +4965,13 @@
         <v>198</v>
       </c>
       <c r="B55" s="8">
-        <v>46125.603622118055</v>
+        <v>46125.43695545139</v>
       </c>
       <c r="C55" s="8">
-        <v>46196.76904752315</v>
+        <v>46196.60238085648</v>
       </c>
       <c r="D55" s="8">
-        <v>46196.7690521412</v>
+        <v>46196.602385474536</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>199</v>
@@ -5018,13 +5018,13 @@
         <v>201</v>
       </c>
       <c r="B56" s="5">
-        <v>46125.60367094907</v>
+        <v>46125.43700428241</v>
       </c>
       <c r="C56" s="5">
-        <v>46196.769048449074</v>
+        <v>46196.6023817824</v>
       </c>
       <c r="D56" s="5">
-        <v>46223.607461875</v>
+        <v>46223.440795208335</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>199</v>
@@ -5071,13 +5071,13 @@
         <v>202</v>
       </c>
       <c r="B57" s="8">
-        <v>46125.60371951389</v>
+        <v>46125.43705284722</v>
       </c>
       <c r="C57" s="8">
-        <v>46196.76904929398</v>
+        <v>46196.602382627316</v>
       </c>
       <c r="D57" s="8">
-        <v>46196.76905283565</v>
+        <v>46196.60238616898</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>199</v>
@@ -5124,13 +5124,13 @@
         <v>203</v>
       </c>
       <c r="B58" s="5">
-        <v>46125.60376462963</v>
+        <v>46125.43709796296</v>
       </c>
       <c r="C58" s="5">
-        <v>46196.769050069444</v>
+        <v>46196.60238340277</v>
       </c>
       <c r="D58" s="5">
-        <v>46196.76905314815</v>
+        <v>46196.60238648148</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>199</v>
@@ -5177,13 +5177,13 @@
         <v>204</v>
       </c>
       <c r="B59" s="8">
-        <v>46125.60381739584</v>
+        <v>46125.437150729165</v>
       </c>
       <c r="C59" s="8">
-        <v>46196.76905077546</v>
+        <v>46196.602384108795</v>
       </c>
       <c r="D59" s="8">
-        <v>46196.76905349537</v>
+        <v>46196.6023868287</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>199</v>
@@ -5230,13 +5230,13 @@
         <v>205</v>
       </c>
       <c r="B60" s="5">
-        <v>46122.551569710646</v>
+        <v>46122.38490304398</v>
       </c>
       <c r="C60" s="5">
-        <v>46181.6677724537</v>
+        <v>46181.501105787036</v>
       </c>
       <c r="D60" s="5">
-        <v>46181.66785324074</v>
+        <v>46181.501186574074</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>206</v>
@@ -5279,13 +5279,13 @@
         <v>208</v>
       </c>
       <c r="B61" s="8">
-        <v>46122.55157321759</v>
+        <v>46122.38490655093</v>
       </c>
       <c r="C61" s="8">
-        <v>46181.667378032405</v>
+        <v>46181.50071136574</v>
       </c>
       <c r="D61" s="8">
-        <v>46181.66739524306</v>
+        <v>46181.500728576386</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>209</v>
@@ -5344,13 +5344,13 @@
         <v>213</v>
       </c>
       <c r="B62" s="5">
-        <v>46122.58491638889</v>
+        <v>46122.41824972222</v>
       </c>
       <c r="C62" s="5">
-        <v>46181.667413206014</v>
+        <v>46181.50074653935</v>
       </c>
       <c r="D62" s="5">
-        <v>46181.667429016205</v>
+        <v>46181.50076234953</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>214</v>
@@ -5409,13 +5409,13 @@
         <v>216</v>
       </c>
       <c r="B63" s="8">
-        <v>46125.53102658565</v>
+        <v>46125.36435991898</v>
       </c>
       <c r="C63" s="8">
-        <v>46181.667430127316</v>
+        <v>46181.500763460645</v>
       </c>
       <c r="D63" s="8">
-        <v>46221.202281238424</v>
+        <v>46221.03561457176</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>217</v>
@@ -5474,13 +5474,13 @@
         <v>219</v>
       </c>
       <c r="B64" s="5">
-        <v>46122.55157846065</v>
+        <v>46122.38491179398</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.66775587963</v>
+        <v>46181.501089212965</v>
       </c>
       <c r="D64" s="5">
-        <v>46227.182452106485</v>
+        <v>46227.01578543981</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>215</v>
@@ -5539,13 +5539,13 @@
         <v>224</v>
       </c>
       <c r="B65" s="8">
-        <v>46122.551583831024</v>
+        <v>46122.38491716435</v>
       </c>
       <c r="C65" s="8">
-        <v>46181.6687946875</v>
+        <v>46181.50212802083</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.66890770833</v>
+        <v>46181.50224104167</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>225</v>
@@ -5588,13 +5588,13 @@
         <v>227</v>
       </c>
       <c r="B66" s="5">
-        <v>46122.55158688658</v>
+        <v>46122.384920219905</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.666093576394</v>
+        <v>46181.49942690972</v>
       </c>
       <c r="D66" s="5">
-        <v>46238.1884728125</v>
+        <v>46238.02180614583</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>228</v>
@@ -5653,13 +5653,13 @@
         <v>232</v>
       </c>
       <c r="B67" s="8">
-        <v>46122.55159185185</v>
+        <v>46122.384925185186</v>
       </c>
       <c r="C67" s="8">
-        <v>46181.6661986574</v>
+        <v>46181.49953199074</v>
       </c>
       <c r="D67" s="8">
-        <v>46256.20327105324</v>
+        <v>46256.03660438657</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>233</v>
@@ -5718,13 +5718,13 @@
         <v>235</v>
       </c>
       <c r="B68" s="5">
-        <v>46125.595811921296</v>
+        <v>46125.42914525463</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.66807699074</v>
+        <v>46181.501410324076</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.66807884259</v>
+        <v>46181.50141217593</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>236</v>
@@ -5773,13 +5773,13 @@
         <v>239</v>
       </c>
       <c r="B69" s="8">
-        <v>46125.59610047453</v>
+        <v>46125.42943380787</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.66808581019</v>
+        <v>46181.50141914352</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.66808728009</v>
+        <v>46181.50142061342</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>199</v>
@@ -5828,13 +5828,13 @@
         <v>240</v>
       </c>
       <c r="B70" s="5">
-        <v>46125.59621038195</v>
+        <v>46125.429543715276</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.66815399306</v>
+        <v>46181.501487326386</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.66815550926</v>
+        <v>46181.501488842594</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>199</v>
@@ -5883,13 +5883,13 @@
         <v>241</v>
       </c>
       <c r="B71" s="8">
-        <v>46125.59625472222</v>
+        <v>46125.42958805556</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.668166689815</v>
+        <v>46181.50150002315</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.66816819445</v>
+        <v>46181.501501527775</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>199</v>
@@ -5938,13 +5938,13 @@
         <v>242</v>
       </c>
       <c r="B72" s="5">
-        <v>46125.59629915509</v>
+        <v>46125.42963248843</v>
       </c>
       <c r="C72" s="5">
-        <v>46181.66817956018</v>
+        <v>46181.50151289352</v>
       </c>
       <c r="D72" s="5">
-        <v>46181.66818078703</v>
+        <v>46181.50151412037</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>199</v>
@@ -5993,13 +5993,13 @@
         <v>243</v>
       </c>
       <c r="B73" s="8">
-        <v>46122.55159751157</v>
+        <v>46122.384930844906</v>
       </c>
       <c r="C73" s="8">
-        <v>46181.66878061343</v>
+        <v>46181.50211394676</v>
       </c>
       <c r="D73" s="8">
-        <v>46252.20192400463</v>
+        <v>46252.035257337964</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>244</v>
@@ -6058,13 +6058,13 @@
         <v>245</v>
       </c>
       <c r="B74" s="5">
-        <v>46125.59648849537</v>
+        <v>46125.4298218287</v>
       </c>
       <c r="C74" s="5">
-        <v>46181.668651921296</v>
+        <v>46181.501985254625</v>
       </c>
       <c r="D74" s="5">
-        <v>46181.6686533912</v>
+        <v>46181.501986724536</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>199</v>
@@ -6113,13 +6113,13 @@
         <v>248</v>
       </c>
       <c r="B75" s="8">
-        <v>46125.59661854166</v>
+        <v>46125.429951875005</v>
       </c>
       <c r="C75" s="8">
-        <v>46181.66866650463</v>
+        <v>46181.50199983796</v>
       </c>
       <c r="D75" s="8">
-        <v>46181.66866782407</v>
+        <v>46181.50200115741</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>199</v>
@@ -6168,13 +6168,13 @@
         <v>250</v>
       </c>
       <c r="B76" s="5">
-        <v>46125.596668750004</v>
+        <v>46125.43000208333</v>
       </c>
       <c r="C76" s="5">
-        <v>46181.66867587963</v>
+        <v>46181.50200921296</v>
       </c>
       <c r="D76" s="5">
-        <v>46181.66867745371</v>
+        <v>46181.50201078704</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>199</v>
@@ -6223,13 +6223,13 @@
         <v>251</v>
       </c>
       <c r="B77" s="8">
-        <v>46125.59671550926</v>
+        <v>46125.430048842594</v>
       </c>
       <c r="C77" s="8">
-        <v>46181.668685625</v>
+        <v>46181.50201895833</v>
       </c>
       <c r="D77" s="8">
-        <v>46181.668687060184</v>
+        <v>46181.50202039352</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>199</v>
@@ -6278,13 +6278,13 @@
         <v>253</v>
       </c>
       <c r="B78" s="5">
-        <v>46125.59675546296</v>
+        <v>46125.430088796296</v>
       </c>
       <c r="C78" s="5">
-        <v>46181.66870385417</v>
+        <v>46181.5020371875</v>
       </c>
       <c r="D78" s="5">
-        <v>46181.66870502315</v>
+        <v>46181.502038356484</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>199</v>
@@ -6333,13 +6333,13 @@
         <v>254</v>
       </c>
       <c r="B79" s="8">
-        <v>46122.55160357639</v>
+        <v>46122.38493690972</v>
       </c>
       <c r="C79" s="8">
-        <v>46195.563125636574</v>
+        <v>46195.3964589699</v>
       </c>
       <c r="D79" s="8">
-        <v>46195.563290335645</v>
+        <v>46195.39662366898</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>206</v>
@@ -6386,13 +6386,13 @@
         <v>256</v>
       </c>
       <c r="B80" s="5">
-        <v>46122.55160679398</v>
+        <v>46122.38494012732</v>
       </c>
       <c r="C80" s="5">
-        <v>46195.563269363425</v>
+        <v>46195.39660269676</v>
       </c>
       <c r="D80" s="5">
-        <v>46240.605594189816</v>
+        <v>46240.43892752315</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>257</v>
@@ -6451,13 +6451,13 @@
         <v>259</v>
       </c>
       <c r="B81" s="8">
-        <v>46122.551612256946</v>
+        <v>46122.38494559028</v>
       </c>
       <c r="C81" s="8">
-        <v>46195.50751318287</v>
+        <v>46195.34084651621</v>
       </c>
       <c r="D81" s="8">
-        <v>46195.50753130787</v>
+        <v>46195.3408646412</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>260</v>
@@ -6502,7 +6502,7 @@
         <v>46267</v>
       </c>
       <c r="S81" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T81" s="9">
         <v>1</v>
@@ -6516,13 +6516,13 @@
         <v>261</v>
       </c>
       <c r="B82" s="5">
-        <v>46122.55161756944</v>
+        <v>46122.38495090278</v>
       </c>
       <c r="C82" s="5">
-        <v>46195.50751851852</v>
+        <v>46195.340851851855</v>
       </c>
       <c r="D82" s="5">
-        <v>46195.50753259259</v>
+        <v>46195.34086592593</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>262</v>
@@ -6567,7 +6567,7 @@
         <v>46310</v>
       </c>
       <c r="S82" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T82" s="6">
         <v>1</v>
@@ -6581,13 +6581,13 @@
         <v>263</v>
       </c>
       <c r="B83" s="8">
-        <v>46122.55162288195</v>
+        <v>46122.384956215275</v>
       </c>
       <c r="C83" s="8">
-        <v>46195.507523437496</v>
+        <v>46195.34085677083</v>
       </c>
       <c r="D83" s="8">
-        <v>46195.507539479164</v>
+        <v>46195.3408728125</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>264</v>
@@ -6646,13 +6646,13 @@
         <v>265</v>
       </c>
       <c r="B84" s="5">
-        <v>46122.59399163195</v>
+        <v>46122.427324965276</v>
       </c>
       <c r="C84" s="5">
-        <v>46193.93315311342</v>
+        <v>46193.76648644676</v>
       </c>
       <c r="D84" s="5">
-        <v>46241.18852804398</v>
+        <v>46241.02186137732</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>266</v>
@@ -6711,13 +6711,13 @@
         <v>268</v>
       </c>
       <c r="B85" s="8">
-        <v>46122.551628182875</v>
+        <v>46122.3849615162</v>
       </c>
       <c r="C85" s="8">
-        <v>46195.5630599537</v>
+        <v>46195.39639328704</v>
       </c>
       <c r="D85" s="8">
-        <v>46228.07806180556</v>
+        <v>46227.911395138886</v>
       </c>
       <c r="E85" s="9" t="s">
         <v>269</v>
@@ -6764,13 +6764,13 @@
         <v>271</v>
       </c>
       <c r="B86" s="5">
-        <v>46122.55163158565</v>
+        <v>46122.38496491898</v>
       </c>
       <c r="C86" s="5">
-        <v>46195.50768850694</v>
+        <v>46195.34102184028</v>
       </c>
       <c r="D86" s="5">
-        <v>46223.60779484954</v>
+        <v>46223.441128182865</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>272</v>
@@ -6815,7 +6815,7 @@
         <v>46279</v>
       </c>
       <c r="S86" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T86" s="6">
         <v>1</v>
@@ -6829,13 +6829,13 @@
         <v>274</v>
       </c>
       <c r="B87" s="8">
-        <v>46125.5974969213</v>
+        <v>46125.43083025463</v>
       </c>
       <c r="C87" s="8">
-        <v>46196.76791707176</v>
+        <v>46196.60125040509</v>
       </c>
       <c r="D87" s="8">
-        <v>46223.60698247685</v>
+        <v>46223.440315810185</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>199</v>
@@ -6884,13 +6884,13 @@
         <v>276</v>
       </c>
       <c r="B88" s="5">
-        <v>46125.59754570602</v>
+        <v>46125.430879039355</v>
       </c>
       <c r="C88" s="5">
-        <v>46196.76795405093</v>
+        <v>46196.601287384256</v>
       </c>
       <c r="D88" s="5">
-        <v>46223.60697355324</v>
+        <v>46223.44030688658</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>199</v>
@@ -6939,13 +6939,13 @@
         <v>277</v>
       </c>
       <c r="B89" s="8">
-        <v>46125.59760710648</v>
+        <v>46125.430940439815</v>
       </c>
       <c r="C89" s="8">
-        <v>46196.767928217596</v>
+        <v>46196.601261550924</v>
       </c>
       <c r="D89" s="8">
-        <v>46223.60697</v>
+        <v>46223.44030333334</v>
       </c>
       <c r="E89" s="9" t="s">
         <v>199</v>
@@ -6994,13 +6994,13 @@
         <v>278</v>
       </c>
       <c r="B90" s="5">
-        <v>46125.59765891204</v>
+        <v>46125.43099224537</v>
       </c>
       <c r="C90" s="5">
-        <v>46196.76794651621</v>
+        <v>46196.601279849536</v>
       </c>
       <c r="D90" s="5">
-        <v>46223.60696642361</v>
+        <v>46223.44029975694</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>199</v>
@@ -7049,13 +7049,13 @@
         <v>279</v>
       </c>
       <c r="B91" s="8">
-        <v>46125.597703391206</v>
+        <v>46125.431036724534</v>
       </c>
       <c r="C91" s="8">
-        <v>46196.76794100694</v>
+        <v>46196.60127434028</v>
       </c>
       <c r="D91" s="8">
-        <v>46223.606961412035</v>
+        <v>46223.44029474537</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>199</v>
@@ -7104,13 +7104,13 @@
         <v>280</v>
       </c>
       <c r="B92" s="5">
-        <v>46122.55170659722</v>
+        <v>46122.38503993055</v>
       </c>
       <c r="C92" s="5">
-        <v>46196.76755512731</v>
+        <v>46196.60088846065</v>
       </c>
       <c r="D92" s="5">
-        <v>46237.53492259259</v>
+        <v>46237.368255925925</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>281</v>
@@ -7155,7 +7155,7 @@
         <v>46282</v>
       </c>
       <c r="S92" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T92" s="6">
         <v>1</v>
@@ -7169,13 +7169,13 @@
         <v>282</v>
       </c>
       <c r="B93" s="8">
-        <v>46125.59982741898</v>
+        <v>46125.43316075232</v>
       </c>
       <c r="C93" s="8">
-        <v>46196.76800195602</v>
+        <v>46196.60133528935</v>
       </c>
       <c r="D93" s="8">
-        <v>46223.60708418982</v>
+        <v>46223.44041752315</v>
       </c>
       <c r="E93" s="9" t="s">
         <v>199</v>
@@ -7224,13 +7224,13 @@
         <v>285</v>
       </c>
       <c r="B94" s="5">
-        <v>46125.599890833335</v>
+        <v>46125.43322416667</v>
       </c>
       <c r="C94" s="5">
-        <v>46196.768023020835</v>
+        <v>46196.601356354164</v>
       </c>
       <c r="D94" s="5">
-        <v>46223.60707991898</v>
+        <v>46223.44041325232</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>199</v>
@@ -7279,13 +7279,13 @@
         <v>287</v>
       </c>
       <c r="B95" s="8">
-        <v>46125.59993134259</v>
+        <v>46125.43326467593</v>
       </c>
       <c r="C95" s="8">
-        <v>46196.76801494213</v>
+        <v>46196.601348275464</v>
       </c>
       <c r="D95" s="8">
-        <v>46223.60707583334</v>
+        <v>46223.440409166666</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>199</v>
@@ -7334,13 +7334,13 @@
         <v>288</v>
       </c>
       <c r="B96" s="5">
-        <v>46125.59996929398</v>
+        <v>46125.433302627316</v>
       </c>
       <c r="C96" s="5">
-        <v>46196.76805109954</v>
+        <v>46196.60138443287</v>
       </c>
       <c r="D96" s="5">
-        <v>46223.607072060186</v>
+        <v>46223.440405393514</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>199</v>
@@ -7389,13 +7389,13 @@
         <v>289</v>
       </c>
       <c r="B97" s="8">
-        <v>46125.6000115162</v>
+        <v>46125.43334484954</v>
       </c>
       <c r="C97" s="8">
-        <v>46196.76805706018</v>
+        <v>46196.60139039352</v>
       </c>
       <c r="D97" s="8">
-        <v>46223.607066192126</v>
+        <v>46223.44039952546</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>199</v>
@@ -7444,13 +7444,13 @@
         <v>290</v>
       </c>
       <c r="B98" s="5">
-        <v>46122.55164413195</v>
+        <v>46122.38497746528</v>
       </c>
       <c r="C98" s="5">
-        <v>46196.76839824074</v>
+        <v>46196.601731574076</v>
       </c>
       <c r="D98" s="5">
-        <v>46228.10704425926</v>
+        <v>46227.94037759259</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>291</v>
@@ -7495,7 +7495,7 @@
         <v>46288</v>
       </c>
       <c r="S98" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T98" s="6">
         <v>1</v>
@@ -7509,13 +7509,13 @@
         <v>293</v>
       </c>
       <c r="B99" s="8">
-        <v>46125.599162743056</v>
+        <v>46125.43249607639</v>
       </c>
       <c r="C99" s="8">
-        <v>46196.76818966435</v>
+        <v>46196.601522997684</v>
       </c>
       <c r="D99" s="8">
-        <v>46223.60720636574</v>
+        <v>46223.44053969908</v>
       </c>
       <c r="E99" s="9" t="s">
         <v>199</v>
@@ -7564,13 +7564,13 @@
         <v>296</v>
       </c>
       <c r="B100" s="5">
-        <v>46125.599302511575</v>
+        <v>46125.4326358449</v>
       </c>
       <c r="C100" s="5">
-        <v>46196.76820421296</v>
+        <v>46196.601537546296</v>
       </c>
       <c r="D100" s="5">
-        <v>46223.60720247685</v>
+        <v>46223.44053581019</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>199</v>
@@ -7619,13 +7619,13 @@
         <v>297</v>
       </c>
       <c r="B101" s="8">
-        <v>46125.59934644676</v>
+        <v>46125.43267978009</v>
       </c>
       <c r="C101" s="8">
-        <v>46196.768375949076</v>
+        <v>46196.601709282404</v>
       </c>
       <c r="D101" s="8">
-        <v>46223.60719819444</v>
+        <v>46223.440531527776</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>199</v>
@@ -7674,13 +7674,13 @@
         <v>298</v>
       </c>
       <c r="B102" s="5">
-        <v>46125.59938857639</v>
+        <v>46125.43272190972</v>
       </c>
       <c r="C102" s="5">
-        <v>46196.76837696759</v>
+        <v>46196.60171030092</v>
       </c>
       <c r="D102" s="5">
-        <v>46223.60719417824</v>
+        <v>46223.44052751157</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>199</v>
@@ -7729,13 +7729,13 @@
         <v>299</v>
       </c>
       <c r="B103" s="8">
-        <v>46125.59943094908</v>
+        <v>46125.43276428241</v>
       </c>
       <c r="C103" s="8">
-        <v>46196.76837790509</v>
+        <v>46196.60171123843</v>
       </c>
       <c r="D103" s="8">
-        <v>46223.60718841435</v>
+        <v>46223.44052174769</v>
       </c>
       <c r="E103" s="9" t="s">
         <v>199</v>
@@ -7784,13 +7784,13 @@
         <v>300</v>
       </c>
       <c r="B104" s="5">
-        <v>46122.551650995374</v>
+        <v>46122.3849843287</v>
       </c>
       <c r="C104" s="5">
-        <v>46196.76854788195</v>
+        <v>46196.601881215276</v>
       </c>
       <c r="D104" s="5">
-        <v>46237.53494261574</v>
+        <v>46237.36827594908</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>301</v>
@@ -7835,7 +7835,7 @@
         <v>46293</v>
       </c>
       <c r="S104" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T104" s="6">
         <v>1</v>
@@ -7849,13 +7849,13 @@
         <v>302</v>
       </c>
       <c r="B105" s="8">
-        <v>46125.59953013889</v>
+        <v>46125.43286347222</v>
       </c>
       <c r="C105" s="8">
-        <v>46196.76852783565</v>
+        <v>46196.60186116898</v>
       </c>
       <c r="D105" s="8">
-        <v>46223.60731153935</v>
+        <v>46223.44064487268</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>199</v>
@@ -7904,13 +7904,13 @@
         <v>304</v>
       </c>
       <c r="B106" s="5">
-        <v>46125.59961423611</v>
+        <v>46125.43294756944</v>
       </c>
       <c r="C106" s="5">
-        <v>46196.76846329861</v>
+        <v>46196.60179663195</v>
       </c>
       <c r="D106" s="5">
-        <v>46223.60730783565</v>
+        <v>46223.440641168985</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>199</v>
@@ -7959,13 +7959,13 @@
         <v>305</v>
       </c>
       <c r="B107" s="8">
-        <v>46125.599654317135</v>
+        <v>46125.43298765046</v>
       </c>
       <c r="C107" s="8">
-        <v>46196.768528796296</v>
+        <v>46196.601862129624</v>
       </c>
       <c r="D107" s="8">
-        <v>46223.60730394676</v>
+        <v>46223.44063728009</v>
       </c>
       <c r="E107" s="9" t="s">
         <v>199</v>
@@ -8014,13 +8014,13 @@
         <v>306</v>
       </c>
       <c r="B108" s="5">
-        <v>46125.59957065972</v>
+        <v>46125.43290399306</v>
       </c>
       <c r="C108" s="5">
-        <v>46196.768529548615</v>
+        <v>46196.601862881944</v>
       </c>
       <c r="D108" s="5">
-        <v>46223.607299675925</v>
+        <v>46223.44063300926</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>199</v>
@@ -8069,13 +8069,13 @@
         <v>307</v>
       </c>
       <c r="B109" s="8">
-        <v>46125.59969711806</v>
+        <v>46125.433030451386</v>
       </c>
       <c r="C109" s="8">
-        <v>46196.7685304051</v>
+        <v>46196.601863738426</v>
       </c>
       <c r="D109" s="8">
-        <v>46223.60729373843</v>
+        <v>46223.44062707176</v>
       </c>
       <c r="E109" s="9" t="s">
         <v>199</v>
@@ -8124,13 +8124,13 @@
         <v>308</v>
       </c>
       <c r="B110" s="5">
-        <v>46122.55163725694</v>
+        <v>46122.38497059028</v>
       </c>
       <c r="C110" s="5">
-        <v>46196.76866755787</v>
+        <v>46196.6020008912</v>
       </c>
       <c r="D110" s="5">
-        <v>46223.607779618054</v>
+        <v>46223.44111295139</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>309</v>
@@ -8175,7 +8175,7 @@
         <v>46314</v>
       </c>
       <c r="S110" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T110" s="6">
         <v>1</v>
@@ -8189,13 +8189,13 @@
         <v>310</v>
       </c>
       <c r="B111" s="8">
-        <v>46125.59780210648</v>
+        <v>46125.431135439816</v>
       </c>
       <c r="C111" s="8">
-        <v>46196.76864902778</v>
+        <v>46196.60198236111</v>
       </c>
       <c r="D111" s="8">
-        <v>46223.607408310185</v>
+        <v>46223.44074164351</v>
       </c>
       <c r="E111" s="9" t="s">
         <v>199</v>
@@ -8244,13 +8244,13 @@
         <v>313</v>
       </c>
       <c r="B112" s="5">
-        <v>46125.597836932866</v>
+        <v>46125.43117026621</v>
       </c>
       <c r="C112" s="5">
-        <v>46196.76865</v>
+        <v>46196.601983333334</v>
       </c>
       <c r="D112" s="5">
-        <v>46223.60740443287</v>
+        <v>46223.4407377662</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>199</v>
@@ -8299,13 +8299,13 @@
         <v>314</v>
       </c>
       <c r="B113" s="8">
-        <v>46125.5979208912</v>
+        <v>46125.43125422453</v>
       </c>
       <c r="C113" s="8">
-        <v>46196.76865077546</v>
+        <v>46196.6019841088</v>
       </c>
       <c r="D113" s="8">
-        <v>46223.607400532404</v>
+        <v>46223.44073386574</v>
       </c>
       <c r="E113" s="9" t="s">
         <v>199</v>
@@ -8354,13 +8354,13 @@
         <v>315</v>
       </c>
       <c r="B114" s="5">
-        <v>46125.59788087963</v>
+        <v>46125.431214212964</v>
       </c>
       <c r="C114" s="5">
-        <v>46196.768651527775</v>
+        <v>46196.60198486111</v>
       </c>
       <c r="D114" s="5">
-        <v>46223.60739668981</v>
+        <v>46223.44073002315</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>199</v>
@@ -8409,13 +8409,13 @@
         <v>316</v>
       </c>
       <c r="B115" s="8">
-        <v>46125.597965023146</v>
+        <v>46125.43129835648</v>
       </c>
       <c r="C115" s="8">
-        <v>46196.768652314815</v>
+        <v>46196.60198564814</v>
       </c>
       <c r="D115" s="8">
-        <v>46223.60739046296</v>
+        <v>46223.440723796295</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>199</v>
@@ -8464,13 +8464,13 @@
         <v>317</v>
       </c>
       <c r="B116" s="5">
-        <v>46122.55172043982</v>
+        <v>46122.38505377315</v>
       </c>
       <c r="C116" s="5">
-        <v>46196.76877224537</v>
+        <v>46196.6021055787</v>
       </c>
       <c r="D116" s="5">
-        <v>46237.53496467593</v>
+        <v>46237.368298009256</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>318</v>
@@ -8515,7 +8515,7 @@
         <v>46315</v>
       </c>
       <c r="S116" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T116" s="6">
         <v>1</v>
@@ -8529,13 +8529,13 @@
         <v>319</v>
       </c>
       <c r="B117" s="8">
-        <v>46125.60038253472</v>
+        <v>46125.43371586806</v>
       </c>
       <c r="C117" s="8">
-        <v>46196.76875258102</v>
+        <v>46196.602085914354</v>
       </c>
       <c r="D117" s="8">
-        <v>46223.60758443287</v>
+        <v>46223.4409177662</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>199</v>
@@ -8582,13 +8582,13 @@
         <v>321</v>
       </c>
       <c r="B118" s="5">
-        <v>46125.60043012731</v>
+        <v>46125.43376346065</v>
       </c>
       <c r="C118" s="5">
-        <v>46223.60745270833</v>
+        <v>46223.44078604167</v>
       </c>
       <c r="D118" s="5">
-        <v>46223.60758005787</v>
+        <v>46223.440913391205</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>199</v>
@@ -8635,13 +8635,13 @@
         <v>322</v>
       </c>
       <c r="B119" s="8">
-        <v>46125.60047290509</v>
+        <v>46125.43380623843</v>
       </c>
       <c r="C119" s="8">
-        <v>46196.768754178236</v>
+        <v>46196.60208751158</v>
       </c>
       <c r="D119" s="8">
-        <v>46223.607575752314</v>
+        <v>46223.44090908565</v>
       </c>
       <c r="E119" s="9" t="s">
         <v>199</v>
@@ -8688,13 +8688,13 @@
         <v>323</v>
       </c>
       <c r="B120" s="5">
-        <v>46125.600514074074</v>
+        <v>46125.4338474074</v>
       </c>
       <c r="C120" s="5">
-        <v>46196.768754930556</v>
+        <v>46196.602088263884</v>
       </c>
       <c r="D120" s="5">
-        <v>46223.607571597226</v>
+        <v>46223.440904930554</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>199</v>
@@ -8741,13 +8741,13 @@
         <v>324</v>
       </c>
       <c r="B121" s="8">
-        <v>46125.60055859954</v>
+        <v>46125.43389193287</v>
       </c>
       <c r="C121" s="8">
-        <v>46196.7687558912</v>
+        <v>46196.602089224536</v>
       </c>
       <c r="D121" s="8">
-        <v>46223.60756553241</v>
+        <v>46223.44089886574</v>
       </c>
       <c r="E121" s="9" t="s">
         <v>199</v>
@@ -8794,13 +8794,13 @@
         <v>325</v>
       </c>
       <c r="B122" s="5">
-        <v>46122.55172986111</v>
+        <v>46122.385063194444</v>
       </c>
       <c r="C122" s="5">
-        <v>46196.76917457176</v>
+        <v>46196.60250790509</v>
       </c>
       <c r="D122" s="5">
-        <v>46223.60776988426</v>
+        <v>46223.44110321759</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>326</v>
@@ -8845,7 +8845,7 @@
         <v>46317</v>
       </c>
       <c r="S122" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T122" s="6">
         <v>1</v>
@@ -8859,13 +8859,13 @@
         <v>328</v>
       </c>
       <c r="B123" s="8">
-        <v>46125.60064416667</v>
+        <v>46125.4339775</v>
       </c>
       <c r="C123" s="8">
-        <v>46196.76915099537</v>
+        <v>46196.6024843287</v>
       </c>
       <c r="D123" s="8">
-        <v>46223.607680601854</v>
+        <v>46223.44101393518</v>
       </c>
       <c r="E123" s="9" t="s">
         <v>199</v>
@@ -8912,13 +8912,13 @@
         <v>330</v>
       </c>
       <c r="B124" s="5">
-        <v>46125.60068740741</v>
+        <v>46125.43402074074</v>
       </c>
       <c r="C124" s="5">
-        <v>46196.76915237268</v>
+        <v>46196.60248570602</v>
       </c>
       <c r="D124" s="5">
-        <v>46223.60767706019</v>
+        <v>46223.44101039352</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>199</v>
@@ -8965,13 +8965,13 @@
         <v>331</v>
       </c>
       <c r="B125" s="8">
-        <v>46125.60073844907</v>
+        <v>46125.43407178241</v>
       </c>
       <c r="C125" s="8">
-        <v>46196.76915341435</v>
+        <v>46196.60248674768</v>
       </c>
       <c r="D125" s="8">
-        <v>46223.607672812504</v>
+        <v>46223.44100614583</v>
       </c>
       <c r="E125" s="9" t="s">
         <v>199</v>
@@ -9018,13 +9018,13 @@
         <v>332</v>
       </c>
       <c r="B126" s="5">
-        <v>46125.60077622686</v>
+        <v>46125.434109560185</v>
       </c>
       <c r="C126" s="5">
-        <v>46196.76915438657</v>
+        <v>46196.60248771991</v>
       </c>
       <c r="D126" s="5">
-        <v>46223.6076684375</v>
+        <v>46223.44100177083</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>199</v>
@@ -9071,13 +9071,13 @@
         <v>333</v>
       </c>
       <c r="B127" s="8">
-        <v>46125.600829143514</v>
+        <v>46125.43416247686</v>
       </c>
       <c r="C127" s="8">
-        <v>46196.769155358794</v>
+        <v>46196.60248869213</v>
       </c>
       <c r="D127" s="8">
-        <v>46223.60766289352</v>
+        <v>46223.440996226855</v>
       </c>
       <c r="E127" s="9" t="s">
         <v>199</v>
@@ -9124,13 +9124,13 @@
         <v>334</v>
       </c>
       <c r="B128" s="5">
-        <v>46122.5517350463</v>
+        <v>46122.38506837963</v>
       </c>
       <c r="C128" s="5">
-        <v>46195.56317517361</v>
+        <v>46195.39650850694</v>
       </c>
       <c r="D128" s="5">
-        <v>46196.76960409722</v>
+        <v>46196.60293743055</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>335</v>
@@ -9177,13 +9177,13 @@
         <v>337</v>
       </c>
       <c r="B129" s="8">
-        <v>46122.5517390625</v>
+        <v>46122.38507239583</v>
       </c>
       <c r="C129" s="8">
-        <v>46196.76936652778</v>
+        <v>46196.60269986111</v>
       </c>
       <c r="D129" s="8">
-        <v>46240.60562268519</v>
+        <v>46240.43895601852</v>
       </c>
       <c r="E129" s="9" t="s">
         <v>338</v>
@@ -9228,7 +9228,7 @@
         <v>46318</v>
       </c>
       <c r="S129" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T129" s="9">
         <v>1</v>
@@ -9242,13 +9242,13 @@
         <v>342</v>
       </c>
       <c r="B130" s="5">
-        <v>46125.60093731481</v>
+        <v>46125.43427064815</v>
       </c>
       <c r="C130" s="5">
-        <v>46196.76934515046</v>
+        <v>46196.602678483796</v>
       </c>
       <c r="D130" s="5">
-        <v>46196.769350682865</v>
+        <v>46196.60268401621</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>199</v>
@@ -9295,13 +9295,13 @@
         <v>344</v>
       </c>
       <c r="B131" s="8">
-        <v>46125.601380821754</v>
+        <v>46125.4347141551</v>
       </c>
       <c r="C131" s="8">
-        <v>46196.769346307876</v>
+        <v>46196.602679641204</v>
       </c>
       <c r="D131" s="8">
-        <v>46196.769351145835</v>
+        <v>46196.60268447916</v>
       </c>
       <c r="E131" s="9" t="s">
         <v>199</v>
@@ -9348,13 +9348,13 @@
         <v>345</v>
       </c>
       <c r="B132" s="5">
-        <v>46125.60142481481</v>
+        <v>46125.43475814815</v>
       </c>
       <c r="C132" s="5">
-        <v>46196.7693472338</v>
+        <v>46196.60268056713</v>
       </c>
       <c r="D132" s="5">
-        <v>46196.76935155093</v>
+        <v>46196.60268488426</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>199</v>
@@ -9401,13 +9401,13 @@
         <v>346</v>
       </c>
       <c r="B133" s="8">
-        <v>46125.60146085648</v>
+        <v>46125.434794189816</v>
       </c>
       <c r="C133" s="8">
-        <v>46196.769348125</v>
+        <v>46196.60268145833</v>
       </c>
       <c r="D133" s="8">
-        <v>46196.76935192129</v>
+        <v>46196.602685254635</v>
       </c>
       <c r="E133" s="9" t="s">
         <v>199</v>
@@ -9454,13 +9454,13 @@
         <v>347</v>
       </c>
       <c r="B134" s="5">
-        <v>46125.60150208333</v>
+        <v>46125.434835416665</v>
       </c>
       <c r="C134" s="5">
-        <v>46196.769348981485</v>
+        <v>46196.60268231481</v>
       </c>
       <c r="D134" s="5">
-        <v>46196.76935229167</v>
+        <v>46196.602685624996</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>199</v>
@@ -9507,13 +9507,13 @@
         <v>348</v>
       </c>
       <c r="B135" s="8">
-        <v>46122.55174383102</v>
+        <v>46122.38507716435</v>
       </c>
       <c r="C135" s="8">
-        <v>46196.769596921295</v>
+        <v>46196.60293025463</v>
       </c>
       <c r="D135" s="8">
-        <v>46228.10760070602</v>
+        <v>46227.94093403935</v>
       </c>
       <c r="E135" s="9" t="s">
         <v>349</v>
@@ -9556,7 +9556,7 @@
         <v>46321</v>
       </c>
       <c r="S135" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T135" s="9">
         <v>1</v>
@@ -9570,13 +9570,13 @@
         <v>350</v>
       </c>
       <c r="B136" s="5">
-        <v>46125.601086979164</v>
+        <v>46125.4344203125</v>
       </c>
       <c r="C136" s="5">
-        <v>46196.76947155093</v>
+        <v>46196.602804884256</v>
       </c>
       <c r="D136" s="5">
-        <v>46223.60837070602</v>
+        <v>46223.44170403935</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>199</v>
@@ -9623,13 +9623,13 @@
         <v>352</v>
       </c>
       <c r="B137" s="8">
-        <v>46125.60115318287</v>
+        <v>46125.4344865162</v>
       </c>
       <c r="C137" s="8">
-        <v>46196.7695043287</v>
+        <v>46196.60283766204</v>
       </c>
       <c r="D137" s="8">
-        <v>46223.60836653935</v>
+        <v>46223.44169987268</v>
       </c>
       <c r="E137" s="9" t="s">
         <v>199</v>
@@ -9676,13 +9676,13 @@
         <v>353</v>
       </c>
       <c r="B138" s="5">
-        <v>46125.60120391204</v>
+        <v>46125.43453724537</v>
       </c>
       <c r="C138" s="5">
-        <v>46196.76950549769</v>
+        <v>46196.60283883102</v>
       </c>
       <c r="D138" s="5">
-        <v>46223.608362604165</v>
+        <v>46223.4416959375</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>199</v>
@@ -9729,13 +9729,13 @@
         <v>354</v>
       </c>
       <c r="B139" s="8">
-        <v>46125.60125796296</v>
+        <v>46125.434591296296</v>
       </c>
       <c r="C139" s="8">
-        <v>46196.76950637731</v>
+        <v>46196.60283971065</v>
       </c>
       <c r="D139" s="8">
-        <v>46223.60835905092</v>
+        <v>46223.44169238426</v>
       </c>
       <c r="E139" s="9" t="s">
         <v>199</v>
@@ -9782,13 +9782,13 @@
         <v>355</v>
       </c>
       <c r="B140" s="5">
-        <v>46125.601304282405</v>
+        <v>46125.43463761574</v>
       </c>
       <c r="C140" s="5">
-        <v>46196.76950730324</v>
+        <v>46196.60284063657</v>
       </c>
       <c r="D140" s="5">
-        <v>46223.60835267361</v>
+        <v>46223.44168600695</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>199</v>
@@ -9835,13 +9835,13 @@
         <v>356</v>
       </c>
       <c r="B141" s="8">
-        <v>46122.55174869213</v>
+        <v>46122.38508202546</v>
       </c>
       <c r="C141" s="8">
-        <v>46191.70598530093</v>
+        <v>46191.539318634255</v>
       </c>
       <c r="D141" s="8">
-        <v>46240.605638368055</v>
+        <v>46240.438971701384</v>
       </c>
       <c r="E141" s="9" t="s">
         <v>357</v>
@@ -9884,7 +9884,7 @@
         <v>46322</v>
       </c>
       <c r="S141" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T141" s="9">
         <v>1</v>
@@ -9898,13 +9898,13 @@
         <v>358</v>
       </c>
       <c r="B142" s="5">
-        <v>46125.60158650463</v>
+        <v>46125.434919837964</v>
       </c>
       <c r="C142" s="5">
-        <v>46196.76968462963</v>
+        <v>46196.60301796296</v>
       </c>
       <c r="D142" s="5">
-        <v>46196.76968989584</v>
+        <v>46196.60302322917</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>199</v>
@@ -9951,13 +9951,13 @@
         <v>360</v>
       </c>
       <c r="B143" s="8">
-        <v>46125.60163133102</v>
+        <v>46125.43496466435</v>
       </c>
       <c r="C143" s="8">
-        <v>46196.76968585648</v>
+        <v>46196.60301918982</v>
       </c>
       <c r="D143" s="8">
-        <v>46196.7696903125</v>
+        <v>46196.60302364583</v>
       </c>
       <c r="E143" s="9" t="s">
         <v>199</v>
@@ -10004,13 +10004,13 @@
         <v>361</v>
       </c>
       <c r="B144" s="5">
-        <v>46125.60167016204</v>
+        <v>46125.43500349537</v>
       </c>
       <c r="C144" s="5">
-        <v>46196.7696866551</v>
+        <v>46196.603019988426</v>
       </c>
       <c r="D144" s="5">
-        <v>46196.769690706016</v>
+        <v>46196.60302403935</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>199</v>
@@ -10057,13 +10057,13 @@
         <v>363</v>
       </c>
       <c r="B145" s="8">
-        <v>46125.60170435185</v>
+        <v>46125.43503768518</v>
       </c>
       <c r="C145" s="8">
-        <v>46196.769687395834</v>
+        <v>46196.60302072916</v>
       </c>
       <c r="D145" s="8">
-        <v>46196.76969114583</v>
+        <v>46196.60302447916</v>
       </c>
       <c r="E145" s="9" t="s">
         <v>199</v>
@@ -10110,13 +10110,13 @@
         <v>364</v>
       </c>
       <c r="B146" s="5">
-        <v>46125.60173947917</v>
+        <v>46125.4350728125</v>
       </c>
       <c r="C146" s="5">
-        <v>46196.769688113425</v>
+        <v>46196.60302144676</v>
       </c>
       <c r="D146" s="5">
-        <v>46196.76969164352</v>
+        <v>46196.60302497685</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>199</v>
@@ -10163,13 +10163,13 @@
         <v>365</v>
       </c>
       <c r="B147" s="8">
-        <v>46122.551753472224</v>
+        <v>46122.38508680556</v>
       </c>
       <c r="C147" s="8">
-        <v>46191.70604009259</v>
+        <v>46191.53937342593</v>
       </c>
       <c r="D147" s="8">
-        <v>46240.60565322917</v>
+        <v>46240.4389865625</v>
       </c>
       <c r="E147" s="9" t="s">
         <v>366</v>
@@ -10212,7 +10212,7 @@
         <v>46323</v>
       </c>
       <c r="S147" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T147" s="9">
         <v>1</v>
@@ -10226,13 +10226,13 @@
         <v>368</v>
       </c>
       <c r="B148" s="5">
-        <v>46125.60181555555</v>
+        <v>46125.43514888889</v>
       </c>
       <c r="C148" s="5">
-        <v>46196.76979265046</v>
+        <v>46196.60312598379</v>
       </c>
       <c r="D148" s="5">
-        <v>46196.76979569445</v>
+        <v>46196.603129027775</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>199</v>
@@ -10279,13 +10279,13 @@
         <v>369</v>
       </c>
       <c r="B149" s="8">
-        <v>46125.60185690972</v>
+        <v>46125.43519024306</v>
       </c>
       <c r="C149" s="8">
-        <v>46196.76979356482</v>
+        <v>46196.603126898146</v>
       </c>
       <c r="D149" s="8">
-        <v>46196.76979614583</v>
+        <v>46196.60312947917</v>
       </c>
       <c r="E149" s="9" t="s">
         <v>199</v>
@@ -10332,13 +10332,13 @@
         <v>370</v>
       </c>
       <c r="B150" s="5">
-        <v>46125.601899490735</v>
+        <v>46125.43523282408</v>
       </c>
       <c r="C150" s="5">
-        <v>46196.769794224536</v>
+        <v>46196.60312755787</v>
       </c>
       <c r="D150" s="5">
-        <v>46196.76979648148</v>
+        <v>46196.603129814815</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>199</v>
@@ -10385,13 +10385,13 @@
         <v>371</v>
       </c>
       <c r="B151" s="8">
-        <v>46125.60193935185</v>
+        <v>46125.43527268519</v>
       </c>
       <c r="C151" s="8">
-        <v>46196.76976476852</v>
+        <v>46196.603098101856</v>
       </c>
       <c r="D151" s="8">
-        <v>46196.769766875004</v>
+        <v>46196.60310020833</v>
       </c>
       <c r="E151" s="9" t="s">
         <v>199</v>
@@ -10438,13 +10438,13 @@
         <v>372</v>
       </c>
       <c r="B152" s="5">
-        <v>46125.60197710648</v>
+        <v>46125.43531043982</v>
       </c>
       <c r="C152" s="5">
-        <v>46196.76977206019</v>
+        <v>46196.603105393515</v>
       </c>
       <c r="D152" s="5">
-        <v>46196.76977370371</v>
+        <v>46196.60310703704</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>199</v>
@@ -10491,13 +10491,13 @@
         <v>373</v>
       </c>
       <c r="B153" s="8">
-        <v>46122.551758622685</v>
+        <v>46122.38509195602</v>
       </c>
       <c r="C153" s="8">
-        <v>46240.65384241898</v>
+        <v>46240.487175752314</v>
       </c>
       <c r="D153" s="8">
-        <v>46240.65385445602</v>
+        <v>46240.48718778935</v>
       </c>
       <c r="E153" s="9" t="s">
         <v>374</v>
@@ -10544,13 +10544,13 @@
         <v>376</v>
       </c>
       <c r="B154" s="5">
-        <v>46122.55176134259</v>
+        <v>46122.38509467593</v>
       </c>
       <c r="C154" s="5">
-        <v>46240.65381834491</v>
+        <v>46240.487151678244</v>
       </c>
       <c r="D154" s="5">
-        <v>46240.65383614584</v>
+        <v>46240.487169479165</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>377</v>
@@ -10595,7 +10595,7 @@
         <v>46332</v>
       </c>
       <c r="S154" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T154" s="6">
         <v>1</v>
@@ -10609,13 +10609,13 @@
         <v>380</v>
       </c>
       <c r="B155" s="8">
-        <v>46122.55176609954</v>
+        <v>46122.38509943287</v>
       </c>
       <c r="C155" s="8">
-        <v>46240.65382724537</v>
+        <v>46240.487160578705</v>
       </c>
       <c r="D155" s="8">
-        <v>46240.65384380787</v>
+        <v>46240.4871771412</v>
       </c>
       <c r="E155" s="9" t="s">
         <v>381</v>
@@ -10660,7 +10660,7 @@
         <v>46332</v>
       </c>
       <c r="S155" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T155" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-24 20:45 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -1844,13 +1844,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46122.38452245371</v>
+        <v>46122.55118912037</v>
       </c>
       <c r="C4" s="5">
-        <v>46128.426341053244</v>
+        <v>46128.59300771991</v>
       </c>
       <c r="D4" s="5">
-        <v>46157.93633454861</v>
+        <v>46158.10300121528</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1893,13 +1893,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46122.38467905093</v>
+        <v>46122.55134571759</v>
       </c>
       <c r="C5" s="8">
-        <v>46128.42632796297</v>
+        <v>46128.59299462963</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.70935505787</v>
+        <v>46133.876021724536</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1956,13 +1956,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46122.384682812495</v>
+        <v>46122.55134947917</v>
       </c>
       <c r="C6" s="5">
-        <v>46128.42601201389</v>
+        <v>46128.59267868055</v>
       </c>
       <c r="D6" s="5">
-        <v>46128.43715965278</v>
+        <v>46128.60382631945</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -2019,13 +2019,13 @@
         <v>37</v>
       </c>
       <c r="B7" s="8">
-        <v>46122.38468587963</v>
+        <v>46122.551352546296</v>
       </c>
       <c r="C7" s="8">
-        <v>46128.42603200232</v>
+        <v>46128.59269866898</v>
       </c>
       <c r="D7" s="8">
-        <v>46161.460593807875</v>
+        <v>46161.62726047453</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>38</v>
@@ -2082,13 +2082,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46122.38468890046</v>
+        <v>46122.551355567135</v>
       </c>
       <c r="C8" s="5">
-        <v>46128.42605055556</v>
+        <v>46128.59271722222</v>
       </c>
       <c r="D8" s="5">
-        <v>46128.43733940972</v>
+        <v>46128.60400607639</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -2145,13 +2145,13 @@
         <v>44</v>
       </c>
       <c r="B9" s="8">
-        <v>46122.384692719905</v>
+        <v>46122.551359386576</v>
       </c>
       <c r="C9" s="8">
-        <v>46128.4261833912</v>
+        <v>46128.592850057874</v>
       </c>
       <c r="D9" s="8">
-        <v>46156.66910643518</v>
+        <v>46156.83577310185</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>45</v>
@@ -2208,13 +2208,13 @@
         <v>47</v>
       </c>
       <c r="B10" s="5">
-        <v>46122.3845274537</v>
+        <v>46122.55119412037</v>
       </c>
       <c r="C10" s="5">
-        <v>46193.766136805556</v>
+        <v>46193.93280347223</v>
       </c>
       <c r="D10" s="5">
-        <v>46223.25695451389</v>
+        <v>46223.423621180555</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>48</v>
@@ -2261,13 +2261,13 @@
         <v>50</v>
       </c>
       <c r="B11" s="8">
-        <v>46122.384696504625</v>
+        <v>46122.5513631713</v>
       </c>
       <c r="C11" s="8">
-        <v>46128.43768854167</v>
+        <v>46128.60435520833</v>
       </c>
       <c r="D11" s="8">
-        <v>46192.80716136574</v>
+        <v>46192.97382803241</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>51</v>
@@ -2326,13 +2326,13 @@
         <v>54</v>
       </c>
       <c r="B12" s="5">
-        <v>46122.38470238426</v>
+        <v>46122.551369050925</v>
       </c>
       <c r="C12" s="5">
-        <v>46128.43976447917</v>
+        <v>46128.60643114583</v>
       </c>
       <c r="D12" s="5">
-        <v>46192.80716146991</v>
+        <v>46192.97382813657</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>55</v>
@@ -2391,13 +2391,13 @@
         <v>58</v>
       </c>
       <c r="B13" s="8">
-        <v>46122.384708020836</v>
+        <v>46122.5513746875</v>
       </c>
       <c r="C13" s="8">
-        <v>46132.40405894676</v>
+        <v>46132.57072561343</v>
       </c>
       <c r="D13" s="8">
-        <v>46192.80716134259</v>
+        <v>46192.97382800926</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>59</v>
@@ -2456,13 +2456,13 @@
         <v>61</v>
       </c>
       <c r="B14" s="5">
-        <v>46122.38692751157</v>
+        <v>46122.553594178244</v>
       </c>
       <c r="C14" s="5">
-        <v>46128.44274908565</v>
+        <v>46128.60941575232</v>
       </c>
       <c r="D14" s="5">
-        <v>46136.03935251157</v>
+        <v>46136.20601917824</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>62</v>
@@ -2521,13 +2521,13 @@
         <v>65</v>
       </c>
       <c r="B15" s="8">
-        <v>46122.38453280093</v>
+        <v>46122.55119946759</v>
       </c>
       <c r="C15" s="8">
-        <v>46195.34056496528</v>
+        <v>46195.50723163194</v>
       </c>
       <c r="D15" s="8">
-        <v>46227.938021354166</v>
+        <v>46228.10468802083</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>66</v>
@@ -2574,13 +2574,13 @@
         <v>68</v>
       </c>
       <c r="B16" s="5">
-        <v>46122.38472188657</v>
+        <v>46122.55138855324</v>
       </c>
       <c r="C16" s="5">
-        <v>46128.44033724537</v>
+        <v>46128.60700391204</v>
       </c>
       <c r="D16" s="5">
-        <v>46133.0133283912</v>
+        <v>46133.17999505787</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>69</v>
@@ -2639,13 +2639,13 @@
         <v>71</v>
       </c>
       <c r="B17" s="8">
-        <v>46122.38472815973</v>
+        <v>46122.55139482639</v>
       </c>
       <c r="C17" s="8">
-        <v>46128.44034490741</v>
+        <v>46128.60701157407</v>
       </c>
       <c r="D17" s="8">
-        <v>46132.01554025463</v>
+        <v>46132.182206921294</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>72</v>
@@ -2704,13 +2704,13 @@
         <v>75</v>
       </c>
       <c r="B18" s="5">
-        <v>46122.38473373842</v>
+        <v>46122.55140040509</v>
       </c>
       <c r="C18" s="5">
-        <v>46195.340545046296</v>
+        <v>46195.50721171296</v>
       </c>
       <c r="D18" s="5">
-        <v>46223.43988759259</v>
+        <v>46223.606554259255</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>76</v>
@@ -2769,13 +2769,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46122.384739375004</v>
+        <v>46122.55140604167</v>
       </c>
       <c r="C19" s="8">
-        <v>46181.499732384254</v>
+        <v>46181.666399050926</v>
       </c>
       <c r="D19" s="8">
-        <v>46223.43988416667</v>
+        <v>46223.606550833334</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2834,13 +2834,13 @@
         <v>84</v>
       </c>
       <c r="B20" s="5">
-        <v>46122.3847449537</v>
+        <v>46122.55141162037</v>
       </c>
       <c r="C20" s="5">
-        <v>46128.442831215274</v>
+        <v>46128.609497881946</v>
       </c>
       <c r="D20" s="5">
-        <v>46132.01553989583</v>
+        <v>46132.1822065625</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>64</v>
@@ -2899,13 +2899,13 @@
         <v>87</v>
       </c>
       <c r="B21" s="8">
-        <v>46122.39987912037</v>
+        <v>46122.566545787035</v>
       </c>
       <c r="C21" s="8">
-        <v>46181.49969386574</v>
+        <v>46181.66636053241</v>
       </c>
       <c r="D21" s="8">
-        <v>46223.43988042824</v>
+        <v>46223.60654709491</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>88</v>
@@ -2964,13 +2964,13 @@
         <v>90</v>
       </c>
       <c r="B22" s="5">
-        <v>46122.39994855324</v>
+        <v>46122.56661521991</v>
       </c>
       <c r="C22" s="5">
-        <v>46181.499709641204</v>
+        <v>46181.66637630787</v>
       </c>
       <c r="D22" s="5">
-        <v>46223.4398771875</v>
+        <v>46223.60654385417</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>91</v>
@@ -3029,13 +3029,13 @@
         <v>93</v>
       </c>
       <c r="B23" s="8">
-        <v>46122.40619606481</v>
+        <v>46122.57286273148</v>
       </c>
       <c r="C23" s="8">
-        <v>46181.4997655787</v>
+        <v>46181.66643224537</v>
       </c>
       <c r="D23" s="8">
-        <v>46223.43987166666</v>
+        <v>46223.60653833333</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>94</v>
@@ -3094,13 +3094,13 @@
         <v>96</v>
       </c>
       <c r="B24" s="5">
-        <v>46122.38453728009</v>
+        <v>46122.55120394676</v>
       </c>
       <c r="C24" s="5">
-        <v>46195.34067315972</v>
+        <v>46195.50733982639</v>
       </c>
       <c r="D24" s="5">
-        <v>46223.25843659722</v>
+        <v>46223.425103263886</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>97</v>
@@ -3147,13 +3147,13 @@
         <v>99</v>
       </c>
       <c r="B25" s="8">
-        <v>46122.38475027778</v>
+        <v>46122.55141694444</v>
       </c>
       <c r="C25" s="8">
-        <v>46174.45950203703</v>
+        <v>46174.626168703704</v>
       </c>
       <c r="D25" s="8">
-        <v>46258.02963747685</v>
+        <v>46258.19630414352</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>100</v>
@@ -3212,13 +3212,13 @@
         <v>104</v>
       </c>
       <c r="B26" s="5">
-        <v>46122.38475541667</v>
+        <v>46122.55142208333</v>
       </c>
       <c r="C26" s="5">
-        <v>46174.45658625</v>
+        <v>46174.62325291667</v>
       </c>
       <c r="D26" s="5">
-        <v>46174.456587824076</v>
+        <v>46174.62325449074</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>105</v>
@@ -3273,13 +3273,13 @@
         <v>109</v>
       </c>
       <c r="B27" s="8">
-        <v>46122.38476032407</v>
+        <v>46122.55142699074</v>
       </c>
       <c r="C27" s="8">
-        <v>46174.45948622686</v>
+        <v>46174.626152893514</v>
       </c>
       <c r="D27" s="8">
-        <v>46174.45948762732</v>
+        <v>46174.62615429398</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>110</v>
@@ -3334,13 +3334,13 @@
         <v>112</v>
       </c>
       <c r="B28" s="5">
-        <v>46122.38476556713</v>
+        <v>46122.5514322338</v>
       </c>
       <c r="C28" s="5">
-        <v>46195.340658553236</v>
+        <v>46195.50732521991</v>
       </c>
       <c r="D28" s="5">
-        <v>46195.545180127316</v>
+        <v>46195.71184679398</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>113</v>
@@ -3399,13 +3399,13 @@
         <v>116</v>
       </c>
       <c r="B29" s="8">
-        <v>46122.38477087963</v>
+        <v>46122.551437546295</v>
       </c>
       <c r="C29" s="8">
-        <v>46195.54471607639</v>
+        <v>46195.71138274306</v>
       </c>
       <c r="D29" s="8">
-        <v>46195.54471850695</v>
+        <v>46195.71138517361</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>117</v>
@@ -3460,13 +3460,13 @@
         <v>119</v>
       </c>
       <c r="B30" s="5">
-        <v>46122.3847758912</v>
+        <v>46122.55144255787</v>
       </c>
       <c r="C30" s="5">
-        <v>46195.54516429398</v>
+        <v>46195.711830960645</v>
       </c>
       <c r="D30" s="5">
-        <v>46195.54516583333</v>
+        <v>46195.711832500005</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>120</v>
@@ -3521,13 +3521,13 @@
         <v>122</v>
       </c>
       <c r="B31" s="8">
-        <v>46122.38478104166</v>
+        <v>46122.551447708334</v>
       </c>
       <c r="C31" s="8">
-        <v>46133.661133263886</v>
+        <v>46133.82779993056</v>
       </c>
       <c r="D31" s="8">
-        <v>46133.66114655093</v>
+        <v>46133.82781321759</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>123</v>
@@ -3586,13 +3586,13 @@
         <v>125</v>
       </c>
       <c r="B32" s="5">
-        <v>46122.38478609954</v>
+        <v>46122.5514527662</v>
       </c>
       <c r="C32" s="5">
-        <v>46133.66106445601</v>
+        <v>46133.827731122685</v>
       </c>
       <c r="D32" s="5">
-        <v>46133.6610659375</v>
+        <v>46133.82773260417</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>126</v>
@@ -3647,13 +3647,13 @@
         <v>128</v>
       </c>
       <c r="B33" s="8">
-        <v>46122.384791296296</v>
+        <v>46122.55145796297</v>
       </c>
       <c r="C33" s="8">
-        <v>46133.66112020833</v>
+        <v>46133.827786875</v>
       </c>
       <c r="D33" s="8">
-        <v>46133.661121412035</v>
+        <v>46133.82778807871</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>129</v>
@@ -3708,13 +3708,13 @@
         <v>131</v>
       </c>
       <c r="B34" s="5">
-        <v>46122.38479633102</v>
+        <v>46122.55146299768</v>
       </c>
       <c r="C34" s="5">
-        <v>46133.6611012963</v>
+        <v>46133.82776796297</v>
       </c>
       <c r="D34" s="5">
-        <v>46133.66110246528</v>
+        <v>46133.827769131945</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>132</v>
@@ -3769,13 +3769,13 @@
         <v>134</v>
       </c>
       <c r="B35" s="8">
-        <v>46122.38480128472</v>
+        <v>46122.55146795139</v>
       </c>
       <c r="C35" s="8">
-        <v>46181.50020540509</v>
+        <v>46181.66687207176</v>
       </c>
       <c r="D35" s="8">
-        <v>46214.01094108797</v>
+        <v>46214.17760775463</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>135</v>
@@ -3834,13 +3834,13 @@
         <v>139</v>
       </c>
       <c r="B36" s="5">
-        <v>46122.38480630787</v>
+        <v>46122.551472974534</v>
       </c>
       <c r="C36" s="5">
-        <v>46181.50015100694</v>
+        <v>46181.66681767361</v>
       </c>
       <c r="D36" s="5">
-        <v>46181.50015280093</v>
+        <v>46181.66681946759</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>140</v>
@@ -3895,13 +3895,13 @@
         <v>142</v>
       </c>
       <c r="B37" s="8">
-        <v>46122.384855868055</v>
+        <v>46122.55152253472</v>
       </c>
       <c r="C37" s="8">
-        <v>46181.50019012731</v>
+        <v>46181.66685679398</v>
       </c>
       <c r="D37" s="8">
-        <v>46181.5001915162</v>
+        <v>46181.66685818287</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>143</v>
@@ -3956,13 +3956,13 @@
         <v>145</v>
       </c>
       <c r="B38" s="5">
-        <v>46122.384862245366</v>
+        <v>46122.55152891204</v>
       </c>
       <c r="C38" s="5">
-        <v>46154.70100114583</v>
+        <v>46154.867667812505</v>
       </c>
       <c r="D38" s="5">
-        <v>46189.00554646991</v>
+        <v>46189.172213136575</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>146</v>
@@ -4021,13 +4021,13 @@
         <v>148</v>
       </c>
       <c r="B39" s="8">
-        <v>46122.384867395835</v>
+        <v>46122.5515340625</v>
       </c>
       <c r="C39" s="8">
-        <v>46154.70085026621</v>
+        <v>46154.86751693287</v>
       </c>
       <c r="D39" s="8">
-        <v>46154.70085260417</v>
+        <v>46154.86751927083</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>86</v>
@@ -4076,13 +4076,13 @@
         <v>150</v>
       </c>
       <c r="B40" s="5">
-        <v>46122.38487178241</v>
+        <v>46122.55153844907</v>
       </c>
       <c r="C40" s="5">
-        <v>46154.70090960649</v>
+        <v>46154.867576273144</v>
       </c>
       <c r="D40" s="5">
-        <v>46154.70091078704</v>
+        <v>46154.867577453704</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>151</v>
@@ -4131,13 +4131,13 @@
         <v>153</v>
       </c>
       <c r="B41" s="8">
-        <v>46122.40826678241</v>
+        <v>46122.574933449076</v>
       </c>
       <c r="C41" s="8">
-        <v>46181.500100335645</v>
+        <v>46181.666767002316</v>
       </c>
       <c r="D41" s="8">
-        <v>46221.03561572917</v>
+        <v>46221.20228239583</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>154</v>
@@ -4196,13 +4196,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46122.40925430556</v>
+        <v>46122.575920972224</v>
       </c>
       <c r="C42" s="5">
-        <v>46181.500040729166</v>
+        <v>46181.66670739584</v>
       </c>
       <c r="D42" s="5">
-        <v>46181.500041886575</v>
+        <v>46181.66670855324</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>89</v>
@@ -4251,13 +4251,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46122.409418090276</v>
+        <v>46122.57608475695</v>
       </c>
       <c r="C43" s="8">
-        <v>46181.50008614583</v>
+        <v>46181.666752812496</v>
       </c>
       <c r="D43" s="8">
-        <v>46181.500087685185</v>
+        <v>46181.666754351856</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4306,13 +4306,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46122.40834771991</v>
+        <v>46122.57501438657</v>
       </c>
       <c r="C44" s="5">
-        <v>46181.500291805554</v>
+        <v>46181.666958472226</v>
       </c>
       <c r="D44" s="5">
-        <v>46239.00492576389</v>
+        <v>46239.17159243056</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4371,13 +4371,13 @@
         <v>166</v>
       </c>
       <c r="B45" s="8">
-        <v>46122.41255444444</v>
+        <v>46122.57922111111</v>
       </c>
       <c r="C45" s="8">
-        <v>46181.50023484953</v>
+        <v>46181.666901516204</v>
       </c>
       <c r="D45" s="8">
-        <v>46181.50023640046</v>
+        <v>46181.66690306713</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>95</v>
@@ -4426,13 +4426,13 @@
         <v>168</v>
       </c>
       <c r="B46" s="5">
-        <v>46122.4128253588</v>
+        <v>46122.57949202546</v>
       </c>
       <c r="C46" s="5">
-        <v>46181.500276562496</v>
+        <v>46181.66694322917</v>
       </c>
       <c r="D46" s="5">
-        <v>46181.50027793982</v>
+        <v>46181.66694460648</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>169</v>
@@ -4481,13 +4481,13 @@
         <v>171</v>
       </c>
       <c r="B47" s="8">
-        <v>46125.362951550924</v>
+        <v>46125.529618217595</v>
       </c>
       <c r="C47" s="8">
-        <v>46181.50055453704</v>
+        <v>46181.66722120371</v>
       </c>
       <c r="D47" s="8">
-        <v>46227.91110196759</v>
+        <v>46228.07776863426</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>172</v>
@@ -4546,13 +4546,13 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46125.36311331019</v>
+        <v>46125.52977997685</v>
       </c>
       <c r="C48" s="5">
-        <v>46181.50049065972</v>
+        <v>46181.66715732639</v>
       </c>
       <c r="D48" s="5">
-        <v>46181.500492453706</v>
+        <v>46181.66715912037</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>92</v>
@@ -4601,13 +4601,13 @@
         <v>176</v>
       </c>
       <c r="B49" s="8">
-        <v>46125.36325149305</v>
+        <v>46125.52991815972</v>
       </c>
       <c r="C49" s="8">
-        <v>46181.5005374537</v>
+        <v>46181.66720412037</v>
       </c>
       <c r="D49" s="8">
-        <v>46181.50053896991</v>
+        <v>46181.66720563658</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>177</v>
@@ -4656,13 +4656,13 @@
         <v>179</v>
       </c>
       <c r="B50" s="5">
-        <v>46122.384541886575</v>
+        <v>46122.55120855324</v>
       </c>
       <c r="C50" s="5">
-        <v>46195.34078462963</v>
+        <v>46195.5074512963</v>
       </c>
       <c r="D50" s="5">
-        <v>46195.34089821759</v>
+        <v>46195.50756488426</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>180</v>
@@ -4709,13 +4709,13 @@
         <v>182</v>
       </c>
       <c r="B51" s="8">
-        <v>46122.38487678241</v>
+        <v>46122.55154344907</v>
       </c>
       <c r="C51" s="8">
-        <v>46133.62917814815</v>
+        <v>46133.79584481481</v>
       </c>
       <c r="D51" s="8">
-        <v>46143.00447921296</v>
+        <v>46143.171145879634</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>183</v>
@@ -4774,13 +4774,13 @@
         <v>187</v>
       </c>
       <c r="B52" s="5">
-        <v>46122.38488232639</v>
+        <v>46122.551548993055</v>
       </c>
       <c r="C52" s="5">
-        <v>46134.62573756944</v>
+        <v>46134.79240423611</v>
       </c>
       <c r="D52" s="5">
-        <v>46198.021150451386</v>
+        <v>46198.18781711806</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>188</v>
@@ -4839,13 +4839,13 @@
         <v>191</v>
       </c>
       <c r="B53" s="8">
-        <v>46122.38489054398</v>
+        <v>46122.55155721065</v>
       </c>
       <c r="C53" s="8">
-        <v>46134.62578480324</v>
+        <v>46134.79245146991</v>
       </c>
       <c r="D53" s="8">
-        <v>46199.01705138889</v>
+        <v>46199.18371805556</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>82</v>
@@ -4902,13 +4902,13 @@
         <v>193</v>
       </c>
       <c r="B54" s="5">
-        <v>46122.38489901621</v>
+        <v>46122.55156568287</v>
       </c>
       <c r="C54" s="5">
-        <v>46195.34094658565</v>
+        <v>46195.50761325231</v>
       </c>
       <c r="D54" s="5">
-        <v>46196.6024115162</v>
+        <v>46196.76907818287</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>194</v>
@@ -4965,13 +4965,13 @@
         <v>198</v>
       </c>
       <c r="B55" s="8">
-        <v>46125.43695545139</v>
+        <v>46125.603622118055</v>
       </c>
       <c r="C55" s="8">
-        <v>46196.60238085648</v>
+        <v>46196.76904752315</v>
       </c>
       <c r="D55" s="8">
-        <v>46196.602385474536</v>
+        <v>46196.7690521412</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>199</v>
@@ -5018,13 +5018,13 @@
         <v>201</v>
       </c>
       <c r="B56" s="5">
-        <v>46125.43700428241</v>
+        <v>46125.60367094907</v>
       </c>
       <c r="C56" s="5">
-        <v>46196.6023817824</v>
+        <v>46196.769048449074</v>
       </c>
       <c r="D56" s="5">
-        <v>46223.440795208335</v>
+        <v>46223.607461875</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>199</v>
@@ -5071,13 +5071,13 @@
         <v>202</v>
       </c>
       <c r="B57" s="8">
-        <v>46125.43705284722</v>
+        <v>46125.60371951389</v>
       </c>
       <c r="C57" s="8">
-        <v>46196.602382627316</v>
+        <v>46196.76904929398</v>
       </c>
       <c r="D57" s="8">
-        <v>46196.60238616898</v>
+        <v>46196.76905283565</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>199</v>
@@ -5124,13 +5124,13 @@
         <v>203</v>
       </c>
       <c r="B58" s="5">
-        <v>46125.43709796296</v>
+        <v>46125.60376462963</v>
       </c>
       <c r="C58" s="5">
-        <v>46196.60238340277</v>
+        <v>46196.769050069444</v>
       </c>
       <c r="D58" s="5">
-        <v>46196.60238648148</v>
+        <v>46196.76905314815</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>199</v>
@@ -5177,13 +5177,13 @@
         <v>204</v>
       </c>
       <c r="B59" s="8">
-        <v>46125.437150729165</v>
+        <v>46125.60381739584</v>
       </c>
       <c r="C59" s="8">
-        <v>46196.602384108795</v>
+        <v>46196.76905077546</v>
       </c>
       <c r="D59" s="8">
-        <v>46196.6023868287</v>
+        <v>46196.76905349537</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>199</v>
@@ -5230,13 +5230,13 @@
         <v>205</v>
       </c>
       <c r="B60" s="5">
-        <v>46122.38490304398</v>
+        <v>46122.551569710646</v>
       </c>
       <c r="C60" s="5">
-        <v>46181.501105787036</v>
+        <v>46181.6677724537</v>
       </c>
       <c r="D60" s="5">
-        <v>46181.501186574074</v>
+        <v>46181.66785324074</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>206</v>
@@ -5279,13 +5279,13 @@
         <v>208</v>
       </c>
       <c r="B61" s="8">
-        <v>46122.38490655093</v>
+        <v>46122.55157321759</v>
       </c>
       <c r="C61" s="8">
-        <v>46181.50071136574</v>
+        <v>46181.667378032405</v>
       </c>
       <c r="D61" s="8">
-        <v>46181.500728576386</v>
+        <v>46181.66739524306</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>209</v>
@@ -5344,13 +5344,13 @@
         <v>213</v>
       </c>
       <c r="B62" s="5">
-        <v>46122.41824972222</v>
+        <v>46122.58491638889</v>
       </c>
       <c r="C62" s="5">
-        <v>46181.50074653935</v>
+        <v>46181.667413206014</v>
       </c>
       <c r="D62" s="5">
-        <v>46181.50076234953</v>
+        <v>46181.667429016205</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>214</v>
@@ -5409,13 +5409,13 @@
         <v>216</v>
       </c>
       <c r="B63" s="8">
-        <v>46125.36435991898</v>
+        <v>46125.53102658565</v>
       </c>
       <c r="C63" s="8">
-        <v>46181.500763460645</v>
+        <v>46181.667430127316</v>
       </c>
       <c r="D63" s="8">
-        <v>46221.03561457176</v>
+        <v>46221.202281238424</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>217</v>
@@ -5474,13 +5474,13 @@
         <v>219</v>
       </c>
       <c r="B64" s="5">
-        <v>46122.38491179398</v>
+        <v>46122.55157846065</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.501089212965</v>
+        <v>46181.66775587963</v>
       </c>
       <c r="D64" s="5">
-        <v>46227.01578543981</v>
+        <v>46227.182452106485</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>215</v>
@@ -5539,13 +5539,13 @@
         <v>224</v>
       </c>
       <c r="B65" s="8">
-        <v>46122.38491716435</v>
+        <v>46122.551583831024</v>
       </c>
       <c r="C65" s="8">
-        <v>46181.50212802083</v>
+        <v>46181.6687946875</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.50224104167</v>
+        <v>46181.66890770833</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>225</v>
@@ -5588,13 +5588,13 @@
         <v>227</v>
       </c>
       <c r="B66" s="5">
-        <v>46122.384920219905</v>
+        <v>46122.55158688658</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.49942690972</v>
+        <v>46181.666093576394</v>
       </c>
       <c r="D66" s="5">
-        <v>46238.02180614583</v>
+        <v>46238.1884728125</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>228</v>
@@ -5653,13 +5653,13 @@
         <v>232</v>
       </c>
       <c r="B67" s="8">
-        <v>46122.384925185186</v>
+        <v>46122.55159185185</v>
       </c>
       <c r="C67" s="8">
-        <v>46181.49953199074</v>
+        <v>46181.6661986574</v>
       </c>
       <c r="D67" s="8">
-        <v>46256.03660438657</v>
+        <v>46256.20327105324</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>233</v>
@@ -5718,13 +5718,13 @@
         <v>235</v>
       </c>
       <c r="B68" s="5">
-        <v>46125.42914525463</v>
+        <v>46125.595811921296</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.501410324076</v>
+        <v>46181.66807699074</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.50141217593</v>
+        <v>46181.66807884259</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>236</v>
@@ -5773,13 +5773,13 @@
         <v>239</v>
       </c>
       <c r="B69" s="8">
-        <v>46125.42943380787</v>
+        <v>46125.59610047453</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.50141914352</v>
+        <v>46181.66808581019</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.50142061342</v>
+        <v>46181.66808728009</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>199</v>
@@ -5828,13 +5828,13 @@
         <v>240</v>
       </c>
       <c r="B70" s="5">
-        <v>46125.429543715276</v>
+        <v>46125.59621038195</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.501487326386</v>
+        <v>46181.66815399306</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.501488842594</v>
+        <v>46181.66815550926</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>199</v>
@@ -5883,13 +5883,13 @@
         <v>241</v>
       </c>
       <c r="B71" s="8">
-        <v>46125.42958805556</v>
+        <v>46125.59625472222</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.50150002315</v>
+        <v>46181.668166689815</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.501501527775</v>
+        <v>46181.66816819445</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>199</v>
@@ -5938,13 +5938,13 @@
         <v>242</v>
       </c>
       <c r="B72" s="5">
-        <v>46125.42963248843</v>
+        <v>46125.59629915509</v>
       </c>
       <c r="C72" s="5">
-        <v>46181.50151289352</v>
+        <v>46181.66817956018</v>
       </c>
       <c r="D72" s="5">
-        <v>46181.50151412037</v>
+        <v>46181.66818078703</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>199</v>
@@ -5993,13 +5993,13 @@
         <v>243</v>
       </c>
       <c r="B73" s="8">
-        <v>46122.384930844906</v>
+        <v>46122.55159751157</v>
       </c>
       <c r="C73" s="8">
-        <v>46181.50211394676</v>
+        <v>46181.66878061343</v>
       </c>
       <c r="D73" s="8">
-        <v>46252.035257337964</v>
+        <v>46252.20192400463</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>244</v>
@@ -6058,13 +6058,13 @@
         <v>245</v>
       </c>
       <c r="B74" s="5">
-        <v>46125.4298218287</v>
+        <v>46125.59648849537</v>
       </c>
       <c r="C74" s="5">
-        <v>46181.501985254625</v>
+        <v>46181.668651921296</v>
       </c>
       <c r="D74" s="5">
-        <v>46181.501986724536</v>
+        <v>46181.6686533912</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>199</v>
@@ -6113,13 +6113,13 @@
         <v>248</v>
       </c>
       <c r="B75" s="8">
-        <v>46125.429951875005</v>
+        <v>46125.59661854166</v>
       </c>
       <c r="C75" s="8">
-        <v>46181.50199983796</v>
+        <v>46181.66866650463</v>
       </c>
       <c r="D75" s="8">
-        <v>46181.50200115741</v>
+        <v>46181.66866782407</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>199</v>
@@ -6168,13 +6168,13 @@
         <v>250</v>
       </c>
       <c r="B76" s="5">
-        <v>46125.43000208333</v>
+        <v>46125.596668750004</v>
       </c>
       <c r="C76" s="5">
-        <v>46181.50200921296</v>
+        <v>46181.66867587963</v>
       </c>
       <c r="D76" s="5">
-        <v>46181.50201078704</v>
+        <v>46181.66867745371</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>199</v>
@@ -6223,13 +6223,13 @@
         <v>251</v>
       </c>
       <c r="B77" s="8">
-        <v>46125.430048842594</v>
+        <v>46125.59671550926</v>
       </c>
       <c r="C77" s="8">
-        <v>46181.50201895833</v>
+        <v>46181.668685625</v>
       </c>
       <c r="D77" s="8">
-        <v>46181.50202039352</v>
+        <v>46181.668687060184</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>199</v>
@@ -6278,13 +6278,13 @@
         <v>253</v>
       </c>
       <c r="B78" s="5">
-        <v>46125.430088796296</v>
+        <v>46125.59675546296</v>
       </c>
       <c r="C78" s="5">
-        <v>46181.5020371875</v>
+        <v>46181.66870385417</v>
       </c>
       <c r="D78" s="5">
-        <v>46181.502038356484</v>
+        <v>46181.66870502315</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>199</v>
@@ -6333,13 +6333,13 @@
         <v>254</v>
       </c>
       <c r="B79" s="8">
-        <v>46122.38493690972</v>
+        <v>46122.55160357639</v>
       </c>
       <c r="C79" s="8">
-        <v>46195.3964589699</v>
+        <v>46195.563125636574</v>
       </c>
       <c r="D79" s="8">
-        <v>46195.39662366898</v>
+        <v>46195.563290335645</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>206</v>
@@ -6386,13 +6386,13 @@
         <v>256</v>
       </c>
       <c r="B80" s="5">
-        <v>46122.38494012732</v>
+        <v>46122.55160679398</v>
       </c>
       <c r="C80" s="5">
-        <v>46195.39660269676</v>
+        <v>46195.563269363425</v>
       </c>
       <c r="D80" s="5">
-        <v>46240.43892752315</v>
+        <v>46240.605594189816</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>257</v>
@@ -6451,13 +6451,13 @@
         <v>259</v>
       </c>
       <c r="B81" s="8">
-        <v>46122.38494559028</v>
+        <v>46122.551612256946</v>
       </c>
       <c r="C81" s="8">
-        <v>46195.34084651621</v>
+        <v>46195.50751318287</v>
       </c>
       <c r="D81" s="8">
-        <v>46195.3408646412</v>
+        <v>46195.50753130787</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>260</v>
@@ -6516,13 +6516,13 @@
         <v>261</v>
       </c>
       <c r="B82" s="5">
-        <v>46122.38495090278</v>
+        <v>46122.55161756944</v>
       </c>
       <c r="C82" s="5">
-        <v>46195.340851851855</v>
+        <v>46195.50751851852</v>
       </c>
       <c r="D82" s="5">
-        <v>46195.34086592593</v>
+        <v>46195.50753259259</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>262</v>
@@ -6581,13 +6581,13 @@
         <v>263</v>
       </c>
       <c r="B83" s="8">
-        <v>46122.384956215275</v>
+        <v>46122.55162288195</v>
       </c>
       <c r="C83" s="8">
-        <v>46195.34085677083</v>
+        <v>46195.507523437496</v>
       </c>
       <c r="D83" s="8">
-        <v>46195.3408728125</v>
+        <v>46195.507539479164</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>264</v>
@@ -6646,13 +6646,13 @@
         <v>265</v>
       </c>
       <c r="B84" s="5">
-        <v>46122.427324965276</v>
+        <v>46122.59399163195</v>
       </c>
       <c r="C84" s="5">
-        <v>46193.76648644676</v>
+        <v>46193.93315311342</v>
       </c>
       <c r="D84" s="5">
-        <v>46241.02186137732</v>
+        <v>46241.18852804398</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>266</v>
@@ -6711,13 +6711,13 @@
         <v>268</v>
       </c>
       <c r="B85" s="8">
-        <v>46122.3849615162</v>
+        <v>46122.551628182875</v>
       </c>
       <c r="C85" s="8">
-        <v>46195.39639328704</v>
+        <v>46195.5630599537</v>
       </c>
       <c r="D85" s="8">
-        <v>46227.911395138886</v>
+        <v>46228.07806180556</v>
       </c>
       <c r="E85" s="9" t="s">
         <v>269</v>
@@ -6764,13 +6764,13 @@
         <v>271</v>
       </c>
       <c r="B86" s="5">
-        <v>46122.38496491898</v>
+        <v>46122.55163158565</v>
       </c>
       <c r="C86" s="5">
-        <v>46195.34102184028</v>
+        <v>46195.50768850694</v>
       </c>
       <c r="D86" s="5">
-        <v>46223.441128182865</v>
+        <v>46223.60779484954</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>272</v>
@@ -6829,13 +6829,13 @@
         <v>274</v>
       </c>
       <c r="B87" s="8">
-        <v>46125.43083025463</v>
+        <v>46125.5974969213</v>
       </c>
       <c r="C87" s="8">
-        <v>46196.60125040509</v>
+        <v>46196.76791707176</v>
       </c>
       <c r="D87" s="8">
-        <v>46223.440315810185</v>
+        <v>46223.60698247685</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>199</v>
@@ -6884,13 +6884,13 @@
         <v>276</v>
       </c>
       <c r="B88" s="5">
-        <v>46125.430879039355</v>
+        <v>46125.59754570602</v>
       </c>
       <c r="C88" s="5">
-        <v>46196.601287384256</v>
+        <v>46196.76795405093</v>
       </c>
       <c r="D88" s="5">
-        <v>46223.44030688658</v>
+        <v>46223.60697355324</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>199</v>
@@ -6939,13 +6939,13 @@
         <v>277</v>
       </c>
       <c r="B89" s="8">
-        <v>46125.430940439815</v>
+        <v>46125.59760710648</v>
       </c>
       <c r="C89" s="8">
-        <v>46196.601261550924</v>
+        <v>46196.767928217596</v>
       </c>
       <c r="D89" s="8">
-        <v>46223.44030333334</v>
+        <v>46223.60697</v>
       </c>
       <c r="E89" s="9" t="s">
         <v>199</v>
@@ -6994,13 +6994,13 @@
         <v>278</v>
       </c>
       <c r="B90" s="5">
-        <v>46125.43099224537</v>
+        <v>46125.59765891204</v>
       </c>
       <c r="C90" s="5">
-        <v>46196.601279849536</v>
+        <v>46196.76794651621</v>
       </c>
       <c r="D90" s="5">
-        <v>46223.44029975694</v>
+        <v>46223.60696642361</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>199</v>
@@ -7049,13 +7049,13 @@
         <v>279</v>
       </c>
       <c r="B91" s="8">
-        <v>46125.431036724534</v>
+        <v>46125.597703391206</v>
       </c>
       <c r="C91" s="8">
-        <v>46196.60127434028</v>
+        <v>46196.76794100694</v>
       </c>
       <c r="D91" s="8">
-        <v>46223.44029474537</v>
+        <v>46223.606961412035</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>199</v>
@@ -7104,13 +7104,13 @@
         <v>280</v>
       </c>
       <c r="B92" s="5">
-        <v>46122.38503993055</v>
+        <v>46122.55170659722</v>
       </c>
       <c r="C92" s="5">
-        <v>46196.60088846065</v>
+        <v>46196.76755512731</v>
       </c>
       <c r="D92" s="5">
-        <v>46237.368255925925</v>
+        <v>46237.53492259259</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>281</v>
@@ -7169,13 +7169,13 @@
         <v>282</v>
       </c>
       <c r="B93" s="8">
-        <v>46125.43316075232</v>
+        <v>46125.59982741898</v>
       </c>
       <c r="C93" s="8">
-        <v>46196.60133528935</v>
+        <v>46196.76800195602</v>
       </c>
       <c r="D93" s="8">
-        <v>46223.44041752315</v>
+        <v>46223.60708418982</v>
       </c>
       <c r="E93" s="9" t="s">
         <v>199</v>
@@ -7224,13 +7224,13 @@
         <v>285</v>
       </c>
       <c r="B94" s="5">
-        <v>46125.43322416667</v>
+        <v>46125.599890833335</v>
       </c>
       <c r="C94" s="5">
-        <v>46196.601356354164</v>
+        <v>46196.768023020835</v>
       </c>
       <c r="D94" s="5">
-        <v>46223.44041325232</v>
+        <v>46223.60707991898</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>199</v>
@@ -7279,13 +7279,13 @@
         <v>287</v>
       </c>
       <c r="B95" s="8">
-        <v>46125.43326467593</v>
+        <v>46125.59993134259</v>
       </c>
       <c r="C95" s="8">
-        <v>46196.601348275464</v>
+        <v>46196.76801494213</v>
       </c>
       <c r="D95" s="8">
-        <v>46223.440409166666</v>
+        <v>46223.60707583334</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>199</v>
@@ -7334,13 +7334,13 @@
         <v>288</v>
       </c>
       <c r="B96" s="5">
-        <v>46125.433302627316</v>
+        <v>46125.59996929398</v>
       </c>
       <c r="C96" s="5">
-        <v>46196.60138443287</v>
+        <v>46196.76805109954</v>
       </c>
       <c r="D96" s="5">
-        <v>46223.440405393514</v>
+        <v>46223.607072060186</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>199</v>
@@ -7389,13 +7389,13 @@
         <v>289</v>
       </c>
       <c r="B97" s="8">
-        <v>46125.43334484954</v>
+        <v>46125.6000115162</v>
       </c>
       <c r="C97" s="8">
-        <v>46196.60139039352</v>
+        <v>46196.76805706018</v>
       </c>
       <c r="D97" s="8">
-        <v>46223.44039952546</v>
+        <v>46223.607066192126</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>199</v>
@@ -7444,13 +7444,13 @@
         <v>290</v>
       </c>
       <c r="B98" s="5">
-        <v>46122.38497746528</v>
+        <v>46122.55164413195</v>
       </c>
       <c r="C98" s="5">
-        <v>46196.601731574076</v>
+        <v>46196.76839824074</v>
       </c>
       <c r="D98" s="5">
-        <v>46227.94037759259</v>
+        <v>46228.10704425926</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>291</v>
@@ -7509,13 +7509,13 @@
         <v>293</v>
       </c>
       <c r="B99" s="8">
-        <v>46125.43249607639</v>
+        <v>46125.599162743056</v>
       </c>
       <c r="C99" s="8">
-        <v>46196.601522997684</v>
+        <v>46196.76818966435</v>
       </c>
       <c r="D99" s="8">
-        <v>46223.44053969908</v>
+        <v>46223.60720636574</v>
       </c>
       <c r="E99" s="9" t="s">
         <v>199</v>
@@ -7564,13 +7564,13 @@
         <v>296</v>
       </c>
       <c r="B100" s="5">
-        <v>46125.4326358449</v>
+        <v>46125.599302511575</v>
       </c>
       <c r="C100" s="5">
-        <v>46196.601537546296</v>
+        <v>46196.76820421296</v>
       </c>
       <c r="D100" s="5">
-        <v>46223.44053581019</v>
+        <v>46223.60720247685</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>199</v>
@@ -7619,13 +7619,13 @@
         <v>297</v>
       </c>
       <c r="B101" s="8">
-        <v>46125.43267978009</v>
+        <v>46125.59934644676</v>
       </c>
       <c r="C101" s="8">
-        <v>46196.601709282404</v>
+        <v>46196.768375949076</v>
       </c>
       <c r="D101" s="8">
-        <v>46223.440531527776</v>
+        <v>46223.60719819444</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>199</v>
@@ -7674,13 +7674,13 @@
         <v>298</v>
       </c>
       <c r="B102" s="5">
-        <v>46125.43272190972</v>
+        <v>46125.59938857639</v>
       </c>
       <c r="C102" s="5">
-        <v>46196.60171030092</v>
+        <v>46196.76837696759</v>
       </c>
       <c r="D102" s="5">
-        <v>46223.44052751157</v>
+        <v>46223.60719417824</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>199</v>
@@ -7729,13 +7729,13 @@
         <v>299</v>
       </c>
       <c r="B103" s="8">
-        <v>46125.43276428241</v>
+        <v>46125.59943094908</v>
       </c>
       <c r="C103" s="8">
-        <v>46196.60171123843</v>
+        <v>46196.76837790509</v>
       </c>
       <c r="D103" s="8">
-        <v>46223.44052174769</v>
+        <v>46223.60718841435</v>
       </c>
       <c r="E103" s="9" t="s">
         <v>199</v>
@@ -7784,13 +7784,13 @@
         <v>300</v>
       </c>
       <c r="B104" s="5">
-        <v>46122.3849843287</v>
+        <v>46122.551650995374</v>
       </c>
       <c r="C104" s="5">
-        <v>46196.601881215276</v>
+        <v>46196.76854788195</v>
       </c>
       <c r="D104" s="5">
-        <v>46237.36827594908</v>
+        <v>46237.53494261574</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>301</v>
@@ -7849,13 +7849,13 @@
         <v>302</v>
       </c>
       <c r="B105" s="8">
-        <v>46125.43286347222</v>
+        <v>46125.59953013889</v>
       </c>
       <c r="C105" s="8">
-        <v>46196.60186116898</v>
+        <v>46196.76852783565</v>
       </c>
       <c r="D105" s="8">
-        <v>46223.44064487268</v>
+        <v>46223.60731153935</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>199</v>
@@ -7904,13 +7904,13 @@
         <v>304</v>
       </c>
       <c r="B106" s="5">
-        <v>46125.43294756944</v>
+        <v>46125.59961423611</v>
       </c>
       <c r="C106" s="5">
-        <v>46196.60179663195</v>
+        <v>46196.76846329861</v>
       </c>
       <c r="D106" s="5">
-        <v>46223.440641168985</v>
+        <v>46223.60730783565</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>199</v>
@@ -7959,13 +7959,13 @@
         <v>305</v>
       </c>
       <c r="B107" s="8">
-        <v>46125.43298765046</v>
+        <v>46125.599654317135</v>
       </c>
       <c r="C107" s="8">
-        <v>46196.601862129624</v>
+        <v>46196.768528796296</v>
       </c>
       <c r="D107" s="8">
-        <v>46223.44063728009</v>
+        <v>46223.60730394676</v>
       </c>
       <c r="E107" s="9" t="s">
         <v>199</v>
@@ -8014,13 +8014,13 @@
         <v>306</v>
       </c>
       <c r="B108" s="5">
-        <v>46125.43290399306</v>
+        <v>46125.59957065972</v>
       </c>
       <c r="C108" s="5">
-        <v>46196.601862881944</v>
+        <v>46196.768529548615</v>
       </c>
       <c r="D108" s="5">
-        <v>46223.44063300926</v>
+        <v>46223.607299675925</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>199</v>
@@ -8069,13 +8069,13 @@
         <v>307</v>
       </c>
       <c r="B109" s="8">
-        <v>46125.433030451386</v>
+        <v>46125.59969711806</v>
       </c>
       <c r="C109" s="8">
-        <v>46196.601863738426</v>
+        <v>46196.7685304051</v>
       </c>
       <c r="D109" s="8">
-        <v>46223.44062707176</v>
+        <v>46223.60729373843</v>
       </c>
       <c r="E109" s="9" t="s">
         <v>199</v>
@@ -8124,13 +8124,13 @@
         <v>308</v>
       </c>
       <c r="B110" s="5">
-        <v>46122.38497059028</v>
+        <v>46122.55163725694</v>
       </c>
       <c r="C110" s="5">
-        <v>46196.6020008912</v>
+        <v>46196.76866755787</v>
       </c>
       <c r="D110" s="5">
-        <v>46223.44111295139</v>
+        <v>46223.607779618054</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>309</v>
@@ -8189,13 +8189,13 @@
         <v>310</v>
       </c>
       <c r="B111" s="8">
-        <v>46125.431135439816</v>
+        <v>46125.59780210648</v>
       </c>
       <c r="C111" s="8">
-        <v>46196.60198236111</v>
+        <v>46196.76864902778</v>
       </c>
       <c r="D111" s="8">
-        <v>46223.44074164351</v>
+        <v>46223.607408310185</v>
       </c>
       <c r="E111" s="9" t="s">
         <v>199</v>
@@ -8244,13 +8244,13 @@
         <v>313</v>
       </c>
       <c r="B112" s="5">
-        <v>46125.43117026621</v>
+        <v>46125.597836932866</v>
       </c>
       <c r="C112" s="5">
-        <v>46196.601983333334</v>
+        <v>46196.76865</v>
       </c>
       <c r="D112" s="5">
-        <v>46223.4407377662</v>
+        <v>46223.60740443287</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>199</v>
@@ -8299,13 +8299,13 @@
         <v>314</v>
       </c>
       <c r="B113" s="8">
-        <v>46125.43125422453</v>
+        <v>46125.5979208912</v>
       </c>
       <c r="C113" s="8">
-        <v>46196.6019841088</v>
+        <v>46196.76865077546</v>
       </c>
       <c r="D113" s="8">
-        <v>46223.44073386574</v>
+        <v>46223.607400532404</v>
       </c>
       <c r="E113" s="9" t="s">
         <v>199</v>
@@ -8354,13 +8354,13 @@
         <v>315</v>
       </c>
       <c r="B114" s="5">
-        <v>46125.431214212964</v>
+        <v>46125.59788087963</v>
       </c>
       <c r="C114" s="5">
-        <v>46196.60198486111</v>
+        <v>46196.768651527775</v>
       </c>
       <c r="D114" s="5">
-        <v>46223.44073002315</v>
+        <v>46223.60739668981</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>199</v>
@@ -8409,13 +8409,13 @@
         <v>316</v>
       </c>
       <c r="B115" s="8">
-        <v>46125.43129835648</v>
+        <v>46125.597965023146</v>
       </c>
       <c r="C115" s="8">
-        <v>46196.60198564814</v>
+        <v>46196.768652314815</v>
       </c>
       <c r="D115" s="8">
-        <v>46223.440723796295</v>
+        <v>46223.60739046296</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>199</v>
@@ -8464,13 +8464,13 @@
         <v>317</v>
       </c>
       <c r="B116" s="5">
-        <v>46122.38505377315</v>
+        <v>46122.55172043982</v>
       </c>
       <c r="C116" s="5">
-        <v>46196.6021055787</v>
+        <v>46196.76877224537</v>
       </c>
       <c r="D116" s="5">
-        <v>46237.368298009256</v>
+        <v>46237.53496467593</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>318</v>
@@ -8529,13 +8529,13 @@
         <v>319</v>
       </c>
       <c r="B117" s="8">
-        <v>46125.43371586806</v>
+        <v>46125.60038253472</v>
       </c>
       <c r="C117" s="8">
-        <v>46196.602085914354</v>
+        <v>46196.76875258102</v>
       </c>
       <c r="D117" s="8">
-        <v>46223.4409177662</v>
+        <v>46223.60758443287</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>199</v>
@@ -8582,13 +8582,13 @@
         <v>321</v>
       </c>
       <c r="B118" s="5">
-        <v>46125.43376346065</v>
+        <v>46125.60043012731</v>
       </c>
       <c r="C118" s="5">
-        <v>46223.44078604167</v>
+        <v>46223.60745270833</v>
       </c>
       <c r="D118" s="5">
-        <v>46223.440913391205</v>
+        <v>46223.60758005787</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>199</v>
@@ -8635,13 +8635,13 @@
         <v>322</v>
       </c>
       <c r="B119" s="8">
-        <v>46125.43380623843</v>
+        <v>46125.60047290509</v>
       </c>
       <c r="C119" s="8">
-        <v>46196.60208751158</v>
+        <v>46196.768754178236</v>
       </c>
       <c r="D119" s="8">
-        <v>46223.44090908565</v>
+        <v>46223.607575752314</v>
       </c>
       <c r="E119" s="9" t="s">
         <v>199</v>
@@ -8688,13 +8688,13 @@
         <v>323</v>
       </c>
       <c r="B120" s="5">
-        <v>46125.4338474074</v>
+        <v>46125.600514074074</v>
       </c>
       <c r="C120" s="5">
-        <v>46196.602088263884</v>
+        <v>46196.768754930556</v>
       </c>
       <c r="D120" s="5">
-        <v>46223.440904930554</v>
+        <v>46223.607571597226</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>199</v>
@@ -8741,13 +8741,13 @@
         <v>324</v>
       </c>
       <c r="B121" s="8">
-        <v>46125.43389193287</v>
+        <v>46125.60055859954</v>
       </c>
       <c r="C121" s="8">
-        <v>46196.602089224536</v>
+        <v>46196.7687558912</v>
       </c>
       <c r="D121" s="8">
-        <v>46223.44089886574</v>
+        <v>46223.60756553241</v>
       </c>
       <c r="E121" s="9" t="s">
         <v>199</v>
@@ -8794,13 +8794,13 @@
         <v>325</v>
       </c>
       <c r="B122" s="5">
-        <v>46122.385063194444</v>
+        <v>46122.55172986111</v>
       </c>
       <c r="C122" s="5">
-        <v>46196.60250790509</v>
+        <v>46196.76917457176</v>
       </c>
       <c r="D122" s="5">
-        <v>46223.44110321759</v>
+        <v>46223.60776988426</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>326</v>
@@ -8859,13 +8859,13 @@
         <v>328</v>
       </c>
       <c r="B123" s="8">
-        <v>46125.4339775</v>
+        <v>46125.60064416667</v>
       </c>
       <c r="C123" s="8">
-        <v>46196.6024843287</v>
+        <v>46196.76915099537</v>
       </c>
       <c r="D123" s="8">
-        <v>46223.44101393518</v>
+        <v>46223.607680601854</v>
       </c>
       <c r="E123" s="9" t="s">
         <v>199</v>
@@ -8912,13 +8912,13 @@
         <v>330</v>
       </c>
       <c r="B124" s="5">
-        <v>46125.43402074074</v>
+        <v>46125.60068740741</v>
       </c>
       <c r="C124" s="5">
-        <v>46196.60248570602</v>
+        <v>46196.76915237268</v>
       </c>
       <c r="D124" s="5">
-        <v>46223.44101039352</v>
+        <v>46223.60767706019</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>199</v>
@@ -8965,13 +8965,13 @@
         <v>331</v>
       </c>
       <c r="B125" s="8">
-        <v>46125.43407178241</v>
+        <v>46125.60073844907</v>
       </c>
       <c r="C125" s="8">
-        <v>46196.60248674768</v>
+        <v>46196.76915341435</v>
       </c>
       <c r="D125" s="8">
-        <v>46223.44100614583</v>
+        <v>46223.607672812504</v>
       </c>
       <c r="E125" s="9" t="s">
         <v>199</v>
@@ -9018,13 +9018,13 @@
         <v>332</v>
       </c>
       <c r="B126" s="5">
-        <v>46125.434109560185</v>
+        <v>46125.60077622686</v>
       </c>
       <c r="C126" s="5">
-        <v>46196.60248771991</v>
+        <v>46196.76915438657</v>
       </c>
       <c r="D126" s="5">
-        <v>46223.44100177083</v>
+        <v>46223.6076684375</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>199</v>
@@ -9071,13 +9071,13 @@
         <v>333</v>
       </c>
       <c r="B127" s="8">
-        <v>46125.43416247686</v>
+        <v>46125.600829143514</v>
       </c>
       <c r="C127" s="8">
-        <v>46196.60248869213</v>
+        <v>46196.769155358794</v>
       </c>
       <c r="D127" s="8">
-        <v>46223.440996226855</v>
+        <v>46223.60766289352</v>
       </c>
       <c r="E127" s="9" t="s">
         <v>199</v>
@@ -9124,13 +9124,13 @@
         <v>334</v>
       </c>
       <c r="B128" s="5">
-        <v>46122.38506837963</v>
+        <v>46122.5517350463</v>
       </c>
       <c r="C128" s="5">
-        <v>46195.39650850694</v>
+        <v>46195.56317517361</v>
       </c>
       <c r="D128" s="5">
-        <v>46196.60293743055</v>
+        <v>46196.76960409722</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>335</v>
@@ -9177,13 +9177,13 @@
         <v>337</v>
       </c>
       <c r="B129" s="8">
-        <v>46122.38507239583</v>
+        <v>46122.5517390625</v>
       </c>
       <c r="C129" s="8">
-        <v>46196.60269986111</v>
+        <v>46196.76936652778</v>
       </c>
       <c r="D129" s="8">
-        <v>46240.43895601852</v>
+        <v>46240.60562268519</v>
       </c>
       <c r="E129" s="9" t="s">
         <v>338</v>
@@ -9242,13 +9242,13 @@
         <v>342</v>
       </c>
       <c r="B130" s="5">
-        <v>46125.43427064815</v>
+        <v>46125.60093731481</v>
       </c>
       <c r="C130" s="5">
-        <v>46196.602678483796</v>
+        <v>46196.76934515046</v>
       </c>
       <c r="D130" s="5">
-        <v>46196.60268401621</v>
+        <v>46196.769350682865</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>199</v>
@@ -9295,13 +9295,13 @@
         <v>344</v>
       </c>
       <c r="B131" s="8">
-        <v>46125.4347141551</v>
+        <v>46125.601380821754</v>
       </c>
       <c r="C131" s="8">
-        <v>46196.602679641204</v>
+        <v>46196.769346307876</v>
       </c>
       <c r="D131" s="8">
-        <v>46196.60268447916</v>
+        <v>46196.769351145835</v>
       </c>
       <c r="E131" s="9" t="s">
         <v>199</v>
@@ -9348,13 +9348,13 @@
         <v>345</v>
       </c>
       <c r="B132" s="5">
-        <v>46125.43475814815</v>
+        <v>46125.60142481481</v>
       </c>
       <c r="C132" s="5">
-        <v>46196.60268056713</v>
+        <v>46196.7693472338</v>
       </c>
       <c r="D132" s="5">
-        <v>46196.60268488426</v>
+        <v>46196.76935155093</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>199</v>
@@ -9401,13 +9401,13 @@
         <v>346</v>
       </c>
       <c r="B133" s="8">
-        <v>46125.434794189816</v>
+        <v>46125.60146085648</v>
       </c>
       <c r="C133" s="8">
-        <v>46196.60268145833</v>
+        <v>46196.769348125</v>
       </c>
       <c r="D133" s="8">
-        <v>46196.602685254635</v>
+        <v>46196.76935192129</v>
       </c>
       <c r="E133" s="9" t="s">
         <v>199</v>
@@ -9454,13 +9454,13 @@
         <v>347</v>
       </c>
       <c r="B134" s="5">
-        <v>46125.434835416665</v>
+        <v>46125.60150208333</v>
       </c>
       <c r="C134" s="5">
-        <v>46196.60268231481</v>
+        <v>46196.769348981485</v>
       </c>
       <c r="D134" s="5">
-        <v>46196.602685624996</v>
+        <v>46196.76935229167</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>199</v>
@@ -9507,13 +9507,13 @@
         <v>348</v>
       </c>
       <c r="B135" s="8">
-        <v>46122.38507716435</v>
+        <v>46122.55174383102</v>
       </c>
       <c r="C135" s="8">
-        <v>46196.60293025463</v>
+        <v>46196.769596921295</v>
       </c>
       <c r="D135" s="8">
-        <v>46227.94093403935</v>
+        <v>46228.10760070602</v>
       </c>
       <c r="E135" s="9" t="s">
         <v>349</v>
@@ -9570,13 +9570,13 @@
         <v>350</v>
       </c>
       <c r="B136" s="5">
-        <v>46125.4344203125</v>
+        <v>46125.601086979164</v>
       </c>
       <c r="C136" s="5">
-        <v>46196.602804884256</v>
+        <v>46196.76947155093</v>
       </c>
       <c r="D136" s="5">
-        <v>46223.44170403935</v>
+        <v>46223.60837070602</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>199</v>
@@ -9623,13 +9623,13 @@
         <v>352</v>
       </c>
       <c r="B137" s="8">
-        <v>46125.4344865162</v>
+        <v>46125.60115318287</v>
       </c>
       <c r="C137" s="8">
-        <v>46196.60283766204</v>
+        <v>46196.7695043287</v>
       </c>
       <c r="D137" s="8">
-        <v>46223.44169987268</v>
+        <v>46223.60836653935</v>
       </c>
       <c r="E137" s="9" t="s">
         <v>199</v>
@@ -9676,13 +9676,13 @@
         <v>353</v>
       </c>
       <c r="B138" s="5">
-        <v>46125.43453724537</v>
+        <v>46125.60120391204</v>
       </c>
       <c r="C138" s="5">
-        <v>46196.60283883102</v>
+        <v>46196.76950549769</v>
       </c>
       <c r="D138" s="5">
-        <v>46223.4416959375</v>
+        <v>46223.608362604165</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>199</v>
@@ -9729,13 +9729,13 @@
         <v>354</v>
       </c>
       <c r="B139" s="8">
-        <v>46125.434591296296</v>
+        <v>46125.60125796296</v>
       </c>
       <c r="C139" s="8">
-        <v>46196.60283971065</v>
+        <v>46196.76950637731</v>
       </c>
       <c r="D139" s="8">
-        <v>46223.44169238426</v>
+        <v>46223.60835905092</v>
       </c>
       <c r="E139" s="9" t="s">
         <v>199</v>
@@ -9782,13 +9782,13 @@
         <v>355</v>
       </c>
       <c r="B140" s="5">
-        <v>46125.43463761574</v>
+        <v>46125.601304282405</v>
       </c>
       <c r="C140" s="5">
-        <v>46196.60284063657</v>
+        <v>46196.76950730324</v>
       </c>
       <c r="D140" s="5">
-        <v>46223.44168600695</v>
+        <v>46223.60835267361</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>199</v>
@@ -9835,13 +9835,13 @@
         <v>356</v>
       </c>
       <c r="B141" s="8">
-        <v>46122.38508202546</v>
+        <v>46122.55174869213</v>
       </c>
       <c r="C141" s="8">
-        <v>46191.539318634255</v>
+        <v>46191.70598530093</v>
       </c>
       <c r="D141" s="8">
-        <v>46240.438971701384</v>
+        <v>46240.605638368055</v>
       </c>
       <c r="E141" s="9" t="s">
         <v>357</v>
@@ -9898,13 +9898,13 @@
         <v>358</v>
       </c>
       <c r="B142" s="5">
-        <v>46125.434919837964</v>
+        <v>46125.60158650463</v>
       </c>
       <c r="C142" s="5">
-        <v>46196.60301796296</v>
+        <v>46196.76968462963</v>
       </c>
       <c r="D142" s="5">
-        <v>46196.60302322917</v>
+        <v>46196.76968989584</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>199</v>
@@ -9951,13 +9951,13 @@
         <v>360</v>
       </c>
       <c r="B143" s="8">
-        <v>46125.43496466435</v>
+        <v>46125.60163133102</v>
       </c>
       <c r="C143" s="8">
-        <v>46196.60301918982</v>
+        <v>46196.76968585648</v>
       </c>
       <c r="D143" s="8">
-        <v>46196.60302364583</v>
+        <v>46196.7696903125</v>
       </c>
       <c r="E143" s="9" t="s">
         <v>199</v>
@@ -10004,13 +10004,13 @@
         <v>361</v>
       </c>
       <c r="B144" s="5">
-        <v>46125.43500349537</v>
+        <v>46125.60167016204</v>
       </c>
       <c r="C144" s="5">
-        <v>46196.603019988426</v>
+        <v>46196.7696866551</v>
       </c>
       <c r="D144" s="5">
-        <v>46196.60302403935</v>
+        <v>46196.769690706016</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>199</v>
@@ -10057,13 +10057,13 @@
         <v>363</v>
       </c>
       <c r="B145" s="8">
-        <v>46125.43503768518</v>
+        <v>46125.60170435185</v>
       </c>
       <c r="C145" s="8">
-        <v>46196.60302072916</v>
+        <v>46196.769687395834</v>
       </c>
       <c r="D145" s="8">
-        <v>46196.60302447916</v>
+        <v>46196.76969114583</v>
       </c>
       <c r="E145" s="9" t="s">
         <v>199</v>
@@ -10110,13 +10110,13 @@
         <v>364</v>
       </c>
       <c r="B146" s="5">
-        <v>46125.4350728125</v>
+        <v>46125.60173947917</v>
       </c>
       <c r="C146" s="5">
-        <v>46196.60302144676</v>
+        <v>46196.769688113425</v>
       </c>
       <c r="D146" s="5">
-        <v>46196.60302497685</v>
+        <v>46196.76969164352</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>199</v>
@@ -10163,13 +10163,13 @@
         <v>365</v>
       </c>
       <c r="B147" s="8">
-        <v>46122.38508680556</v>
+        <v>46122.551753472224</v>
       </c>
       <c r="C147" s="8">
-        <v>46191.53937342593</v>
+        <v>46191.70604009259</v>
       </c>
       <c r="D147" s="8">
-        <v>46240.4389865625</v>
+        <v>46240.60565322917</v>
       </c>
       <c r="E147" s="9" t="s">
         <v>366</v>
@@ -10226,13 +10226,13 @@
         <v>368</v>
       </c>
       <c r="B148" s="5">
-        <v>46125.43514888889</v>
+        <v>46125.60181555555</v>
       </c>
       <c r="C148" s="5">
-        <v>46196.60312598379</v>
+        <v>46196.76979265046</v>
       </c>
       <c r="D148" s="5">
-        <v>46196.603129027775</v>
+        <v>46196.76979569445</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>199</v>
@@ -10279,13 +10279,13 @@
         <v>369</v>
       </c>
       <c r="B149" s="8">
-        <v>46125.43519024306</v>
+        <v>46125.60185690972</v>
       </c>
       <c r="C149" s="8">
-        <v>46196.603126898146</v>
+        <v>46196.76979356482</v>
       </c>
       <c r="D149" s="8">
-        <v>46196.60312947917</v>
+        <v>46196.76979614583</v>
       </c>
       <c r="E149" s="9" t="s">
         <v>199</v>
@@ -10332,13 +10332,13 @@
         <v>370</v>
       </c>
       <c r="B150" s="5">
-        <v>46125.43523282408</v>
+        <v>46125.601899490735</v>
       </c>
       <c r="C150" s="5">
-        <v>46196.60312755787</v>
+        <v>46196.769794224536</v>
       </c>
       <c r="D150" s="5">
-        <v>46196.603129814815</v>
+        <v>46196.76979648148</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>199</v>
@@ -10385,13 +10385,13 @@
         <v>371</v>
       </c>
       <c r="B151" s="8">
-        <v>46125.43527268519</v>
+        <v>46125.60193935185</v>
       </c>
       <c r="C151" s="8">
-        <v>46196.603098101856</v>
+        <v>46196.76976476852</v>
       </c>
       <c r="D151" s="8">
-        <v>46196.60310020833</v>
+        <v>46196.769766875004</v>
       </c>
       <c r="E151" s="9" t="s">
         <v>199</v>
@@ -10438,13 +10438,13 @@
         <v>372</v>
       </c>
       <c r="B152" s="5">
-        <v>46125.43531043982</v>
+        <v>46125.60197710648</v>
       </c>
       <c r="C152" s="5">
-        <v>46196.603105393515</v>
+        <v>46196.76977206019</v>
       </c>
       <c r="D152" s="5">
-        <v>46196.60310703704</v>
+        <v>46196.76977370371</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>199</v>
@@ -10491,13 +10491,13 @@
         <v>373</v>
       </c>
       <c r="B153" s="8">
-        <v>46122.38509195602</v>
+        <v>46122.551758622685</v>
       </c>
       <c r="C153" s="8">
-        <v>46240.487175752314</v>
+        <v>46240.65384241898</v>
       </c>
       <c r="D153" s="8">
-        <v>46240.48718778935</v>
+        <v>46240.65385445602</v>
       </c>
       <c r="E153" s="9" t="s">
         <v>374</v>
@@ -10544,13 +10544,13 @@
         <v>376</v>
       </c>
       <c r="B154" s="5">
-        <v>46122.38509467593</v>
+        <v>46122.55176134259</v>
       </c>
       <c r="C154" s="5">
-        <v>46240.487151678244</v>
+        <v>46240.65381834491</v>
       </c>
       <c r="D154" s="5">
-        <v>46240.487169479165</v>
+        <v>46240.65383614584</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>377</v>
@@ -10609,13 +10609,13 @@
         <v>380</v>
       </c>
       <c r="B155" s="8">
-        <v>46122.38509943287</v>
+        <v>46122.55176609954</v>
       </c>
       <c r="C155" s="8">
-        <v>46240.487160578705</v>
+        <v>46240.65382724537</v>
       </c>
       <c r="D155" s="8">
-        <v>46240.4871771412</v>
+        <v>46240.65384380787</v>
       </c>
       <c r="E155" s="9" t="s">
         <v>381</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-26 13:59 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -5999,7 +5999,7 @@
         <v>46181.66878061343</v>
       </c>
       <c r="D73" s="8">
-        <v>46252.20192400463</v>
+        <v>46260.20541972222</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>244</v>
@@ -6043,8 +6043,8 @@
       <c r="R73" s="8">
         <v>46259</v>
       </c>
-      <c r="S73" s="12" t="s">
-        <v>74</v>
+      <c r="S73" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T73" s="9">
         <v>1</v>
@@ -6457,7 +6457,7 @@
         <v>46195.50751318287</v>
       </c>
       <c r="D81" s="8">
-        <v>46195.50753130787</v>
+        <v>46260.18797238426</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>260</v>
@@ -6501,8 +6501,8 @@
       <c r="R81" s="8">
         <v>46267</v>
       </c>
-      <c r="S81" s="11" t="s">
-        <v>107</v>
+      <c r="S81" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T81" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-01 17:19 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -3153,7 +3153,7 @@
         <v>46174.626168703704</v>
       </c>
       <c r="D25" s="8">
-        <v>46258.19630414352</v>
+        <v>46266.17935409722</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>100</v>
@@ -3197,8 +3197,8 @@
       <c r="R25" s="8">
         <v>46265</v>
       </c>
-      <c r="S25" s="12" t="s">
-        <v>74</v>
+      <c r="S25" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T25" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-03 17:03 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -6457,7 +6457,7 @@
         <v>46195.50751318287</v>
       </c>
       <c r="D81" s="8">
-        <v>46260.18797238426</v>
+        <v>46268.17383480324</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>260</v>
@@ -6501,8 +6501,8 @@
       <c r="R81" s="8">
         <v>46267</v>
       </c>
-      <c r="S81" s="12" t="s">
-        <v>74</v>
+      <c r="S81" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T81" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-07 18:15 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -6770,7 +6770,7 @@
         <v>46195.50768850694</v>
       </c>
       <c r="D86" s="5">
-        <v>46223.60779484954</v>
+        <v>46272.13737606481</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>272</v>
@@ -6814,8 +6814,8 @@
       <c r="R86" s="5">
         <v>46279</v>
       </c>
-      <c r="S86" s="11" t="s">
-        <v>107</v>
+      <c r="S86" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T86" s="6">
         <v>1</v>

</xml_diff>